<commit_message>
thay đổi bước xích từ 25.4 -> 15.875
</commit_message>
<xml_diff>
--- a/tínhtoans.xlsx
+++ b/tínhtoans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Đồ án tkm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4FCC2A2-9E68-4B7E-87D1-7117AC3CC9D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9912E964-EA1A-4D28-8859-2C3A7BF400C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{75337E03-C337-4BFE-A279-78895F300CE2}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="287">
   <si>
     <t>Bánh răng trụ răng thẳng</t>
   </si>
@@ -722,12 +722,6 @@
     <t>Bánh răng lớn</t>
   </si>
   <si>
-    <t>Tra bảng 5.5 tr82 với n01 = 200 và P_t &lt;= [P], có</t>
-  </si>
-  <si>
-    <t>với i = 3.04 &lt; [i] = 50 khi p = 25.4 mm</t>
-  </si>
-  <si>
     <t>HB192...240</t>
   </si>
   <si>
@@ -897,6 +891,15 @@
   </si>
   <si>
     <t xml:space="preserve">Khoảng cách trục </t>
+  </si>
+  <si>
+    <t>với i = 3.04 &lt; [i] = 30 khi p = 15.875 mm</t>
+  </si>
+  <si>
+    <t>bảng 5.2 tr78</t>
+  </si>
+  <si>
+    <t>Tra bảng 5.5 tr82 với n01 = 1200 và P_t &lt;= [P], có</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1063,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1110,14 +1113,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3804,7 +3803,7 @@
       <c r="B90" s="6">
         <v>1.25</v>
       </c>
-      <c r="F90" s="25" t="s">
+      <c r="F90" s="26" t="s">
         <v>118</v>
       </c>
     </row>
@@ -3812,7 +3811,7 @@
       <c r="A91" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="F91" s="25"/>
+      <c r="F91" s="26"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
@@ -3824,13 +3823,13 @@
       <c r="C92" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="F92" s="25"/>
+      <c r="F92" s="26"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="F93" s="25"/>
+      <c r="F93" s="26"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
@@ -3842,13 +3841,13 @@
       <c r="C94" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="F94" s="25"/>
+      <c r="F94" s="26"/>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="F95" s="25"/>
+      <c r="F95" s="26"/>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
@@ -3860,13 +3859,13 @@
       <c r="C96" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="F96" s="25"/>
+      <c r="F96" s="26"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="F97" s="25"/>
+      <c r="F97" s="26"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
@@ -3878,13 +3877,13 @@
       <c r="C98" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="F98" s="25"/>
+      <c r="F98" s="26"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="F99" s="25"/>
+      <c r="F99" s="26"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
@@ -3896,7 +3895,7 @@
       <c r="C100" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="F100" s="25"/>
+      <c r="F100" s="26"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="12" t="s">
@@ -3928,7 +3927,7 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>227</v>
+        <v>286</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
@@ -3941,7 +3940,7 @@
         <v>120</v>
       </c>
       <c r="B108" s="6">
-        <v>25.4</v>
+        <v>15.875</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
@@ -3954,7 +3953,7 @@
         <v>122</v>
       </c>
       <c r="B110" s="6">
-        <v>7.95</v>
+        <v>5.08</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -3967,7 +3966,7 @@
         <v>124</v>
       </c>
       <c r="B112" s="6">
-        <v>22.61</v>
+        <v>13.28</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
@@ -3980,7 +3979,7 @@
         <v>126</v>
       </c>
       <c r="B114" s="6">
-        <v>11</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
@@ -4009,7 +4008,7 @@
       </c>
       <c r="B120" s="6">
         <f>40*B108</f>
-        <v>1016</v>
+        <v>635</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
@@ -4045,7 +4044,7 @@
       </c>
       <c r="B125" s="6">
         <f>B123*B108</f>
-        <v>3302</v>
+        <v>2063.75</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
@@ -4059,7 +4058,7 @@
       </c>
       <c r="B127" s="6">
         <f>ROUND(0.25*B108*(B123-0.5*(C75+C74)+SQRT((B123-0.5*(C74+C75))^2-2*((C75-C74)/3.14)^2)),2)</f>
-        <v>1021.38</v>
+        <v>638.36</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.25">
@@ -4073,11 +4072,11 @@
       </c>
       <c r="B129" s="6">
         <f>0.002*B127</f>
-        <v>2.0427599999999999</v>
+        <v>1.2767200000000001</v>
       </c>
       <c r="C129" s="6">
         <f>0.004*B127</f>
-        <v>4.0855199999999998</v>
+        <v>2.5534400000000002</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
@@ -4085,7 +4084,7 @@
         <v>141</v>
       </c>
       <c r="B130" s="6">
-        <v>2.38</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
@@ -4099,7 +4098,7 @@
       </c>
       <c r="B133" s="6">
         <f>B127-B130</f>
-        <v>1019</v>
+        <v>636</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
@@ -4123,7 +4122,7 @@
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>228</v>
+        <v>284</v>
       </c>
       <c r="B138" s="6" t="s">
         <v>146</v>
@@ -4150,7 +4149,7 @@
       </c>
       <c r="B143" s="6">
         <f>ROUND(C74*B108*D66/60000,2)</f>
-        <v>2.5099999999999998</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
@@ -4187,7 +4186,7 @@
       </c>
       <c r="B146" s="6">
         <f>ROUND(1000*D65/B143,2)</f>
-        <v>1661.35</v>
+        <v>2656.05</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.25">
@@ -4196,7 +4195,7 @@
       </c>
       <c r="B147" s="6">
         <f>ROUND(F145*B143^2,2)</f>
-        <v>16.38</v>
+        <v>6.41</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.25">
@@ -4205,7 +4204,7 @@
       </c>
       <c r="B148" s="6">
         <f>ROUND(9.81*D148*F145*B133/1000,2)</f>
-        <v>51.98</v>
+        <v>32.44</v>
       </c>
       <c r="C148" s="6" t="s">
         <v>161</v>
@@ -4219,7 +4218,7 @@
         <v>155</v>
       </c>
       <c r="B149" s="6">
-        <v>8.1999999999999993</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.25">
@@ -4228,7 +4227,7 @@
       </c>
       <c r="B151" s="6">
         <f>ROUND(B144*10^3/(B145*B146+B148+B147),2)</f>
-        <v>27.5</v>
+        <v>17.579999999999998</v>
       </c>
       <c r="C151" s="6" t="s">
         <v>162</v>
@@ -4250,7 +4249,7 @@
       </c>
       <c r="B155" s="6">
         <f>ROUND(B108/SIN(3.14/C74),2)</f>
-        <v>186.63</v>
+        <v>116.64</v>
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.25">
@@ -4259,7 +4258,7 @@
       </c>
       <c r="B156" s="6">
         <f>ROUND(B108/SIN(3.14/C75),2)</f>
-        <v>590.69000000000005</v>
+        <v>369.18</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.25">
@@ -4273,7 +4272,7 @@
       </c>
       <c r="B158" s="6">
         <f>ROUND(B108*(0.5+_xlfn.COT(3.14/C74)),2)</f>
-        <v>197.59</v>
+        <v>123.5</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.25">
@@ -4282,7 +4281,7 @@
       </c>
       <c r="B159" s="6">
         <f>ROUND(B108*(0.5+_xlfn.COT(3.14/C75)),2)</f>
-        <v>602.85</v>
+        <v>376.78</v>
       </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.25">
@@ -4293,7 +4292,10 @@
         <v>172</v>
       </c>
       <c r="C160" s="6">
-        <v>15.88</v>
+        <v>10.16</v>
+      </c>
+      <c r="D160" s="6" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
@@ -4302,7 +4304,7 @@
       </c>
       <c r="B161" s="6">
         <f>ROUND(0.5025*C160+0.05,2)</f>
-        <v>8.0299999999999994</v>
+        <v>5.16</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
@@ -4316,7 +4318,7 @@
       </c>
       <c r="B163" s="6">
         <f>B155-2*B161</f>
-        <v>170.57</v>
+        <v>106.32</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
@@ -4325,7 +4327,7 @@
       </c>
       <c r="B164" s="6">
         <f>B156-2*B161</f>
-        <v>574.63000000000011</v>
+        <v>358.86</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
@@ -4339,7 +4341,7 @@
       </c>
       <c r="B166" s="6">
         <f>ROUND(13*10^-7*D66*B108^3*1,2)</f>
-        <v>5.49</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
@@ -4386,7 +4388,7 @@
       <c r="A170"/>
       <c r="B170" s="6">
         <f>ROUND(0.47*SQRT(C168*(B146*B168+B166)*D168/(E168*A168)),2)</f>
-        <v>454.09</v>
+        <v>573.35</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.25">
@@ -4454,7 +4456,7 @@
       </c>
       <c r="B180" s="6">
         <f>ROUND(B178*B146,2)</f>
-        <v>1744.42</v>
+        <v>2788.85</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
@@ -4498,7 +4500,7 @@
       <c r="B187"/>
       <c r="C187">
         <f>B108</f>
-        <v>25.4</v>
+        <v>15.875</v>
       </c>
     </row>
     <row r="188" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -4518,7 +4520,7 @@
       <c r="B189"/>
       <c r="C189">
         <f>B125</f>
-        <v>3302</v>
+        <v>2063.75</v>
       </c>
     </row>
     <row r="190" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -4528,7 +4530,7 @@
       <c r="B190"/>
       <c r="C190">
         <f>B133</f>
-        <v>1019</v>
+        <v>636</v>
       </c>
     </row>
     <row r="191" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -4558,7 +4560,7 @@
       <c r="B193"/>
       <c r="C193">
         <f>B155</f>
-        <v>186.63</v>
+        <v>116.64</v>
       </c>
     </row>
     <row r="194" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -4568,7 +4570,7 @@
       <c r="B194"/>
       <c r="C194">
         <f>B156</f>
-        <v>590.69000000000005</v>
+        <v>369.18</v>
       </c>
     </row>
     <row r="195" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -4578,7 +4580,7 @@
       <c r="B195"/>
       <c r="C195">
         <f>B158</f>
-        <v>197.59</v>
+        <v>123.5</v>
       </c>
     </row>
     <row r="196" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -4588,7 +4590,7 @@
       <c r="B196"/>
       <c r="C196">
         <f>B159</f>
-        <v>602.85</v>
+        <v>376.78</v>
       </c>
     </row>
     <row r="197" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -4598,7 +4600,7 @@
       <c r="B197"/>
       <c r="C197">
         <f>B161</f>
-        <v>8.0299999999999994</v>
+        <v>5.16</v>
       </c>
     </row>
     <row r="198" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -4608,7 +4610,7 @@
       <c r="B198"/>
       <c r="C198">
         <f>B163</f>
-        <v>170.57</v>
+        <v>106.32</v>
       </c>
     </row>
     <row r="199" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -4618,7 +4620,7 @@
       <c r="B199"/>
       <c r="C199">
         <f>B164</f>
-        <v>574.63000000000011</v>
+        <v>358.86</v>
       </c>
     </row>
     <row r="200" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -4628,7 +4630,7 @@
       <c r="B200"/>
       <c r="C200">
         <f>B170</f>
-        <v>454.09</v>
+        <v>573.35</v>
       </c>
     </row>
     <row r="201" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -4667,7 +4669,7 @@
       <c r="B204"/>
       <c r="C204">
         <f>B180</f>
-        <v>1744.42</v>
+        <v>2788.85</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
@@ -4722,7 +4724,7 @@
         <v>60</v>
       </c>
       <c r="E212" s="22" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="F212" s="6">
         <v>850</v>
@@ -4745,7 +4747,7 @@
         <v>100</v>
       </c>
       <c r="E213" s="22" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="F213" s="6">
         <v>750</v>
@@ -4777,7 +4779,7 @@
     </row>
     <row r="218" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A218" s="4" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="219" spans="1:7" x14ac:dyDescent="0.25">
@@ -4788,7 +4790,7 @@
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" s="6" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B225" s="6">
         <v>250</v>
@@ -4796,7 +4798,7 @@
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" s="6" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B226" s="6">
         <v>220</v>
@@ -4806,141 +4808,141 @@
       <c r="A227" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="C227" s="25" t="s">
-        <v>233</v>
+      <c r="C227" s="26" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228"/>
-      <c r="C228" s="25"/>
+      <c r="C228" s="26"/>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B229" s="6">
         <f>2*B225+70</f>
         <v>570</v>
       </c>
-      <c r="C229" s="25"/>
+      <c r="C229" s="26"/>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B230" s="6">
         <f>2*B226+70</f>
         <v>510</v>
       </c>
-      <c r="C230" s="25"/>
+      <c r="C230" s="26"/>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="C231" s="25"/>
+        <v>230</v>
+      </c>
+      <c r="C231" s="26"/>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232"/>
-      <c r="C232" s="25"/>
+      <c r="C232" s="26"/>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B233" s="6">
         <f>1.8*B225</f>
         <v>450</v>
       </c>
-      <c r="C233" s="25"/>
+      <c r="C233" s="26"/>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B234" s="6">
         <f>1.8*B226</f>
         <v>396</v>
       </c>
-      <c r="C234" s="25"/>
+      <c r="C234" s="26"/>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C235" s="25"/>
+      <c r="C235" s="26"/>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" s="12" t="s">
-        <v>238</v>
-      </c>
-      <c r="C236" s="25"/>
+        <v>236</v>
+      </c>
+      <c r="C236" s="26"/>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B237" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C237" s="25"/>
+      <c r="C237" s="26"/>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B238" s="6">
         <v>1.75</v>
       </c>
-      <c r="C238" s="25"/>
+      <c r="C238" s="26"/>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" s="12" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B241" s="6">
         <f>1</f>
         <v>1</v>
       </c>
       <c r="C241" s="6" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" s="12" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B244" s="6">
         <v>6</v>
       </c>
-      <c r="C244" s="25" t="s">
-        <v>247</v>
+      <c r="C244" s="26" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B245" s="6">
         <v>6</v>
       </c>
-      <c r="C245" s="25"/>
+      <c r="C245" s="26"/>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" s="12" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B248" s="6">
         <f>30*B225^2.4</f>
@@ -4949,7 +4951,7 @@
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B249" s="6">
         <f>30*B226^2.4</f>
@@ -4958,35 +4960,35 @@
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251" s="12" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B252" s="6">
         <f>4*10^6</f>
         <v>4000000</v>
       </c>
       <c r="C252" s="6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="B254" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C254" s="6" t="s">
         <v>252</v>
-      </c>
-      <c r="B254" s="6" t="s">
-        <v>253</v>
-      </c>
-      <c r="C254" s="6" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B255" s="6">
         <f>60*1*C66*F2</f>
@@ -4995,7 +4997,7 @@
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B256" s="6">
         <f>60*1*D66*F2</f>
@@ -5004,7 +5006,7 @@
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B258" s="6">
         <v>1</v>
@@ -5012,7 +5014,7 @@
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B259" s="6">
         <v>1</v>
@@ -5020,7 +5022,7 @@
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B260" s="6">
         <v>1</v>
@@ -5028,7 +5030,7 @@
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B261">
         <v>1</v>
@@ -5041,7 +5043,7 @@
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B264" s="6">
         <f>ROUND(B229*B258/B237,2)</f>
@@ -5050,7 +5052,7 @@
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B265" s="6">
         <f>ROUND(B230*B260/B237,2)</f>
@@ -5059,12 +5061,12 @@
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A266" s="12" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B267" s="6">
         <f>ROUND(B233*B259/B238,2)</f>
@@ -5073,7 +5075,7 @@
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B268" s="6">
         <f>ROUND(B234*B260/B238,2)</f>
@@ -5082,7 +5084,7 @@
     </row>
     <row r="270" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A270" s="12" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.25">
@@ -5094,7 +5096,7 @@
     </row>
     <row r="272" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A272" s="11" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="273" spans="1:2" x14ac:dyDescent="0.25">
@@ -5106,7 +5108,7 @@
     </row>
     <row r="274" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A274" s="11" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="275" spans="1:2" x14ac:dyDescent="0.25">
@@ -5125,17 +5127,17 @@
     </row>
     <row r="278" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A278" s="4" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="279" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A279" s="4" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="280" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B280" s="6">
         <v>49.5</v>
@@ -5165,7 +5167,7 @@
     </row>
     <row r="285" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A285" s="11" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="286" spans="1:2" x14ac:dyDescent="0.25">
@@ -5177,23 +5179,23 @@
     </row>
     <row r="288" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A288" s="4" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" s="11" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" s="6" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B290" s="6">
         <f>0.01*B286</f>
         <v>1.4195</v>
       </c>
-      <c r="C290" s="25">
+      <c r="C290" s="26">
         <v>2</v>
       </c>
     </row>
@@ -5202,19 +5204,19 @@
         <f>0.02*B286</f>
         <v>2.839</v>
       </c>
-      <c r="C291" s="25"/>
+      <c r="C291" s="26"/>
       <c r="D291" s="6" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" s="12" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B294" s="6">
         <v>0</v>
@@ -5222,7 +5224,7 @@
     </row>
     <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" s="6" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B295" s="6">
         <f>ROUND(2*B286/(2*(B31+1)),2)</f>
@@ -5233,8 +5235,8 @@
       </c>
     </row>
     <row r="296" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A296" s="26" t="s">
-        <v>274</v>
+      <c r="A296" t="s">
+        <v>272</v>
       </c>
       <c r="B296" s="6">
         <f>C295*B31</f>
@@ -5245,27 +5247,27 @@
       </c>
     </row>
     <row r="297" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A297" s="27" t="s">
-        <v>275</v>
+      <c r="A297" s="12" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="298" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A298" s="26" t="s">
-        <v>276</v>
-      </c>
-      <c r="B298" s="28">
+      <c r="A298" t="s">
+        <v>274</v>
+      </c>
+      <c r="B298" s="25">
         <f>C290*(C296+C295)/2</f>
         <v>139</v>
       </c>
     </row>
     <row r="299" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A299" s="30" t="s">
+      <c r="A299" s="12" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A300" s="29" t="s">
-        <v>277</v>
+      <c r="A300" t="s">
+        <v>275</v>
       </c>
       <c r="B300" s="6">
         <f>ROUND(C296/C295,2)</f>
@@ -5273,12 +5275,12 @@
       </c>
     </row>
     <row r="301" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A301" s="30" t="s">
+      <c r="A301" s="12" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A302" s="29" t="s">
+      <c r="A302" t="s">
         <v>91</v>
       </c>
       <c r="B302" s="6">
@@ -5286,23 +5288,23 @@
         <v>1.7825311942958621E-3</v>
       </c>
       <c r="C302" s="6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="304" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A304" s="12" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A305" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="304" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A304" s="27" t="s">
+      <c r="B305" s="6" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="305" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A305" s="26" t="s">
+      <c r="C305" s="6" t="s">
         <v>280</v>
-      </c>
-      <c r="B305" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="C305" s="6" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.25">
@@ -5315,12 +5317,12 @@
     </row>
     <row r="307" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A307" s="4" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="308" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A308" s="27" t="s">
-        <v>284</v>
+      <c r="A308" s="12" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="309" spans="1:3" x14ac:dyDescent="0.25">
@@ -5333,13 +5335,13 @@
       </c>
     </row>
     <row r="310" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A310" s="27" t="s">
-        <v>285</v>
+      <c r="A310" s="12" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="311" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A311" s="6" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tính xong các thông số ăn khớp
</commit_message>
<xml_diff>
--- a/tínhtoans.xlsx
+++ b/tínhtoans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Đồ án tkm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9912E964-EA1A-4D28-8859-2C3A7BF400C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E84CE9C9-377A-44CF-A964-F48F0F996376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{75337E03-C337-4BFE-A279-78895F300CE2}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="304">
   <si>
     <t>Bánh răng trụ răng thẳng</t>
   </si>
@@ -900,6 +900,57 @@
   </si>
   <si>
     <t>Tra bảng 5.5 tr82 với n01 = 1200 và P_t &lt;= [P], có</t>
+  </si>
+  <si>
+    <t>Đường kính chia</t>
+  </si>
+  <si>
+    <t>d1</t>
+  </si>
+  <si>
+    <t>d2</t>
+  </si>
+  <si>
+    <t>Đường kính lăn</t>
+  </si>
+  <si>
+    <t>d_w1</t>
+  </si>
+  <si>
+    <t>d_w2</t>
+  </si>
+  <si>
+    <t>Đường kính đỉnh răng</t>
+  </si>
+  <si>
+    <t>Đường kính đáy răng</t>
+  </si>
+  <si>
+    <t>Đường kính cơ sở</t>
+  </si>
+  <si>
+    <t>d_b1</t>
+  </si>
+  <si>
+    <t>d_b2</t>
+  </si>
+  <si>
+    <t>Góc profin gốc</t>
+  </si>
+  <si>
+    <t>alpha</t>
+  </si>
+  <si>
+    <t>Góc profin răng</t>
+  </si>
+  <si>
+    <t>alpha_t</t>
+  </si>
+  <si>
+    <t>Góc ăn khớp</t>
+  </si>
+  <si>
+    <t>alpha_tw</t>
   </si>
 </sst>
 </file>
@@ -1063,7 +1114,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1117,6 +1168,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3076,7 +3131,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77F27C94-6297-45CB-8ED2-81D711DA05BE}">
-  <dimension ref="A1:J311"/>
+  <dimension ref="A1:J332"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="55.8984375" style="6" bestFit="1" customWidth="1"/>
@@ -5343,6 +5398,166 @@
       <c r="A311" s="6" t="s">
         <v>274</v>
       </c>
+      <c r="B311" s="6">
+        <f>B309+(B306+C306-0)*C290</f>
+        <v>139</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A312" s="11" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A313" s="27" t="s">
+        <v>288</v>
+      </c>
+      <c r="B313" s="6">
+        <f>C290*C295/COS(B294)</f>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="314" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A314" s="29" t="s">
+        <v>289</v>
+      </c>
+      <c r="B314" s="6">
+        <f>C290*C296/COS(B294)</f>
+        <v>236</v>
+      </c>
+    </row>
+    <row r="315" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A315" s="11" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A316" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="B316" s="6">
+        <f>ROUND(2*B311/(B300+1),2)</f>
+        <v>41.99</v>
+      </c>
+    </row>
+    <row r="317" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A317" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="B317" s="6">
+        <f>ROUND(B316*B300,2)</f>
+        <v>235.98</v>
+      </c>
+    </row>
+    <row r="318" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A318" s="30" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="319" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A319" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="B319" s="6">
+        <f>B313+2*(1+B306-0)*C290</f>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="320" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A320" s="27" t="s">
+        <v>169</v>
+      </c>
+      <c r="B320" s="6">
+        <f>B314+2*(1+C306-0)*C290</f>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="321" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A321" s="28" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="322" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A322" s="27" t="s">
+        <v>174</v>
+      </c>
+      <c r="B322" s="6">
+        <f>B313-(2.5-2*B306)*C290</f>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A323" s="27" t="s">
+        <v>175</v>
+      </c>
+      <c r="B323" s="6">
+        <f>B314-(2.5-2*C306)*C290</f>
+        <v>231</v>
+      </c>
+    </row>
+    <row r="324" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A324" s="28" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="325" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A325" s="27" t="s">
+        <v>296</v>
+      </c>
+      <c r="B325" s="6">
+        <f>ROUND(B313*COS(B328),2)</f>
+        <v>17.14</v>
+      </c>
+    </row>
+    <row r="326" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A326" s="27" t="s">
+        <v>297</v>
+      </c>
+      <c r="B326" s="6">
+        <f>ROUND(B314*COS(B328),2)</f>
+        <v>96.31</v>
+      </c>
+    </row>
+    <row r="327" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A327" s="28" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="328" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A328" s="27" t="s">
+        <v>299</v>
+      </c>
+      <c r="B328" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="329" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A329" s="28" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="330" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A330" s="27" t="s">
+        <v>301</v>
+      </c>
+      <c r="B330" s="6">
+        <f>DEGREES(ATAN(TAN(RADIANS(B328))/COS(RADIANS(B294))))</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="331" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A331" s="28" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="332" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A332" s="27" t="s">
+        <v>303</v>
+      </c>
+      <c r="B332">
+        <f>DEGREES(ACOS(B309*COS(RADIANS(B330))/B311))</f>
+        <v>19.999999999999989</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
hoàn thành tính toán bộ truyền trong và ngoài
</commit_message>
<xml_diff>
--- a/tínhtoans.xlsx
+++ b/tínhtoans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Đồ án tkm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E84CE9C9-377A-44CF-A964-F48F0F996376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F02D2B6D-C6BD-4219-A7B9-60D00225043B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{75337E03-C337-4BFE-A279-78895F300CE2}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{75337E03-C337-4BFE-A279-78895F300CE2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,8 +38,340 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="32">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="4"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="5"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="6"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="7"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="8"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="9"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="10"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="11"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="12"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="13"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="14"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="15"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="16"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="17"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="18"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="19"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="20"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="21"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="22"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="23"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="24"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="25"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="26"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="27"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="28"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="29"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="30"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="31"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="32">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+    <bk>
+      <rc t="1" v="1"/>
+    </bk>
+    <bk>
+      <rc t="1" v="2"/>
+    </bk>
+    <bk>
+      <rc t="1" v="3"/>
+    </bk>
+    <bk>
+      <rc t="1" v="4"/>
+    </bk>
+    <bk>
+      <rc t="1" v="5"/>
+    </bk>
+    <bk>
+      <rc t="1" v="6"/>
+    </bk>
+    <bk>
+      <rc t="1" v="7"/>
+    </bk>
+    <bk>
+      <rc t="1" v="8"/>
+    </bk>
+    <bk>
+      <rc t="1" v="9"/>
+    </bk>
+    <bk>
+      <rc t="1" v="10"/>
+    </bk>
+    <bk>
+      <rc t="1" v="11"/>
+    </bk>
+    <bk>
+      <rc t="1" v="12"/>
+    </bk>
+    <bk>
+      <rc t="1" v="13"/>
+    </bk>
+    <bk>
+      <rc t="1" v="14"/>
+    </bk>
+    <bk>
+      <rc t="1" v="15"/>
+    </bk>
+    <bk>
+      <rc t="1" v="16"/>
+    </bk>
+    <bk>
+      <rc t="1" v="17"/>
+    </bk>
+    <bk>
+      <rc t="1" v="18"/>
+    </bk>
+    <bk>
+      <rc t="1" v="19"/>
+    </bk>
+    <bk>
+      <rc t="1" v="20"/>
+    </bk>
+    <bk>
+      <rc t="1" v="21"/>
+    </bk>
+    <bk>
+      <rc t="1" v="22"/>
+    </bk>
+    <bk>
+      <rc t="1" v="23"/>
+    </bk>
+    <bk>
+      <rc t="1" v="24"/>
+    </bk>
+    <bk>
+      <rc t="1" v="25"/>
+    </bk>
+    <bk>
+      <rc t="1" v="26"/>
+    </bk>
+    <bk>
+      <rc t="1" v="27"/>
+    </bk>
+    <bk>
+      <rc t="1" v="28"/>
+    </bk>
+    <bk>
+      <rc t="1" v="29"/>
+    </bk>
+    <bk>
+      <rc t="1" v="30"/>
+    </bk>
+    <bk>
+      <rc t="1" v="31"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="378">
   <si>
     <t>Bánh răng trụ răng thẳng</t>
   </si>
@@ -731,9 +1063,6 @@
     <t>3.2. Xác định ứng suất cho phép</t>
   </si>
   <si>
-    <t>Ứng suất uống cho phép</t>
-  </si>
-  <si>
     <t>tra bảng 6.2 tr 94</t>
   </si>
   <si>
@@ -951,13 +1280,260 @@
   </si>
   <si>
     <t>alpha_tw</t>
+  </si>
+  <si>
+    <t>3.3.4. Kiểm nghiệm răng về độ bền tiếp xúc</t>
+  </si>
+  <si>
+    <t>Hệ số kể đến cơ tính vật liệu của BR ăn khớp</t>
+  </si>
+  <si>
+    <t>Z_M (bảng 6.5 tr 96)</t>
+  </si>
+  <si>
+    <t>Z_H</t>
+  </si>
+  <si>
+    <r>
+      <t>Z_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>ξ</t>
+    </r>
+  </si>
+  <si>
+    <t>Hệ số kể đến hình dạng bề mặt tiếp xúc</t>
+  </si>
+  <si>
+    <t>Hệ số trùng khớp ngang</t>
+  </si>
+  <si>
+    <t>Hệ số kể đến sự trùng khớp của răng</t>
+  </si>
+  <si>
+    <t>Hệ số tải trọng khi tính về tiếp xúc</t>
+  </si>
+  <si>
+    <t>K_H</t>
+  </si>
+  <si>
+    <t>K_HB (Bảng 6.7 tr 98)</t>
+  </si>
+  <si>
+    <t>K_HA</t>
+  </si>
+  <si>
+    <t>vận tốc vòng</t>
+  </si>
+  <si>
+    <t>CCX 8</t>
+  </si>
+  <si>
+    <t>Bảng 6.13</t>
+  </si>
+  <si>
+    <t>Tra bảng P2.3 tr 250</t>
+  </si>
+  <si>
+    <t>K_Hv (nội suy)</t>
+  </si>
+  <si>
+    <t>K_Fv (nội suy)</t>
+  </si>
+  <si>
+    <t>Ứng suất tiếp xúc xuất hiện trên mặt răng của bộ truyền</t>
+  </si>
+  <si>
+    <t>Chiều rộng vành răng</t>
+  </si>
+  <si>
+    <t>b_w</t>
+  </si>
+  <si>
+    <t>Thỏa mãn &lt; 463.64</t>
+  </si>
+  <si>
+    <t>3.3.5. Kiểm nghiệm răng về độ bền uốn</t>
+  </si>
+  <si>
+    <t>ξ_a</t>
+  </si>
+  <si>
+    <t>Hệ số trùng khớp dọc</t>
+  </si>
+  <si>
+    <t>ξ_b</t>
+  </si>
+  <si>
+    <t>Hệ số kể đến sự  trùng khớp của BR</t>
+  </si>
+  <si>
+    <r>
+      <t>Y_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>ξ</t>
+    </r>
+  </si>
+  <si>
+    <t>Hệ số kể đến độ nghiêng của răng</t>
+  </si>
+  <si>
+    <t>Y_B</t>
+  </si>
+  <si>
+    <t>Y_F1</t>
+  </si>
+  <si>
+    <t>Y_F2</t>
+  </si>
+  <si>
+    <t>Hệ số dạng răng (nội suy)</t>
+  </si>
+  <si>
+    <t>Hệ số kể đến sự phân bố không đều tải trọng cho các đôi răng đồng thời ăn khớp khi tính về uốn</t>
+  </si>
+  <si>
+    <t>K_Fv</t>
+  </si>
+  <si>
+    <t>Hệ số tải trọng khi tính về uốn</t>
+  </si>
+  <si>
+    <t>K_Fa</t>
+  </si>
+  <si>
+    <t>Hệ số kể đến tải trọng động xuất hiện trong vùng ăn khớp khi tính về uốn</t>
+  </si>
+  <si>
+    <t>K_F</t>
+  </si>
+  <si>
+    <t>K_FB (Bảng 6.7 tr 98)</t>
+  </si>
+  <si>
+    <t>Ứng suất uốn của bánh răng chủ động</t>
+  </si>
+  <si>
+    <t>Ứng suất uốn của bánh răng bị động</t>
+  </si>
+  <si>
+    <t>Thỏa mãn yêu cầu</t>
+  </si>
+  <si>
+    <t>3.3.6. Kiểm nghiệm răng về quá tải</t>
+  </si>
+  <si>
+    <t>Hệ số quá tải</t>
+  </si>
+  <si>
+    <t>K_qt</t>
+  </si>
+  <si>
+    <t>Tra 234</t>
+  </si>
+  <si>
+    <t>thỏa mãn &lt; 1624</t>
+  </si>
+  <si>
+    <t>Thỏa mãn &lt; 464</t>
+  </si>
+  <si>
+    <t>Thỏa mãn &lt; 360</t>
+  </si>
+  <si>
+    <t>3.3.7. Bảng thông số thiết kế cặp bánh răng</t>
+  </si>
+  <si>
+    <t>Ký hiệu (đơn vị)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số răng bánh chủ động </t>
+  </si>
+  <si>
+    <t>Số răng bánh bị động</t>
+  </si>
+  <si>
+    <t>Môđun</t>
+  </si>
+  <si>
+    <t>Chiều rộng vành răng chủ động</t>
+  </si>
+  <si>
+    <t>Chiều rộng vành răng bị động</t>
+  </si>
+  <si>
+    <t>Tỷ số truyền thực</t>
+  </si>
+  <si>
+    <t>3,71</t>
+  </si>
+  <si>
+    <t>Cấp chính xác</t>
+  </si>
+  <si>
+    <t>Vật liệu làm bánh răng</t>
+  </si>
+  <si>
+    <t>C45</t>
+  </si>
+  <si>
+    <t>Độ cứng  bề mặt bánh răng chủ động</t>
+  </si>
+  <si>
+    <t>Độ cứng bề mặt bánh răng bị động</t>
+  </si>
+  <si>
+    <t>Đường kính vòng lăn bánh răng chủ động</t>
+  </si>
+  <si>
+    <t>Đường kính vòng lăn bánh răng bị động</t>
+  </si>
+  <si>
+    <t>Đường kính vòng đỉnh bánh răng chủ động</t>
+  </si>
+  <si>
+    <t>(mm)</t>
+  </si>
+  <si>
+    <t>Đường kính vòng đỉnh bánh răng bị động</t>
+  </si>
+  <si>
+    <t>Đường kính vòng đáy răng bánh chủ động</t>
+  </si>
+  <si>
+    <t>Đường kính vòng đáy răng bánh bị động</t>
+  </si>
+  <si>
+    <t>Đường kính vòng cơ sở bánh răng chủ động</t>
+  </si>
+  <si>
+    <t>Đường kính vòng cơ sở bánh răng bị động</t>
+  </si>
+  <si>
+    <t>Góc áp lực</t>
+  </si>
+  <si>
+    <t>Vận tốc vòng của bánh răng</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1037,6 +1613,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1058,7 +1653,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -1109,12 +1704,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1165,13 +1784,25 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2732,7 +3363,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>221226</xdr:colOff>
+      <xdr:colOff>211701</xdr:colOff>
       <xdr:row>287</xdr:row>
       <xdr:rowOff>93398</xdr:rowOff>
     </xdr:to>
@@ -2776,9 +3407,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>1059741</xdr:colOff>
+      <xdr:colOff>1050216</xdr:colOff>
       <xdr:row>337</xdr:row>
-      <xdr:rowOff>23446</xdr:rowOff>
+      <xdr:rowOff>15826</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2811,7 +3442,1041 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>357</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>3962743</xdr:colOff>
+      <xdr:row>361</xdr:row>
+      <xdr:rowOff>17206</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="Picture 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6DA46C7-E958-6608-CFD2-C9AE1BAC6DF2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="61236225"/>
+          <a:ext cx="3962743" cy="704911"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>355</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>182880</xdr:colOff>
+      <xdr:row>356</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="29" name="Picture 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0A258AF1-39FE-0F86-DCB9-74B152521CCC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="62179200"/>
+          <a:ext cx="182880" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2800350</xdr:colOff>
+      <xdr:row>355</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>3095625</xdr:colOff>
+      <xdr:row>356</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="30" name="Picture 29">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D42E70E-F0E4-238B-155B-5966EBEDEAE5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="9505950" y="60893325"/>
+          <a:ext cx="295275" cy="200025"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1552575</xdr:colOff>
+      <xdr:row>363</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>817652</xdr:colOff>
+      <xdr:row>368</xdr:row>
+      <xdr:rowOff>91521</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="33" name="Picture 32">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1C58CF17-5D2F-995E-1C58-57C9D48D3294}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10134600" y="62617350"/>
+          <a:ext cx="4703852" cy="929721"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>378</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>379</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="34" name="Picture 33">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{93F68DF0-21C5-A663-504D-F0B7178CC66A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId28">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="66743580"/>
+          <a:ext cx="228600" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>380</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>381</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="35" name="Picture 34">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9173B798-0792-3999-3FE4-295E6DE0FEF9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId29">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="67094100"/>
+          <a:ext cx="228600" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1190625</xdr:colOff>
+      <xdr:row>385</xdr:row>
+      <xdr:rowOff>159575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>4497705</xdr:colOff>
+      <xdr:row>388</xdr:row>
+      <xdr:rowOff>53384</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="36" name="Picture 35">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{288AE920-A656-6089-0303-8810D963EB59}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1190625" y="66710750"/>
+          <a:ext cx="3307080" cy="402444"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>393</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>426720</xdr:colOff>
+      <xdr:row>394</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="37" name="Picture 36">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AFC62AB2-9723-25F8-3B4A-446BC574A867}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId31">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="69372480"/>
+          <a:ext cx="426720" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1314450</xdr:colOff>
+      <xdr:row>394</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>4968556</xdr:colOff>
+      <xdr:row>396</xdr:row>
+      <xdr:rowOff>133390</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="38" name="Picture 37">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7BA46608-ECDE-9717-BC9C-1B85A5837BAB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId32"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1314450" y="68113275"/>
+          <a:ext cx="3644581" cy="457240"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>397</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>480060</xdr:colOff>
+      <xdr:row>398</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="39" name="Picture 38">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7E5530B2-2416-0F93-7555-5390798D88A1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId33">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="70073520"/>
+          <a:ext cx="480060" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>398</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>480060</xdr:colOff>
+      <xdr:row>399</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="40" name="Picture 39">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D53EE0C1-E74F-FF3B-E055-9C9B7CE39AA2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId34">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="70248780"/>
+          <a:ext cx="480060" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>418</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>243840</xdr:colOff>
+      <xdr:row>418</xdr:row>
+      <xdr:rowOff>205740</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="41" name="Picture 40">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8257366D-1879-10E3-F2CC-C81BFEBAA2E1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId35">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="6134100" y="74447400"/>
+          <a:ext cx="243840" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>419</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>243840</xdr:colOff>
+      <xdr:row>419</xdr:row>
+      <xdr:rowOff>205740</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="42" name="Picture 41">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DDA959F7-0575-FDB6-E473-18F860F695C7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId36">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="6134100" y="74668380"/>
+          <a:ext cx="243840" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="32">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>2</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>3</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>4</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>5</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>6</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>7</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>8</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>9</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>10</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>11</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>12</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>13</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>14</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>15</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>16</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>17</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>18</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>19</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>20</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>21</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>22</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>23</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>24</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>25</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>26</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>27</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>28</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>29</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>30</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>31</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+  <rel r:id="rId2"/>
+  <rel r:id="rId3"/>
+  <rel r:id="rId4"/>
+  <rel r:id="rId5"/>
+  <rel r:id="rId6"/>
+  <rel r:id="rId7"/>
+  <rel r:id="rId8"/>
+  <rel r:id="rId9"/>
+  <rel r:id="rId10"/>
+  <rel r:id="rId11"/>
+  <rel r:id="rId12"/>
+  <rel r:id="rId13"/>
+  <rel r:id="rId14"/>
+  <rel r:id="rId15"/>
+  <rel r:id="rId16"/>
+  <rel r:id="rId17"/>
+  <rel r:id="rId18"/>
+  <rel r:id="rId19"/>
+  <rel r:id="rId20"/>
+  <rel r:id="rId21"/>
+  <rel r:id="rId22"/>
+  <rel r:id="rId23"/>
+  <rel r:id="rId24"/>
+  <rel r:id="rId25"/>
+  <rel r:id="rId26"/>
+  <rel r:id="rId27"/>
+  <rel r:id="rId28"/>
+  <rel r:id="rId29"/>
+  <rel r:id="rId30"/>
+  <rel r:id="rId31"/>
+  <rel r:id="rId32"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3131,10 +4796,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77F27C94-6297-45CB-8ED2-81D711DA05BE}">
-  <dimension ref="A1:J332"/>
+  <dimension ref="A1:J426"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="55.8984375" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="80.5" style="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32.09765625" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="41.296875" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="30.09765625" style="6" bestFit="1" customWidth="1"/>
@@ -3858,7 +5523,7 @@
       <c r="B90" s="6">
         <v>1.25</v>
       </c>
-      <c r="F90" s="26" t="s">
+      <c r="F90" s="27" t="s">
         <v>118</v>
       </c>
     </row>
@@ -3866,7 +5531,7 @@
       <c r="A91" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="F91" s="26"/>
+      <c r="F91" s="27"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
@@ -3878,13 +5543,13 @@
       <c r="C92" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="F92" s="26"/>
+      <c r="F92" s="27"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="F93" s="26"/>
+      <c r="F93" s="27"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
@@ -3896,13 +5561,13 @@
       <c r="C94" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="F94" s="26"/>
+      <c r="F94" s="27"/>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="F95" s="26"/>
+      <c r="F95" s="27"/>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
@@ -3914,13 +5579,13 @@
       <c r="C96" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="F96" s="26"/>
+      <c r="F96" s="27"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="F97" s="26"/>
+      <c r="F97" s="27"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
@@ -3932,13 +5597,13 @@
       <c r="C98" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="F98" s="26"/>
+      <c r="F98" s="27"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="F99" s="26"/>
+      <c r="F99" s="27"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
@@ -3950,7 +5615,7 @@
       <c r="C100" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="F100" s="26"/>
+      <c r="F100" s="27"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="12" t="s">
@@ -3982,7 +5647,7 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
@@ -4177,7 +5842,7 @@
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B138" s="6" t="s">
         <v>146</v>
@@ -4350,7 +6015,7 @@
         <v>10.16</v>
       </c>
       <c r="D160" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
@@ -4845,7 +6510,7 @@
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B225" s="6">
         <v>250</v>
@@ -4853,7 +6518,7 @@
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" s="6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B226" s="6">
         <v>220</v>
@@ -4863,141 +6528,141 @@
       <c r="A227" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="C227" s="26" t="s">
-        <v>231</v>
+      <c r="C227" s="27" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228"/>
-      <c r="C228" s="26"/>
+      <c r="C228" s="27"/>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B229" s="6">
         <f>2*B225+70</f>
         <v>570</v>
       </c>
-      <c r="C229" s="26"/>
+      <c r="C229" s="27"/>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B230" s="6">
         <f>2*B226+70</f>
         <v>510</v>
       </c>
-      <c r="C230" s="26"/>
+      <c r="C230" s="27"/>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="C231" s="26"/>
+        <v>256</v>
+      </c>
+      <c r="C231" s="27"/>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232"/>
-      <c r="C232" s="26"/>
+      <c r="C232" s="27"/>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B233" s="6">
         <f>1.8*B225</f>
         <v>450</v>
       </c>
-      <c r="C233" s="26"/>
+      <c r="C233" s="27"/>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B234" s="6">
         <f>1.8*B226</f>
         <v>396</v>
       </c>
-      <c r="C234" s="26"/>
+      <c r="C234" s="27"/>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C235" s="26"/>
+      <c r="C235" s="27"/>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" s="12" t="s">
-        <v>236</v>
-      </c>
-      <c r="C236" s="26"/>
+        <v>235</v>
+      </c>
+      <c r="C236" s="27"/>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B237" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C237" s="26"/>
+      <c r="C237" s="27"/>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B238" s="6">
         <v>1.75</v>
       </c>
-      <c r="C238" s="26"/>
+      <c r="C238" s="27"/>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" s="12" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B241" s="6">
         <f>1</f>
         <v>1</v>
       </c>
       <c r="C241" s="6" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" s="12" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B244" s="6">
         <v>6</v>
       </c>
-      <c r="C244" s="26" t="s">
-        <v>245</v>
+      <c r="C244" s="27" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B245" s="6">
         <v>6</v>
       </c>
-      <c r="C245" s="26"/>
+      <c r="C245" s="27"/>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" s="12" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B248" s="6">
         <f>30*B225^2.4</f>
@@ -5006,7 +6671,7 @@
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B249" s="6">
         <f>30*B226^2.4</f>
@@ -5015,35 +6680,35 @@
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251" s="12" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B252" s="6">
         <f>4*10^6</f>
         <v>4000000</v>
       </c>
       <c r="C252" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="B254" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="B254" s="6" t="s">
+      <c r="C254" s="6" t="s">
         <v>251</v>
-      </c>
-      <c r="C254" s="6" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B255" s="6">
         <f>60*1*C66*F2</f>
@@ -5052,7 +6717,7 @@
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B256" s="6">
         <f>60*1*D66*F2</f>
@@ -5061,7 +6726,7 @@
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B258" s="6">
         <v>1</v>
@@ -5069,7 +6734,7 @@
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B259" s="6">
         <v>1</v>
@@ -5077,7 +6742,7 @@
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B260" s="6">
         <v>1</v>
@@ -5085,7 +6750,7 @@
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B261">
         <v>1</v>
@@ -5098,7 +6763,7 @@
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B264" s="6">
         <f>ROUND(B229*B258/B237,2)</f>
@@ -5107,7 +6772,7 @@
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B265" s="6">
         <f>ROUND(B230*B260/B237,2)</f>
@@ -5116,12 +6781,12 @@
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A266" s="12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B267" s="6">
         <f>ROUND(B233*B259/B238,2)</f>
@@ -5130,7 +6795,7 @@
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B268" s="6">
         <f>ROUND(B234*B260/B238,2)</f>
@@ -5139,7 +6804,7 @@
     </row>
     <row r="270" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A270" s="12" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.25">
@@ -5151,7 +6816,7 @@
     </row>
     <row r="272" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A272" s="11" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="273" spans="1:2" x14ac:dyDescent="0.25">
@@ -5163,7 +6828,7 @@
     </row>
     <row r="274" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A274" s="11" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="275" spans="1:2" x14ac:dyDescent="0.25">
@@ -5182,17 +6847,17 @@
     </row>
     <row r="278" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A278" s="4" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="279" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A279" s="4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="280" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B280" s="6">
         <v>49.5</v>
@@ -5222,7 +6887,7 @@
     </row>
     <row r="285" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A285" s="11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="286" spans="1:2" x14ac:dyDescent="0.25">
@@ -5234,23 +6899,23 @@
     </row>
     <row r="288" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A288" s="4" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" s="11" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" s="6" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B290" s="6">
         <f>0.01*B286</f>
         <v>1.4195</v>
       </c>
-      <c r="C290" s="26">
+      <c r="C290" s="27">
         <v>2</v>
       </c>
     </row>
@@ -5259,19 +6924,19 @@
         <f>0.02*B286</f>
         <v>2.839</v>
       </c>
-      <c r="C291" s="26"/>
+      <c r="C291" s="27"/>
       <c r="D291" s="6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" s="12" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B294" s="6">
         <v>0</v>
@@ -5279,7 +6944,7 @@
     </row>
     <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B295" s="6">
         <f>ROUND(2*B286/(2*(B31+1)),2)</f>
@@ -5291,7 +6956,7 @@
     </row>
     <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B296" s="6">
         <f>C295*B31</f>
@@ -5303,12 +6968,12 @@
     </row>
     <row r="297" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A297" s="12" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="298" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B298" s="25">
         <f>C290*(C296+C295)/2</f>
@@ -5322,7 +6987,7 @@
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B300" s="6">
         <f>ROUND(C296/C295,2)</f>
@@ -5343,23 +7008,23 @@
         <v>1.7825311942958621E-3</v>
       </c>
       <c r="C302" s="6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="304" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A304" s="12" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="305" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
+        <v>277</v>
+      </c>
+      <c r="B305" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="B305" s="6" t="s">
+      <c r="C305" s="6" t="s">
         <v>279</v>
-      </c>
-      <c r="C305" s="6" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.25">
@@ -5372,12 +7037,12 @@
     </row>
     <row r="307" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A307" s="4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="308" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A308" s="12" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="309" spans="1:3" x14ac:dyDescent="0.25">
@@ -5391,12 +7056,12 @@
     </row>
     <row r="310" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A310" s="12" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="311" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A311" s="6" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B311" s="6">
         <f>B309+(B306+C306-0)*C290</f>
@@ -5405,12 +7070,12 @@
     </row>
     <row r="312" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A312" s="11" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A313" t="s">
         <v>287</v>
-      </c>
-    </row>
-    <row r="313" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A313" s="27" t="s">
-        <v>288</v>
       </c>
       <c r="B313" s="6">
         <f>C290*C295/COS(B294)</f>
@@ -5418,8 +7083,8 @@
       </c>
     </row>
     <row r="314" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A314" s="29" t="s">
-        <v>289</v>
+      <c r="A314" s="26" t="s">
+        <v>288</v>
       </c>
       <c r="B314" s="6">
         <f>C290*C296/COS(B294)</f>
@@ -5428,12 +7093,12 @@
     </row>
     <row r="315" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A315" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="316" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A316" s="6" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B316" s="6">
         <f>ROUND(2*B311/(B300+1),2)</f>
@@ -5442,7 +7107,7 @@
     </row>
     <row r="317" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A317" s="6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B317" s="6">
         <f>ROUND(B316*B300,2)</f>
@@ -5450,8 +7115,8 @@
       </c>
     </row>
     <row r="318" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A318" s="30" t="s">
-        <v>293</v>
+      <c r="A318" s="12" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="319" spans="1:3" x14ac:dyDescent="0.25">
@@ -5464,7 +7129,7 @@
       </c>
     </row>
     <row r="320" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A320" s="27" t="s">
+      <c r="A320" t="s">
         <v>169</v>
       </c>
       <c r="B320" s="6">
@@ -5473,12 +7138,12 @@
       </c>
     </row>
     <row r="321" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A321" s="28" t="s">
-        <v>294</v>
+      <c r="A321" s="12" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="322" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A322" s="27" t="s">
+      <c r="A322" t="s">
         <v>174</v>
       </c>
       <c r="B322" s="6">
@@ -5487,7 +7152,7 @@
       </c>
     </row>
     <row r="323" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A323" s="27" t="s">
+      <c r="A323" t="s">
         <v>175</v>
       </c>
       <c r="B323" s="6">
@@ -5496,13 +7161,13 @@
       </c>
     </row>
     <row r="324" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A324" s="28" t="s">
+      <c r="A324" s="12" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="325" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A325" t="s">
         <v>295</v>
-      </c>
-    </row>
-    <row r="325" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A325" s="27" t="s">
-        <v>296</v>
       </c>
       <c r="B325" s="6">
         <f>ROUND(B313*COS(B328),2)</f>
@@ -5510,8 +7175,8 @@
       </c>
     </row>
     <row r="326" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A326" s="27" t="s">
-        <v>297</v>
+      <c r="A326" t="s">
+        <v>296</v>
       </c>
       <c r="B326" s="6">
         <f>ROUND(B314*COS(B328),2)</f>
@@ -5519,26 +7184,26 @@
       </c>
     </row>
     <row r="327" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A327" s="28" t="s">
+      <c r="A327" s="12" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="328" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A328" t="s">
         <v>298</v>
-      </c>
-    </row>
-    <row r="328" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A328" s="27" t="s">
-        <v>299</v>
       </c>
       <c r="B328" s="6">
         <v>20</v>
       </c>
     </row>
     <row r="329" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A329" s="28" t="s">
+      <c r="A329" s="12" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="330" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A330" t="s">
         <v>300</v>
-      </c>
-    </row>
-    <row r="330" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A330" s="27" t="s">
-        <v>301</v>
       </c>
       <c r="B330" s="6">
         <f>DEGREES(ATAN(TAN(RADIANS(B328))/COS(RADIANS(B294))))</f>
@@ -5546,17 +7211,627 @@
       </c>
     </row>
     <row r="331" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A331" s="28" t="s">
+      <c r="A331" s="12" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="332" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A332" t="s">
         <v>302</v>
-      </c>
-    </row>
-    <row r="332" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A332" s="27" t="s">
-        <v>303</v>
       </c>
       <c r="B332">
         <f>DEGREES(ACOS(B309*COS(RADIANS(B330))/B311))</f>
         <v>19.999999999999989</v>
+      </c>
+    </row>
+    <row r="335" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A335" s="4" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A339" s="11" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A340" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="B340" s="6">
+        <f>B281*B311</f>
+        <v>41.699999999999996</v>
+      </c>
+    </row>
+    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A342" s="11" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A343" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="B343" s="6">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A344" s="11" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A345" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="B345" s="6">
+        <f>ROUND(SQRT(2*COS(0)/SIN(RADIANS(2*B332))),2)</f>
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A346" s="29" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A347" s="28" t="s">
+        <v>326</v>
+      </c>
+      <c r="B347" s="6">
+        <f>ROUND((1.88-3.2*(1/C295+1/C296))*COS(B306),2)</f>
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A348" s="29" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A349" s="28" t="s">
+        <v>328</v>
+      </c>
+      <c r="B349" s="6">
+        <f>B340*SIN(B306)/(C290*PI())</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A350" s="29" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="351" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A351" s="28" t="s">
+        <v>307</v>
+      </c>
+      <c r="B351" s="6">
+        <f>ROUND(SQRT((4-B347)/3),2)</f>
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A352" s="29" t="s">
+        <v>311</v>
+      </c>
+      <c r="C352" s="22" t="s">
+        <v>313</v>
+      </c>
+      <c r="D352" s="22" t="s">
+        <v>314</v>
+      </c>
+      <c r="E352" s="22" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="353" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A353" s="28" t="s">
+        <v>312</v>
+      </c>
+      <c r="B353" s="6">
+        <f>ROUND(C353*D353*F356,2)</f>
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="C353" s="6">
+        <v>1.03</v>
+      </c>
+      <c r="D353" s="6">
+        <v>1</v>
+      </c>
+      <c r="E353" s="6">
+        <f>ROUND(PI()*B316*C66/60000,2)</f>
+        <v>3.18</v>
+      </c>
+      <c r="F353" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="G353" s="6" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="354" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A354" s="28"/>
+      <c r="C354" s="22" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="355" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A355" s="29" t="s">
+        <v>321</v>
+      </c>
+      <c r="C355" s="6">
+        <v>1.05</v>
+      </c>
+      <c r="E355" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="F355" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="G355" s="6" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="356" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A356"/>
+      <c r="B356" s="6">
+        <f>ROUND(B343*B345*B351*SQRT(2*C67*B353*(B300+1)/(B340*B300*B316^2)),2)</f>
+        <v>438.18</v>
+      </c>
+      <c r="C356" s="21"/>
+      <c r="D356" s="6">
+        <f>B271</f>
+        <v>463.64</v>
+      </c>
+      <c r="F356" s="6">
+        <v>1.1272</v>
+      </c>
+      <c r="G356" s="6">
+        <v>1.3062</v>
+      </c>
+    </row>
+    <row r="357" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B357" s="6" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="363" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A363" s="4" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="365" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A365" s="11" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="366" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A366" s="28" t="s">
+        <v>330</v>
+      </c>
+      <c r="B366" s="6">
+        <f>ROUND(1/B347,3)</f>
+        <v>0.58799999999999997</v>
+      </c>
+    </row>
+    <row r="367" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A367" s="29" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="368" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A368" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="B368" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="369" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A369" s="29" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="370" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A370" s="28" t="s">
+        <v>333</v>
+      </c>
+      <c r="B370" s="6">
+        <v>4.04</v>
+      </c>
+    </row>
+    <row r="371" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A371" s="30" t="s">
+        <v>334</v>
+      </c>
+      <c r="B371" s="6">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="372" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A372" s="11" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="373" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A373" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="B373" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="374" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A374" s="11" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="375" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A375" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="B375" s="28">
+        <f>G356</f>
+        <v>1.3062</v>
+      </c>
+    </row>
+    <row r="376" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A376" s="11" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="377" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A377" s="28" t="s">
+        <v>341</v>
+      </c>
+      <c r="B377" s="6">
+        <f>C355*B373*B375</f>
+        <v>1.37151</v>
+      </c>
+    </row>
+    <row r="378" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A378" s="29" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="379" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A379"/>
+      <c r="B379" s="6">
+        <f>ROUND(2*C67*B377*B366*B368*B370/(B340*B316*C290),2)</f>
+        <v>53.37</v>
+      </c>
+    </row>
+    <row r="380" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A380" s="29" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="381" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A381"/>
+      <c r="B381" s="6">
+        <f>ROUND(B379*B371/B370,2)</f>
+        <v>47.56</v>
+      </c>
+    </row>
+    <row r="383" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A383" s="6" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="385" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A385" s="4" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="391" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A391" s="11" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="392" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A392" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="B392" s="6">
+        <v>2</v>
+      </c>
+      <c r="C392" s="6" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="394" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A394"/>
+      <c r="B394" s="6">
+        <f>ROUND(B356*SQRT(B392),2)</f>
+        <v>619.67999999999995</v>
+      </c>
+      <c r="C394" s="6" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="398" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A398"/>
+      <c r="B398" s="6">
+        <f>B379*B392</f>
+        <v>106.74</v>
+      </c>
+      <c r="C398" s="6" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="399" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A399"/>
+      <c r="B399" s="6">
+        <f>B381*B392</f>
+        <v>95.12</v>
+      </c>
+      <c r="C399" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="402" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A402" s="4" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="403" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="404" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A404" s="31" t="s">
+        <v>200</v>
+      </c>
+      <c r="B404" s="32" t="s">
+        <v>354</v>
+      </c>
+      <c r="C404" s="32" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="405" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A405" s="33" t="s">
+        <v>132</v>
+      </c>
+      <c r="B405" s="34" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C405" s="34">
+        <f>B298</f>
+        <v>139</v>
+      </c>
+    </row>
+    <row r="406" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A406" s="33" t="s">
+        <v>355</v>
+      </c>
+      <c r="B406" s="34" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C406" s="34">
+        <f>C295</f>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="407" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A407" s="33" t="s">
+        <v>356</v>
+      </c>
+      <c r="B407" s="34" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C407" s="34">
+        <f>C296</f>
+        <v>118</v>
+      </c>
+    </row>
+    <row r="408" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A408" s="33" t="s">
+        <v>357</v>
+      </c>
+      <c r="B408" s="34" t="e" vm="4">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C408" s="34">
+        <f>C290</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="409" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A409" s="33" t="s">
+        <v>301</v>
+      </c>
+      <c r="B409" s="34" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C409" s="34">
+        <f>B332</f>
+        <v>19.999999999999989</v>
+      </c>
+    </row>
+    <row r="410" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A410" s="33" t="s">
+        <v>358</v>
+      </c>
+      <c r="B410" s="34" t="e" vm="6">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C410" s="34">
+        <f>C295</f>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="411" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A411" s="33" t="s">
+        <v>359</v>
+      </c>
+      <c r="B411" s="34" t="e" vm="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C411" s="34" t="e" vm="8">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="412" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A412" s="33" t="s">
+        <v>360</v>
+      </c>
+      <c r="B412" s="34" t="e" vm="9">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C412" s="34" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="413" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A413" s="33" t="s">
+        <v>362</v>
+      </c>
+      <c r="B413" s="34"/>
+      <c r="C413" s="34" t="e" vm="10">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="414" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A414" s="33" t="s">
+        <v>363</v>
+      </c>
+      <c r="B414" s="34" t="s">
+        <v>364</v>
+      </c>
+      <c r="C414" s="34" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="415" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A415" s="33" t="s">
+        <v>365</v>
+      </c>
+      <c r="B415" s="34" t="e" vm="11">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C415" s="34" t="e" vm="12">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="416" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A416" s="33" t="s">
+        <v>366</v>
+      </c>
+      <c r="B416" s="34" t="e" vm="13">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C416" s="34" t="e" vm="14">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="417" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A417" s="33" t="s">
+        <v>367</v>
+      </c>
+      <c r="B417" s="34" t="e" vm="15">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C417" s="34" t="e" vm="16">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="418" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A418" s="33" t="s">
+        <v>368</v>
+      </c>
+      <c r="B418" s="34" t="e" vm="17">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C418" s="34" t="e" vm="18">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="419" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A419" s="33" t="s">
+        <v>369</v>
+      </c>
+      <c r="B419" s="34" t="s">
+        <v>370</v>
+      </c>
+      <c r="C419" s="34" t="e" vm="19">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="420" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A420" s="33" t="s">
+        <v>371</v>
+      </c>
+      <c r="B420" s="34" t="s">
+        <v>370</v>
+      </c>
+      <c r="C420" s="34" t="e" vm="20">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="421" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A421" s="33" t="s">
+        <v>372</v>
+      </c>
+      <c r="B421" s="34" t="e" vm="21">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C421" s="34" t="e" vm="22">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="422" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A422" s="33" t="s">
+        <v>373</v>
+      </c>
+      <c r="B422" s="34" t="e" vm="23">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C422" s="34" t="e" vm="24">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="423" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A423" s="33" t="s">
+        <v>374</v>
+      </c>
+      <c r="B423" s="34" t="e" vm="25">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C423" s="34" t="e" vm="26">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="424" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A424" s="33" t="s">
+        <v>375</v>
+      </c>
+      <c r="B424" s="34" t="e" vm="27">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C424" s="34" t="e" vm="28">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="425" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A425" s="33" t="s">
+        <v>376</v>
+      </c>
+      <c r="B425" s="34" t="e" vm="29">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C425" s="34" t="e" vm="30">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="426" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A426" s="33" t="s">
+        <v>377</v>
+      </c>
+      <c r="B426" s="34" t="e" vm="31">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C426" s="34" t="e" vm="32">
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -5566,6 +7841,7 @@
     <mergeCell ref="C244:C245"/>
     <mergeCell ref="C290:C291"/>
   </mergeCells>
+  <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
xong thuyết minh chọn động cơ
</commit_message>
<xml_diff>
--- a/tínhtoans.xlsx
+++ b/tínhtoans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Đồ án tkm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F02D2B6D-C6BD-4219-A7B9-60D00225043B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473EB28C-4F73-476A-969F-CE33387BEBCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{75337E03-C337-4BFE-A279-78895F300CE2}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{75337E03-C337-4BFE-A279-78895F300CE2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,340 +38,8 @@
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="32">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="1"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="2"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="3"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="4"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="5"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="6"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="7"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="8"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="9"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="10"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="11"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="12"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="13"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="14"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="15"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="16"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="17"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="18"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="19"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="20"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="21"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="22"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="23"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="24"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="25"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="26"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="27"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="28"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="29"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="30"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="31"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <valueMetadata count="32">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-    <bk>
-      <rc t="1" v="1"/>
-    </bk>
-    <bk>
-      <rc t="1" v="2"/>
-    </bk>
-    <bk>
-      <rc t="1" v="3"/>
-    </bk>
-    <bk>
-      <rc t="1" v="4"/>
-    </bk>
-    <bk>
-      <rc t="1" v="5"/>
-    </bk>
-    <bk>
-      <rc t="1" v="6"/>
-    </bk>
-    <bk>
-      <rc t="1" v="7"/>
-    </bk>
-    <bk>
-      <rc t="1" v="8"/>
-    </bk>
-    <bk>
-      <rc t="1" v="9"/>
-    </bk>
-    <bk>
-      <rc t="1" v="10"/>
-    </bk>
-    <bk>
-      <rc t="1" v="11"/>
-    </bk>
-    <bk>
-      <rc t="1" v="12"/>
-    </bk>
-    <bk>
-      <rc t="1" v="13"/>
-    </bk>
-    <bk>
-      <rc t="1" v="14"/>
-    </bk>
-    <bk>
-      <rc t="1" v="15"/>
-    </bk>
-    <bk>
-      <rc t="1" v="16"/>
-    </bk>
-    <bk>
-      <rc t="1" v="17"/>
-    </bk>
-    <bk>
-      <rc t="1" v="18"/>
-    </bk>
-    <bk>
-      <rc t="1" v="19"/>
-    </bk>
-    <bk>
-      <rc t="1" v="20"/>
-    </bk>
-    <bk>
-      <rc t="1" v="21"/>
-    </bk>
-    <bk>
-      <rc t="1" v="22"/>
-    </bk>
-    <bk>
-      <rc t="1" v="23"/>
-    </bk>
-    <bk>
-      <rc t="1" v="24"/>
-    </bk>
-    <bk>
-      <rc t="1" v="25"/>
-    </bk>
-    <bk>
-      <rc t="1" v="26"/>
-    </bk>
-    <bk>
-      <rc t="1" v="27"/>
-    </bk>
-    <bk>
-      <rc t="1" v="28"/>
-    </bk>
-    <bk>
-      <rc t="1" v="29"/>
-    </bk>
-    <bk>
-      <rc t="1" v="30"/>
-    </bk>
-    <bk>
-      <rc t="1" v="31"/>
-    </bk>
-  </valueMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="354">
   <si>
     <t>Bánh răng trụ răng thẳng</t>
   </si>
@@ -1226,9 +894,6 @@
   </si>
   <si>
     <t>bảng 5.2 tr78</t>
-  </si>
-  <si>
-    <t>Tra bảng 5.5 tr82 với n01 = 1200 và P_t &lt;= [P], có</t>
   </si>
   <si>
     <t>Đường kính chia</t>
@@ -1457,76 +1122,7 @@
     <t>3.3.7. Bảng thông số thiết kế cặp bánh răng</t>
   </si>
   <si>
-    <t>Ký hiệu (đơn vị)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Số răng bánh chủ động </t>
-  </si>
-  <si>
-    <t>Số răng bánh bị động</t>
-  </si>
-  <si>
-    <t>Môđun</t>
-  </si>
-  <si>
-    <t>Chiều rộng vành răng chủ động</t>
-  </si>
-  <si>
-    <t>Chiều rộng vành răng bị động</t>
-  </si>
-  <si>
-    <t>Tỷ số truyền thực</t>
-  </si>
-  <si>
-    <t>3,71</t>
-  </si>
-  <si>
-    <t>Cấp chính xác</t>
-  </si>
-  <si>
-    <t>Vật liệu làm bánh răng</t>
-  </si>
-  <si>
-    <t>C45</t>
-  </si>
-  <si>
-    <t>Độ cứng  bề mặt bánh răng chủ động</t>
-  </si>
-  <si>
-    <t>Độ cứng bề mặt bánh răng bị động</t>
-  </si>
-  <si>
-    <t>Đường kính vòng lăn bánh răng chủ động</t>
-  </si>
-  <si>
-    <t>Đường kính vòng lăn bánh răng bị động</t>
-  </si>
-  <si>
-    <t>Đường kính vòng đỉnh bánh răng chủ động</t>
-  </si>
-  <si>
-    <t>(mm)</t>
-  </si>
-  <si>
-    <t>Đường kính vòng đỉnh bánh răng bị động</t>
-  </si>
-  <si>
-    <t>Đường kính vòng đáy răng bánh chủ động</t>
-  </si>
-  <si>
-    <t>Đường kính vòng đáy răng bánh bị động</t>
-  </si>
-  <si>
-    <t>Đường kính vòng cơ sở bánh răng chủ động</t>
-  </si>
-  <si>
-    <t>Đường kính vòng cơ sở bánh răng bị động</t>
-  </si>
-  <si>
-    <t>Góc áp lực</t>
-  </si>
-  <si>
-    <t>Vận tốc vòng của bánh răng</t>
+    <t>Tra bảng 5.5 tr82 với n01 = 200 và P_t &lt;= [P], có</t>
   </si>
 </sst>
 </file>
@@ -1653,7 +1249,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1704,36 +1300,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1785,23 +1357,20 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3401,15 +2970,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1706880</xdr:colOff>
-      <xdr:row>298</xdr:row>
-      <xdr:rowOff>99060</xdr:rowOff>
+      <xdr:colOff>868680</xdr:colOff>
+      <xdr:row>297</xdr:row>
+      <xdr:rowOff>72390</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>1050216</xdr:colOff>
-      <xdr:row>337</xdr:row>
-      <xdr:rowOff>15826</xdr:rowOff>
+      <xdr:colOff>212016</xdr:colOff>
+      <xdr:row>336</xdr:row>
+      <xdr:rowOff>586</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3432,8 +3001,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8412480" y="52806600"/>
-          <a:ext cx="6477561" cy="6759526"/>
+          <a:off x="9450705" y="51516915"/>
+          <a:ext cx="6464226" cy="6610936"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4115,368 +3684,7 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>418</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>243840</xdr:colOff>
-      <xdr:row>418</xdr:row>
-      <xdr:rowOff>205740</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="41" name="Picture 40">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8257366D-1879-10E3-F2CC-C81BFEBAA2E1}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId35">
-          <a:clrChange>
-            <a:clrFrom>
-              <a:srgbClr val="FFFFFF"/>
-            </a:clrFrom>
-            <a:clrTo>
-              <a:srgbClr val="FFFFFF">
-                <a:alpha val="0"/>
-              </a:srgbClr>
-            </a:clrTo>
-          </a:clrChange>
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="6134100" y="74447400"/>
-          <a:ext cx="243840" cy="205740"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>419</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>243840</xdr:colOff>
-      <xdr:row>419</xdr:row>
-      <xdr:rowOff>205740</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="42" name="Picture 41">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DDA959F7-0575-FDB6-E473-18F860F695C7}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId36">
-          <a:clrChange>
-            <a:clrFrom>
-              <a:srgbClr val="FFFFFF"/>
-            </a:clrFrom>
-            <a:clrTo>
-              <a:srgbClr val="FFFFFF">
-                <a:alpha val="0"/>
-              </a:srgbClr>
-            </a:clrTo>
-          </a:clrChange>
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="6134100" y="74668380"/>
-          <a:ext cx="243840" cy="205740"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
-</file>
-
-<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="32">
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>1</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>2</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>3</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>4</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>5</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>6</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>7</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>8</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>9</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>10</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>11</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>12</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>13</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>14</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>15</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>16</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>17</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>18</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>19</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>20</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>21</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>22</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>23</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>24</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>25</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>26</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>27</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>28</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>29</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>30</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>31</v>
-    <v>5</v>
-  </rv>
-</rvData>
-</file>
-
-<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <s t="_localImage">
-    <k n="_rvRel:LocalImageIdentifier" t="i"/>
-    <k n="CalcOrigin" t="i"/>
-  </s>
-</rvStructures>
-</file>
-
-<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
-<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <rel r:id="rId1"/>
-  <rel r:id="rId2"/>
-  <rel r:id="rId3"/>
-  <rel r:id="rId4"/>
-  <rel r:id="rId5"/>
-  <rel r:id="rId6"/>
-  <rel r:id="rId7"/>
-  <rel r:id="rId8"/>
-  <rel r:id="rId9"/>
-  <rel r:id="rId10"/>
-  <rel r:id="rId11"/>
-  <rel r:id="rId12"/>
-  <rel r:id="rId13"/>
-  <rel r:id="rId14"/>
-  <rel r:id="rId15"/>
-  <rel r:id="rId16"/>
-  <rel r:id="rId17"/>
-  <rel r:id="rId18"/>
-  <rel r:id="rId19"/>
-  <rel r:id="rId20"/>
-  <rel r:id="rId21"/>
-  <rel r:id="rId22"/>
-  <rel r:id="rId23"/>
-  <rel r:id="rId24"/>
-  <rel r:id="rId25"/>
-  <rel r:id="rId26"/>
-  <rel r:id="rId27"/>
-  <rel r:id="rId28"/>
-  <rel r:id="rId29"/>
-  <rel r:id="rId30"/>
-  <rel r:id="rId31"/>
-  <rel r:id="rId32"/>
-</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5523,7 +4731,7 @@
       <c r="B90" s="6">
         <v>1.25</v>
       </c>
-      <c r="F90" s="27" t="s">
+      <c r="F90" s="30" t="s">
         <v>118</v>
       </c>
     </row>
@@ -5531,7 +4739,7 @@
       <c r="A91" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="F91" s="27"/>
+      <c r="F91" s="30"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
@@ -5543,13 +4751,13 @@
       <c r="C92" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="F92" s="27"/>
+      <c r="F92" s="30"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="F93" s="27"/>
+      <c r="F93" s="30"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
@@ -5561,13 +4769,13 @@
       <c r="C94" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="F94" s="27"/>
+      <c r="F94" s="30"/>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="F95" s="27"/>
+      <c r="F95" s="30"/>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
@@ -5579,13 +4787,13 @@
       <c r="C96" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="F96" s="27"/>
+      <c r="F96" s="30"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="F97" s="27"/>
+      <c r="F97" s="30"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
@@ -5597,13 +4805,13 @@
       <c r="C98" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="F98" s="27"/>
+      <c r="F98" s="30"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="F99" s="27"/>
+      <c r="F99" s="30"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
@@ -5615,7 +4823,7 @@
       <c r="C100" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="F100" s="27"/>
+      <c r="F100" s="30"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="12" t="s">
@@ -5647,7 +4855,7 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>285</v>
+        <v>353</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
@@ -5660,7 +4868,7 @@
         <v>120</v>
       </c>
       <c r="B108" s="6">
-        <v>15.875</v>
+        <v>25.4</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
@@ -5673,7 +4881,7 @@
         <v>122</v>
       </c>
       <c r="B110" s="6">
-        <v>5.08</v>
+        <v>7.95</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -5686,7 +4894,7 @@
         <v>124</v>
       </c>
       <c r="B112" s="6">
-        <v>13.28</v>
+        <v>22.61</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
@@ -5699,7 +4907,7 @@
         <v>126</v>
       </c>
       <c r="B114" s="6">
-        <v>10.8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
@@ -5728,7 +4936,7 @@
       </c>
       <c r="B120" s="6">
         <f>40*B108</f>
-        <v>635</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
@@ -5764,7 +4972,7 @@
       </c>
       <c r="B125" s="6">
         <f>B123*B108</f>
-        <v>2063.75</v>
+        <v>3302</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
@@ -5778,7 +4986,7 @@
       </c>
       <c r="B127" s="6">
         <f>ROUND(0.25*B108*(B123-0.5*(C75+C74)+SQRT((B123-0.5*(C74+C75))^2-2*((C75-C74)/3.14)^2)),2)</f>
-        <v>638.36</v>
+        <v>1021.38</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.25">
@@ -5792,11 +5000,11 @@
       </c>
       <c r="B129" s="6">
         <f>0.002*B127</f>
-        <v>1.2767200000000001</v>
+        <v>2.0427599999999999</v>
       </c>
       <c r="C129" s="6">
         <f>0.004*B127</f>
-        <v>2.5534400000000002</v>
+        <v>4.0855199999999998</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
@@ -5804,7 +5012,7 @@
         <v>141</v>
       </c>
       <c r="B130" s="6">
-        <v>2.36</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
@@ -5818,7 +5026,7 @@
       </c>
       <c r="B133" s="6">
         <f>B127-B130</f>
-        <v>636</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
@@ -5869,7 +5077,7 @@
       </c>
       <c r="B143" s="6">
         <f>ROUND(C74*B108*D66/60000,2)</f>
-        <v>1.57</v>
+        <v>2.5099999999999998</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
@@ -5906,7 +5114,7 @@
       </c>
       <c r="B146" s="6">
         <f>ROUND(1000*D65/B143,2)</f>
-        <v>2656.05</v>
+        <v>1661.35</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.25">
@@ -5915,7 +5123,7 @@
       </c>
       <c r="B147" s="6">
         <f>ROUND(F145*B143^2,2)</f>
-        <v>6.41</v>
+        <v>16.38</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.25">
@@ -5924,7 +5132,7 @@
       </c>
       <c r="B148" s="6">
         <f>ROUND(9.81*D148*F145*B133/1000,2)</f>
-        <v>32.44</v>
+        <v>51.98</v>
       </c>
       <c r="C148" s="6" t="s">
         <v>161</v>
@@ -5947,7 +5155,7 @@
       </c>
       <c r="B151" s="6">
         <f>ROUND(B144*10^3/(B145*B146+B148+B147),2)</f>
-        <v>17.579999999999998</v>
+        <v>27.5</v>
       </c>
       <c r="C151" s="6" t="s">
         <v>162</v>
@@ -5969,7 +5177,7 @@
       </c>
       <c r="B155" s="6">
         <f>ROUND(B108/SIN(3.14/C74),2)</f>
-        <v>116.64</v>
+        <v>186.63</v>
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.25">
@@ -5978,7 +5186,7 @@
       </c>
       <c r="B156" s="6">
         <f>ROUND(B108/SIN(3.14/C75),2)</f>
-        <v>369.18</v>
+        <v>590.69000000000005</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.25">
@@ -5992,7 +5200,7 @@
       </c>
       <c r="B158" s="6">
         <f>ROUND(B108*(0.5+_xlfn.COT(3.14/C74)),2)</f>
-        <v>123.5</v>
+        <v>197.59</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.25">
@@ -6001,7 +5209,7 @@
       </c>
       <c r="B159" s="6">
         <f>ROUND(B108*(0.5+_xlfn.COT(3.14/C75)),2)</f>
-        <v>376.78</v>
+        <v>602.85</v>
       </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.25">
@@ -6038,7 +5246,7 @@
       </c>
       <c r="B163" s="6">
         <f>B155-2*B161</f>
-        <v>106.32</v>
+        <v>176.31</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
@@ -6047,7 +5255,7 @@
       </c>
       <c r="B164" s="6">
         <f>B156-2*B161</f>
-        <v>358.86</v>
+        <v>580.37</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
@@ -6061,7 +5269,7 @@
       </c>
       <c r="B166" s="6">
         <f>ROUND(13*10^-7*D66*B108^3*1,2)</f>
-        <v>1.34</v>
+        <v>5.49</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
@@ -6108,7 +5316,7 @@
       <c r="A170"/>
       <c r="B170" s="6">
         <f>ROUND(0.47*SQRT(C168*(B146*B168+B166)*D168/(E168*A168)),2)</f>
-        <v>573.35</v>
+        <v>454.09</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.25">
@@ -6176,7 +5384,7 @@
       </c>
       <c r="B180" s="6">
         <f>ROUND(B178*B146,2)</f>
-        <v>2788.85</v>
+        <v>1744.42</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
@@ -6220,7 +5428,7 @@
       <c r="B187"/>
       <c r="C187">
         <f>B108</f>
-        <v>15.875</v>
+        <v>25.4</v>
       </c>
     </row>
     <row r="188" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -6240,7 +5448,7 @@
       <c r="B189"/>
       <c r="C189">
         <f>B125</f>
-        <v>2063.75</v>
+        <v>3302</v>
       </c>
     </row>
     <row r="190" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -6250,7 +5458,7 @@
       <c r="B190"/>
       <c r="C190">
         <f>B133</f>
-        <v>636</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="191" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -6280,7 +5488,7 @@
       <c r="B193"/>
       <c r="C193">
         <f>B155</f>
-        <v>116.64</v>
+        <v>186.63</v>
       </c>
     </row>
     <row r="194" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -6290,7 +5498,7 @@
       <c r="B194"/>
       <c r="C194">
         <f>B156</f>
-        <v>369.18</v>
+        <v>590.69000000000005</v>
       </c>
     </row>
     <row r="195" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -6300,7 +5508,7 @@
       <c r="B195"/>
       <c r="C195">
         <f>B158</f>
-        <v>123.5</v>
+        <v>197.59</v>
       </c>
     </row>
     <row r="196" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -6310,7 +5518,7 @@
       <c r="B196"/>
       <c r="C196">
         <f>B159</f>
-        <v>376.78</v>
+        <v>602.85</v>
       </c>
     </row>
     <row r="197" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -6330,7 +5538,7 @@
       <c r="B198"/>
       <c r="C198">
         <f>B163</f>
-        <v>106.32</v>
+        <v>176.31</v>
       </c>
     </row>
     <row r="199" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -6340,7 +5548,7 @@
       <c r="B199"/>
       <c r="C199">
         <f>B164</f>
-        <v>358.86</v>
+        <v>580.37</v>
       </c>
     </row>
     <row r="200" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -6350,7 +5558,7 @@
       <c r="B200"/>
       <c r="C200">
         <f>B170</f>
-        <v>573.35</v>
+        <v>454.09</v>
       </c>
     </row>
     <row r="201" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -6389,7 +5597,7 @@
       <c r="B204"/>
       <c r="C204">
         <f>B180</f>
-        <v>2788.85</v>
+        <v>1744.42</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
@@ -6528,13 +5736,13 @@
       <c r="A227" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="C227" s="27" t="s">
+      <c r="C227" s="30" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228"/>
-      <c r="C228" s="27"/>
+      <c r="C228" s="30"/>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
@@ -6544,7 +5752,7 @@
         <f>2*B225+70</f>
         <v>570</v>
       </c>
-      <c r="C229" s="27"/>
+      <c r="C229" s="30"/>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
@@ -6554,17 +5762,17 @@
         <f>2*B226+70</f>
         <v>510</v>
       </c>
-      <c r="C230" s="27"/>
+      <c r="C230" s="30"/>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" s="11" t="s">
         <v>256</v>
       </c>
-      <c r="C231" s="27"/>
+      <c r="C231" s="30"/>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232"/>
-      <c r="C232" s="27"/>
+      <c r="C232" s="30"/>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
@@ -6574,7 +5782,7 @@
         <f>1.8*B225</f>
         <v>450</v>
       </c>
-      <c r="C233" s="27"/>
+      <c r="C233" s="30"/>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
@@ -6584,16 +5792,16 @@
         <f>1.8*B226</f>
         <v>396</v>
       </c>
-      <c r="C234" s="27"/>
+      <c r="C234" s="30"/>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C235" s="27"/>
+      <c r="C235" s="30"/>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="C236" s="27"/>
+      <c r="C236" s="30"/>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
@@ -6602,7 +5810,7 @@
       <c r="B237" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C237" s="27"/>
+      <c r="C237" s="30"/>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
@@ -6611,7 +5819,7 @@
       <c r="B238" s="6">
         <v>1.75</v>
       </c>
-      <c r="C238" s="27"/>
+      <c r="C238" s="30"/>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" s="12" t="s">
@@ -6642,7 +5850,7 @@
       <c r="B244" s="6">
         <v>6</v>
       </c>
-      <c r="C244" s="27" t="s">
+      <c r="C244" s="30" t="s">
         <v>244</v>
       </c>
     </row>
@@ -6653,7 +5861,7 @@
       <c r="B245" s="6">
         <v>6</v>
       </c>
-      <c r="C245" s="27"/>
+      <c r="C245" s="30"/>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" s="12" t="s">
@@ -6915,7 +6123,7 @@
         <f>0.01*B286</f>
         <v>1.4195</v>
       </c>
-      <c r="C290" s="27">
+      <c r="C290" s="30">
         <v>2</v>
       </c>
     </row>
@@ -6924,7 +6132,7 @@
         <f>0.02*B286</f>
         <v>2.839</v>
       </c>
-      <c r="C291" s="27"/>
+      <c r="C291" s="30"/>
       <c r="D291" s="6" t="s">
         <v>267</v>
       </c>
@@ -7028,10 +6236,10 @@
       </c>
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B306" s="6">
+      <c r="B306" s="31">
         <v>0</v>
       </c>
-      <c r="C306" s="6">
+      <c r="C306" s="31">
         <v>0</v>
       </c>
     </row>
@@ -7070,12 +6278,12 @@
     </row>
     <row r="312" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A312" s="11" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="313" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B313" s="6">
         <f>C290*C295/COS(B294)</f>
@@ -7084,7 +6292,7 @@
     </row>
     <row r="314" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A314" s="26" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B314" s="6">
         <f>C290*C296/COS(B294)</f>
@@ -7093,12 +6301,12 @@
     </row>
     <row r="315" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A315" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="316" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A316" s="6" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B316" s="6">
         <f>ROUND(2*B311/(B300+1),2)</f>
@@ -7107,7 +6315,7 @@
     </row>
     <row r="317" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A317" s="6" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B317" s="6">
         <f>ROUND(B316*B300,2)</f>
@@ -7116,7 +6324,7 @@
     </row>
     <row r="318" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A318" s="12" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="319" spans="1:3" x14ac:dyDescent="0.25">
@@ -7139,7 +6347,7 @@
     </row>
     <row r="321" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A321" s="12" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="322" spans="1:2" x14ac:dyDescent="0.25">
@@ -7162,12 +6370,12 @@
     </row>
     <row r="324" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A324" s="12" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="325" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B325" s="6">
         <f>ROUND(B313*COS(B328),2)</f>
@@ -7176,7 +6384,7 @@
     </row>
     <row r="326" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B326" s="6">
         <f>ROUND(B314*COS(B328),2)</f>
@@ -7185,12 +6393,12 @@
     </row>
     <row r="327" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A327" s="12" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="328" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B328" s="6">
         <v>20</v>
@@ -7198,12 +6406,12 @@
     </row>
     <row r="329" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A329" s="12" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="330" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B330" s="6">
         <f>DEGREES(ATAN(TAN(RADIANS(B328))/COS(RADIANS(B294))))</f>
@@ -7212,12 +6420,12 @@
     </row>
     <row r="331" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A331" s="12" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="332" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B332">
         <f>DEGREES(ACOS(B309*COS(RADIANS(B330))/B311))</f>
@@ -7226,17 +6434,17 @@
     </row>
     <row r="335" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A335" s="4" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="339" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A339" s="11" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="340" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A340" s="6" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B340" s="6">
         <f>B281*B311</f>
@@ -7245,12 +6453,12 @@
     </row>
     <row r="342" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A342" s="11" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="343" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A343" s="6" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B343" s="6">
         <v>274</v>
@@ -7258,12 +6466,12 @@
     </row>
     <row r="344" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A344" s="11" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="345" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A345" s="6" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B345" s="6">
         <f>ROUND(SQRT(2*COS(0)/SIN(RADIANS(2*B332))),2)</f>
@@ -7271,13 +6479,13 @@
       </c>
     </row>
     <row r="346" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A346" s="29" t="s">
-        <v>309</v>
+      <c r="A346" s="12" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="347" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A347" s="28" t="s">
-        <v>326</v>
+      <c r="A347" t="s">
+        <v>325</v>
       </c>
       <c r="B347" s="6">
         <f>ROUND((1.88-3.2*(1/C295+1/C296))*COS(B306),2)</f>
@@ -7285,13 +6493,13 @@
       </c>
     </row>
     <row r="348" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A348" s="29" t="s">
+      <c r="A348" s="12" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A349" t="s">
         <v>327</v>
-      </c>
-    </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A349" s="28" t="s">
-        <v>328</v>
       </c>
       <c r="B349" s="6">
         <f>B340*SIN(B306)/(C290*PI())</f>
@@ -7299,13 +6507,13 @@
       </c>
     </row>
     <row r="350" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A350" s="29" t="s">
-        <v>310</v>
+      <c r="A350" s="12" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="351" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A351" s="28" t="s">
-        <v>307</v>
+      <c r="A351" t="s">
+        <v>306</v>
       </c>
       <c r="B351" s="6">
         <f>ROUND(SQRT((4-B347)/3),2)</f>
@@ -7313,22 +6521,22 @@
       </c>
     </row>
     <row r="352" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A352" s="29" t="s">
+      <c r="A352" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="C352" s="22" t="s">
+        <v>312</v>
+      </c>
+      <c r="D352" s="22" t="s">
+        <v>313</v>
+      </c>
+      <c r="E352" s="22" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="353" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A353" t="s">
         <v>311</v>
-      </c>
-      <c r="C352" s="22" t="s">
-        <v>313</v>
-      </c>
-      <c r="D352" s="22" t="s">
-        <v>314</v>
-      </c>
-      <c r="E352" s="22" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="353" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A353" s="28" t="s">
-        <v>312</v>
       </c>
       <c r="B353" s="6">
         <f>ROUND(C353*D353*F356,2)</f>
@@ -7345,33 +6553,33 @@
         <v>3.18</v>
       </c>
       <c r="F353" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="G353" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="G353" s="6" t="s">
-        <v>317</v>
-      </c>
     </row>
     <row r="354" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A354" s="28"/>
+      <c r="A354"/>
       <c r="C354" s="22" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="355" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A355" s="29" t="s">
-        <v>321</v>
+      <c r="A355" s="12" t="s">
+        <v>320</v>
       </c>
       <c r="C355" s="6">
         <v>1.05</v>
       </c>
       <c r="E355" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="F355" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="F355" s="6" t="s">
+      <c r="G355" s="6" t="s">
         <v>319</v>
-      </c>
-      <c r="G355" s="6" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="356" spans="1:7" x14ac:dyDescent="0.25">
@@ -7394,22 +6602,22 @@
     </row>
     <row r="357" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B357" s="6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="363" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A363" s="4" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="365" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A365" s="11" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="366" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A366" t="s">
         <v>329</v>
-      </c>
-    </row>
-    <row r="366" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A366" s="28" t="s">
-        <v>330</v>
       </c>
       <c r="B366" s="6">
         <f>ROUND(1/B347,3)</f>
@@ -7417,34 +6625,34 @@
       </c>
     </row>
     <row r="367" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A367" s="29" t="s">
-        <v>331</v>
+      <c r="A367" s="12" t="s">
+        <v>330</v>
       </c>
     </row>
     <row r="368" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A368" s="6" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B368" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="369" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A369" s="29" t="s">
-        <v>335</v>
+      <c r="A369" s="12" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="370" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A370" s="28" t="s">
-        <v>333</v>
+      <c r="A370" t="s">
+        <v>332</v>
       </c>
       <c r="B370" s="6">
         <v>4.04</v>
       </c>
     </row>
     <row r="371" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A371" s="30" t="s">
-        <v>334</v>
+      <c r="A371" s="18" t="s">
+        <v>333</v>
       </c>
       <c r="B371" s="6">
         <v>3.6</v>
@@ -7452,39 +6660,39 @@
     </row>
     <row r="372" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A372" s="11" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="373" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A373" s="6" t="s">
-        <v>339</v>
-      </c>
-      <c r="B373" s="28">
+        <v>338</v>
+      </c>
+      <c r="B373">
         <v>1</v>
       </c>
     </row>
     <row r="374" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A374" s="11" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="375" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A375" s="6" t="s">
-        <v>337</v>
-      </c>
-      <c r="B375" s="28">
+        <v>336</v>
+      </c>
+      <c r="B375">
         <f>G356</f>
         <v>1.3062</v>
       </c>
     </row>
     <row r="376" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A376" s="11" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="377" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A377" s="28" t="s">
-        <v>341</v>
+      <c r="A377" t="s">
+        <v>340</v>
       </c>
       <c r="B377" s="6">
         <f>C355*B373*B375</f>
@@ -7492,8 +6700,8 @@
       </c>
     </row>
     <row r="378" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A378" s="29" t="s">
-        <v>343</v>
+      <c r="A378" s="12" t="s">
+        <v>342</v>
       </c>
     </row>
     <row r="379" spans="1:2" x14ac:dyDescent="0.25">
@@ -7504,8 +6712,8 @@
       </c>
     </row>
     <row r="380" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A380" s="29" t="s">
-        <v>344</v>
+      <c r="A380" s="12" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="381" spans="1:2" x14ac:dyDescent="0.25">
@@ -7517,28 +6725,28 @@
     </row>
     <row r="383" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A383" s="6" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="385" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A385" s="4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="391" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A391" s="11" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="392" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A392" s="6" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B392" s="6">
         <v>2</v>
       </c>
       <c r="C392" s="6" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="394" spans="1:3" x14ac:dyDescent="0.25">
@@ -7548,7 +6756,7 @@
         <v>619.67999999999995</v>
       </c>
       <c r="C394" s="6" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="398" spans="1:3" x14ac:dyDescent="0.25">
@@ -7558,7 +6766,7 @@
         <v>106.74</v>
       </c>
       <c r="C398" s="6" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="399" spans="1:3" x14ac:dyDescent="0.25">
@@ -7568,271 +6776,128 @@
         <v>95.12</v>
       </c>
       <c r="C399" s="6" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="402" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A402" s="4" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="403" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="404" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A404" s="31" t="s">
-        <v>200</v>
-      </c>
-      <c r="B404" s="32" t="s">
-        <v>354</v>
-      </c>
-      <c r="C404" s="32" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="405" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A405" s="33" t="s">
-        <v>132</v>
-      </c>
-      <c r="B405" s="34" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C405" s="34">
-        <f>B298</f>
-        <v>139</v>
-      </c>
-    </row>
-    <row r="406" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A406" s="33" t="s">
-        <v>355</v>
-      </c>
-      <c r="B406" s="34" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C406" s="34">
-        <f>C295</f>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="407" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A407" s="33" t="s">
-        <v>356</v>
-      </c>
-      <c r="B407" s="34" t="e" vm="3">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C407" s="34">
-        <f>C296</f>
-        <v>118</v>
-      </c>
-    </row>
-    <row r="408" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A408" s="33" t="s">
-        <v>357</v>
-      </c>
-      <c r="B408" s="34" t="e" vm="4">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C408" s="34">
-        <f>C290</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="409" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A409" s="33" t="s">
-        <v>301</v>
-      </c>
-      <c r="B409" s="34" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C409" s="34">
-        <f>B332</f>
-        <v>19.999999999999989</v>
-      </c>
-    </row>
-    <row r="410" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A410" s="33" t="s">
-        <v>358</v>
-      </c>
-      <c r="B410" s="34" t="e" vm="6">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C410" s="34">
-        <f>C295</f>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="411" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A411" s="33" t="s">
-        <v>359</v>
-      </c>
-      <c r="B411" s="34" t="e" vm="7">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C411" s="34" t="e" vm="8">
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="412" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A412" s="33" t="s">
-        <v>360</v>
-      </c>
-      <c r="B412" s="34" t="e" vm="9">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C412" s="34" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="413" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A413" s="33" t="s">
-        <v>362</v>
-      </c>
-      <c r="B413" s="34"/>
-      <c r="C413" s="34" t="e" vm="10">
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="414" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A414" s="33" t="s">
-        <v>363</v>
-      </c>
-      <c r="B414" s="34" t="s">
-        <v>364</v>
-      </c>
-      <c r="C414" s="34" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="415" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A415" s="33" t="s">
-        <v>365</v>
-      </c>
-      <c r="B415" s="34" t="e" vm="11">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C415" s="34" t="e" vm="12">
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="416" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A416" s="33" t="s">
-        <v>366</v>
-      </c>
-      <c r="B416" s="34" t="e" vm="13">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C416" s="34" t="e" vm="14">
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="417" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A417" s="33" t="s">
-        <v>367</v>
-      </c>
-      <c r="B417" s="34" t="e" vm="15">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C417" s="34" t="e" vm="16">
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="418" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A418" s="33" t="s">
-        <v>368</v>
-      </c>
-      <c r="B418" s="34" t="e" vm="17">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C418" s="34" t="e" vm="18">
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="419" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A419" s="33" t="s">
-        <v>369</v>
-      </c>
-      <c r="B419" s="34" t="s">
-        <v>370</v>
-      </c>
-      <c r="C419" s="34" t="e" vm="19">
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="420" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A420" s="33" t="s">
-        <v>371</v>
-      </c>
-      <c r="B420" s="34" t="s">
-        <v>370</v>
-      </c>
-      <c r="C420" s="34" t="e" vm="20">
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="421" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A421" s="33" t="s">
-        <v>372</v>
-      </c>
-      <c r="B421" s="34" t="e" vm="21">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C421" s="34" t="e" vm="22">
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="422" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A422" s="33" t="s">
-        <v>373</v>
-      </c>
-      <c r="B422" s="34" t="e" vm="23">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C422" s="34" t="e" vm="24">
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="423" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A423" s="33" t="s">
-        <v>374</v>
-      </c>
-      <c r="B423" s="34" t="e" vm="25">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C423" s="34" t="e" vm="26">
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="424" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A424" s="33" t="s">
-        <v>375</v>
-      </c>
-      <c r="B424" s="34" t="e" vm="27">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C424" s="34" t="e" vm="28">
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="425" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A425" s="33" t="s">
-        <v>376</v>
-      </c>
-      <c r="B425" s="34" t="e" vm="29">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C425" s="34" t="e" vm="30">
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="426" spans="1:3" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A426" s="33" t="s">
-        <v>377</v>
-      </c>
-      <c r="B426" s="34" t="e" vm="31">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C426" s="34" t="e" vm="32">
-        <v>#VALUE!</v>
-      </c>
+        <v>352</v>
+      </c>
+    </row>
+    <row r="404" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A404" s="27"/>
+      <c r="B404" s="28"/>
+      <c r="C404" s="28"/>
+    </row>
+    <row r="405" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A405" s="27"/>
+      <c r="B405" s="29"/>
+      <c r="C405" s="29"/>
+    </row>
+    <row r="406" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A406" s="27"/>
+      <c r="B406" s="29"/>
+      <c r="C406" s="29"/>
+    </row>
+    <row r="407" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A407" s="27"/>
+      <c r="B407" s="29"/>
+      <c r="C407" s="29"/>
+    </row>
+    <row r="408" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A408" s="27"/>
+      <c r="B408" s="29"/>
+      <c r="C408" s="29"/>
+    </row>
+    <row r="409" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A409" s="27"/>
+      <c r="B409" s="29"/>
+      <c r="C409" s="29"/>
+    </row>
+    <row r="410" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A410" s="27"/>
+      <c r="B410" s="29"/>
+      <c r="C410" s="29"/>
+    </row>
+    <row r="411" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A411" s="27"/>
+      <c r="B411" s="29"/>
+      <c r="C411" s="29"/>
+    </row>
+    <row r="412" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A412" s="27"/>
+      <c r="B412" s="29"/>
+      <c r="C412" s="29"/>
+    </row>
+    <row r="413" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A413" s="27"/>
+      <c r="B413" s="29"/>
+      <c r="C413" s="29"/>
+    </row>
+    <row r="414" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A414" s="27"/>
+      <c r="B414" s="29"/>
+      <c r="C414" s="29"/>
+    </row>
+    <row r="415" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A415" s="27"/>
+      <c r="B415" s="29"/>
+      <c r="C415" s="29"/>
+    </row>
+    <row r="416" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A416" s="27"/>
+      <c r="B416" s="29"/>
+      <c r="C416" s="29"/>
+    </row>
+    <row r="417" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A417" s="27"/>
+      <c r="B417" s="29"/>
+      <c r="C417" s="29"/>
+    </row>
+    <row r="418" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A418" s="27"/>
+      <c r="B418" s="29"/>
+      <c r="C418" s="29"/>
+    </row>
+    <row r="419" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A419" s="27"/>
+      <c r="B419" s="29"/>
+      <c r="C419" s="29"/>
+    </row>
+    <row r="420" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A420" s="27"/>
+      <c r="B420" s="29"/>
+      <c r="C420" s="29"/>
+    </row>
+    <row r="421" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A421" s="27"/>
+      <c r="B421" s="29"/>
+      <c r="C421" s="29"/>
+    </row>
+    <row r="422" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A422" s="27"/>
+      <c r="B422" s="29"/>
+      <c r="C422" s="29"/>
+    </row>
+    <row r="423" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A423" s="27"/>
+      <c r="B423" s="29"/>
+      <c r="C423" s="29"/>
+    </row>
+    <row r="424" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A424" s="27"/>
+      <c r="B424" s="29"/>
+      <c r="C424" s="29"/>
+    </row>
+    <row r="425" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A425" s="27"/>
+      <c r="B425" s="29"/>
+      <c r="C425" s="29"/>
+    </row>
+    <row r="426" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A426" s="27"/>
+      <c r="B426" s="29"/>
+      <c r="C426" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
hoàn thành thuyết minh tính toán bộ truyền xích
</commit_message>
<xml_diff>
--- a/tínhtoans.xlsx
+++ b/tínhtoans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Đồ án tkm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473EB28C-4F73-476A-969F-CE33387BEBCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1DBD1EA-1F95-49CF-82C0-9BD4563E6E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{75337E03-C337-4BFE-A279-78895F300CE2}"/>
+    <workbookView xWindow="43110" yWindow="0" windowWidth="14595" windowHeight="15585" xr2:uid="{75337E03-C337-4BFE-A279-78895F300CE2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1367,10 +1367,10 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1401,7 +1401,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1126086</xdr:colOff>
+      <xdr:colOff>1122276</xdr:colOff>
       <xdr:row>282</xdr:row>
       <xdr:rowOff>38</xdr:rowOff>
     </xdr:to>
@@ -1658,9 +1658,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1082373</xdr:colOff>
+      <xdr:colOff>1086183</xdr:colOff>
       <xdr:row>223</xdr:row>
-      <xdr:rowOff>95335</xdr:rowOff>
+      <xdr:rowOff>91525</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2188,7 +2188,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>707020</xdr:colOff>
+      <xdr:colOff>703210</xdr:colOff>
       <xdr:row>231</xdr:row>
       <xdr:rowOff>38253</xdr:rowOff>
     </xdr:to>
@@ -2232,9 +2232,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2878637</xdr:colOff>
+      <xdr:colOff>2874827</xdr:colOff>
       <xdr:row>249</xdr:row>
-      <xdr:rowOff>20996</xdr:rowOff>
+      <xdr:rowOff>17186</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2276,9 +2276,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>250025</xdr:colOff>
+      <xdr:colOff>246215</xdr:colOff>
       <xdr:row>255</xdr:row>
-      <xdr:rowOff>91476</xdr:rowOff>
+      <xdr:rowOff>95286</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2675,7 +2675,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>476582</xdr:colOff>
+      <xdr:colOff>472772</xdr:colOff>
       <xdr:row>283</xdr:row>
       <xdr:rowOff>77</xdr:rowOff>
     </xdr:to>
@@ -2932,9 +2932,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>211701</xdr:colOff>
+      <xdr:colOff>207891</xdr:colOff>
       <xdr:row>287</xdr:row>
-      <xdr:rowOff>93398</xdr:rowOff>
+      <xdr:rowOff>97208</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2976,7 +2976,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>212016</xdr:colOff>
+      <xdr:colOff>208206</xdr:colOff>
       <xdr:row>336</xdr:row>
       <xdr:rowOff>586</xdr:rowOff>
     </xdr:to>
@@ -3022,7 +3022,7 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>3962743</xdr:colOff>
       <xdr:row>361</xdr:row>
-      <xdr:rowOff>17206</xdr:rowOff>
+      <xdr:rowOff>21016</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3206,9 +3206,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>817652</xdr:colOff>
+      <xdr:colOff>821462</xdr:colOff>
       <xdr:row>368</xdr:row>
-      <xdr:rowOff>91521</xdr:rowOff>
+      <xdr:rowOff>95331</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3394,7 +3394,7 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>4497705</xdr:colOff>
       <xdr:row>388</xdr:row>
-      <xdr:rowOff>53384</xdr:rowOff>
+      <xdr:rowOff>57194</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3507,9 +3507,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>4968556</xdr:colOff>
+      <xdr:colOff>4972366</xdr:colOff>
       <xdr:row>396</xdr:row>
-      <xdr:rowOff>133390</xdr:rowOff>
+      <xdr:rowOff>129580</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4731,7 +4731,7 @@
       <c r="B90" s="6">
         <v>1.25</v>
       </c>
-      <c r="F90" s="30" t="s">
+      <c r="F90" s="31" t="s">
         <v>118</v>
       </c>
     </row>
@@ -4739,7 +4739,7 @@
       <c r="A91" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="F91" s="30"/>
+      <c r="F91" s="31"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
@@ -4751,13 +4751,13 @@
       <c r="C92" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="F92" s="30"/>
+      <c r="F92" s="31"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="F93" s="30"/>
+      <c r="F93" s="31"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
@@ -4769,13 +4769,13 @@
       <c r="C94" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="F94" s="30"/>
+      <c r="F94" s="31"/>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="F95" s="30"/>
+      <c r="F95" s="31"/>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
@@ -4787,13 +4787,13 @@
       <c r="C96" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="F96" s="30"/>
+      <c r="F96" s="31"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="F97" s="30"/>
+      <c r="F97" s="31"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
@@ -4805,13 +4805,13 @@
       <c r="C98" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="F98" s="30"/>
+      <c r="F98" s="31"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="F99" s="30"/>
+      <c r="F99" s="31"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
@@ -4823,7 +4823,7 @@
       <c r="C100" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="F100" s="30"/>
+      <c r="F100" s="31"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="12" t="s">
@@ -5146,7 +5146,7 @@
         <v>155</v>
       </c>
       <c r="B149" s="6">
-        <v>11.7</v>
+        <v>8.1999999999999993</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.25">
@@ -5220,7 +5220,7 @@
         <v>172</v>
       </c>
       <c r="C160" s="6">
-        <v>10.16</v>
+        <v>15.88</v>
       </c>
       <c r="D160" s="6" t="s">
         <v>284</v>
@@ -5232,7 +5232,7 @@
       </c>
       <c r="B161" s="6">
         <f>ROUND(0.5025*C160+0.05,2)</f>
-        <v>5.16</v>
+        <v>8.0299999999999994</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
@@ -5246,7 +5246,7 @@
       </c>
       <c r="B163" s="6">
         <f>B155-2*B161</f>
-        <v>176.31</v>
+        <v>170.57</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
@@ -5255,7 +5255,7 @@
       </c>
       <c r="B164" s="6">
         <f>B156-2*B161</f>
-        <v>580.37</v>
+        <v>574.63000000000011</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
@@ -5528,7 +5528,7 @@
       <c r="B197"/>
       <c r="C197">
         <f>B161</f>
-        <v>5.16</v>
+        <v>8.0299999999999994</v>
       </c>
     </row>
     <row r="198" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -5538,7 +5538,7 @@
       <c r="B198"/>
       <c r="C198">
         <f>B163</f>
-        <v>176.31</v>
+        <v>170.57</v>
       </c>
     </row>
     <row r="199" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -5548,7 +5548,7 @@
       <c r="B199"/>
       <c r="C199">
         <f>B164</f>
-        <v>580.37</v>
+        <v>574.63000000000011</v>
       </c>
     </row>
     <row r="200" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
@@ -5736,13 +5736,13 @@
       <c r="A227" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="C227" s="30" t="s">
+      <c r="C227" s="31" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228"/>
-      <c r="C228" s="30"/>
+      <c r="C228" s="31"/>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
@@ -5752,7 +5752,7 @@
         <f>2*B225+70</f>
         <v>570</v>
       </c>
-      <c r="C229" s="30"/>
+      <c r="C229" s="31"/>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
@@ -5762,17 +5762,17 @@
         <f>2*B226+70</f>
         <v>510</v>
       </c>
-      <c r="C230" s="30"/>
+      <c r="C230" s="31"/>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" s="11" t="s">
         <v>256</v>
       </c>
-      <c r="C231" s="30"/>
+      <c r="C231" s="31"/>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232"/>
-      <c r="C232" s="30"/>
+      <c r="C232" s="31"/>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
@@ -5782,7 +5782,7 @@
         <f>1.8*B225</f>
         <v>450</v>
       </c>
-      <c r="C233" s="30"/>
+      <c r="C233" s="31"/>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
@@ -5792,16 +5792,16 @@
         <f>1.8*B226</f>
         <v>396</v>
       </c>
-      <c r="C234" s="30"/>
+      <c r="C234" s="31"/>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C235" s="30"/>
+      <c r="C235" s="31"/>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="C236" s="30"/>
+      <c r="C236" s="31"/>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
@@ -5810,7 +5810,7 @@
       <c r="B237" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C237" s="30"/>
+      <c r="C237" s="31"/>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
@@ -5819,7 +5819,7 @@
       <c r="B238" s="6">
         <v>1.75</v>
       </c>
-      <c r="C238" s="30"/>
+      <c r="C238" s="31"/>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" s="12" t="s">
@@ -5850,7 +5850,7 @@
       <c r="B244" s="6">
         <v>6</v>
       </c>
-      <c r="C244" s="30" t="s">
+      <c r="C244" s="31" t="s">
         <v>244</v>
       </c>
     </row>
@@ -5861,7 +5861,7 @@
       <c r="B245" s="6">
         <v>6</v>
       </c>
-      <c r="C245" s="30"/>
+      <c r="C245" s="31"/>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" s="12" t="s">
@@ -6123,7 +6123,7 @@
         <f>0.01*B286</f>
         <v>1.4195</v>
       </c>
-      <c r="C290" s="30">
+      <c r="C290" s="31">
         <v>2</v>
       </c>
     </row>
@@ -6132,7 +6132,7 @@
         <f>0.02*B286</f>
         <v>2.839</v>
       </c>
-      <c r="C291" s="30"/>
+      <c r="C291" s="31"/>
       <c r="D291" s="6" t="s">
         <v>267</v>
       </c>
@@ -6236,10 +6236,10 @@
       </c>
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B306" s="31">
+      <c r="B306" s="30">
         <v>0</v>
       </c>
-      <c r="C306" s="31">
+      <c r="C306" s="30">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
hoàn thành tính toán chọn đường kính trục
</commit_message>
<xml_diff>
--- a/tínhtoans.xlsx
+++ b/tínhtoans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Đồ án tkm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1DBD1EA-1F95-49CF-82C0-9BD4563E6E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0C0F40-5B29-4B5C-8B8D-629F6D72C7CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43110" yWindow="0" windowWidth="14595" windowHeight="15585" xr2:uid="{75337E03-C337-4BFE-A279-78895F300CE2}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{75337E03-C337-4BFE-A279-78895F300CE2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,8 +38,40 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="2">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="2">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+    <bk>
+      <rc t="1" v="1"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="438">
   <si>
     <t>Bánh răng trụ răng thẳng</t>
   </si>
@@ -1124,12 +1156,264 @@
   <si>
     <t>Tra bảng 5.5 tr82 với n01 = 200 và P_t &lt;= [P], có</t>
   </si>
+  <si>
+    <t>CHƯƠNG IV: TÍNH TOÁN THIẾT KẾ TRỤC</t>
+  </si>
+  <si>
+    <t>4.1. Tính chọn khớp nối</t>
+  </si>
+  <si>
+    <t>Momen cần truyền</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>Đường kính trục động cơ</t>
+  </si>
+  <si>
+    <t>d_đc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.1.1. Chọn khớp nối </t>
+  </si>
+  <si>
+    <t>khớp nối trục vòng đàn hồi</t>
+  </si>
+  <si>
+    <t>T_t</t>
+  </si>
+  <si>
+    <t>Hệ số chế độ làm việc - k</t>
+  </si>
+  <si>
+    <t>Đảm bảo sức bền dập của vòng đàn hồi</t>
+  </si>
+  <si>
+    <t>4.1.2. Kiểm nghiệm điều kiện bền của vòng đàn hồi và chốt</t>
+  </si>
+  <si>
+    <t>Điều kiện sức bền của chốt</t>
+  </si>
+  <si>
+    <t>Z</t>
+  </si>
+  <si>
+    <t>D0</t>
+  </si>
+  <si>
+    <t>l3</t>
+  </si>
+  <si>
+    <t>l1</t>
+  </si>
+  <si>
+    <t>l2</t>
+  </si>
+  <si>
+    <t>l0</t>
+  </si>
+  <si>
+    <t>dc</t>
+  </si>
+  <si>
+    <t>thỏa mãn</t>
+  </si>
+  <si>
+    <t>4.2. Thiết kế trục I</t>
+  </si>
+  <si>
+    <t>4.2.1. Chọn vật liệu thiết kế trục</t>
+  </si>
+  <si>
+    <t>Mác thép</t>
+  </si>
+  <si>
+    <t>Độ cứng</t>
+  </si>
+  <si>
+    <t>C45</t>
+  </si>
+  <si>
+    <t>HB 192 .. 240</t>
+  </si>
+  <si>
+    <t>4.2.2. Tải trọng tác dụng lên các trục</t>
+  </si>
+  <si>
+    <t>Lực vòng</t>
+  </si>
+  <si>
+    <t>Ft1 = Ft2</t>
+  </si>
+  <si>
+    <t>Lực hướng tâm</t>
+  </si>
+  <si>
+    <t>Fr1 = Fr2</t>
+  </si>
+  <si>
+    <t>Lực dọc trục</t>
+  </si>
+  <si>
+    <t>Fa1 = Fa2</t>
+  </si>
+  <si>
+    <t>4.2.3. Tính sơ bộ trục</t>
+  </si>
+  <si>
+    <t>Đường kính trục</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>chọn d</t>
+  </si>
+  <si>
+    <t>b0</t>
+  </si>
+  <si>
+    <t>bảng 10.2[2] tr 189</t>
+  </si>
+  <si>
+    <t>Chiều rộng ổ lăn</t>
+  </si>
+  <si>
+    <t>Chiều dài mayo nửa khớp nối</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khoảng cách từ mặt mút của chi tiết quay đến thành trong của hộp hoặc khoảng cách giữa các chi tiết quay </t>
+  </si>
+  <si>
+    <t>k1</t>
+  </si>
+  <si>
+    <t>Khoảng cách từ mặt mút ổ đến thành trong của hộp</t>
+  </si>
+  <si>
+    <t>k2</t>
+  </si>
+  <si>
+    <t>Khoảng cách từ mặt mút của chi tiết quay đến nắp ổ</t>
+  </si>
+  <si>
+    <t>k3</t>
+  </si>
+  <si>
+    <t>Chiều cao nắp ổ và đầu bu lông</t>
+  </si>
+  <si>
+    <t>h_n</t>
+  </si>
+  <si>
+    <t>Khoảng công xôn (khoảng chìa) trên trục thứ 1, tính từ chi tiết thứ 2 ở ngoài hgt đến gối đỡ</t>
+  </si>
+  <si>
+    <t>Chiều dài mayo BR trụ</t>
+  </si>
+  <si>
+    <t>l_m13</t>
+  </si>
+  <si>
+    <t>l_m12 (nối trục vòng đàn hồi)</t>
+  </si>
+  <si>
+    <t>l_c12 = -l12</t>
+  </si>
+  <si>
+    <t>Khoảng cách từ gối đỡ 0 đến tiết diện thứ 3 trên trục thứ 1</t>
+  </si>
+  <si>
+    <t>l13</t>
+  </si>
+  <si>
+    <t>Chiều rộng vành bánh răng thứ 3 trên trục thứ 1</t>
+  </si>
+  <si>
+    <t>b13 = bw1</t>
+  </si>
+  <si>
+    <t>4.2.5. Tính toán lực cho trục I</t>
+  </si>
+  <si>
+    <t>Khoảng cách giữa các gối đỡ 0 và 1 trên trục thứ 1</t>
+  </si>
+  <si>
+    <t>l1l = 2*l13</t>
+  </si>
+  <si>
+    <t>F_t</t>
+  </si>
+  <si>
+    <t>f_kn</t>
+  </si>
+  <si>
+    <t>FxB</t>
+  </si>
+  <si>
+    <t>FyB</t>
+  </si>
+  <si>
+    <t>FxD</t>
+  </si>
+  <si>
+    <t>FyD</t>
+  </si>
+  <si>
+    <t>My</t>
+  </si>
+  <si>
+    <t>Momen uốn lớn nhất</t>
+  </si>
+  <si>
+    <t>Mx</t>
+  </si>
+  <si>
+    <t>4.2.6. Tính momen tương đương</t>
+  </si>
+  <si>
+    <t>Momen tương đương tại khớp nối</t>
+  </si>
+  <si>
+    <t>Mtd1</t>
+  </si>
+  <si>
+    <t>Momen tương đương tại ổ lăn B</t>
+  </si>
+  <si>
+    <t>MtdB</t>
+  </si>
+  <si>
+    <t>Momen tương đương tại BR</t>
+  </si>
+  <si>
+    <t>Mtd BR</t>
+  </si>
+  <si>
+    <t>tại bánh răng chủ động</t>
+  </si>
+  <si>
+    <t>4.2.7. Đường kính các đoạn trục</t>
+  </si>
+  <si>
+    <t>Đường kính trục tại vị trí tiết diện khớp nối</t>
+  </si>
+  <si>
+    <t>Đường kính trục tại vị trí tiết diện ổ lăn B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đường kính trục tại vị trí tiết diện bánh răng </t>
+  </si>
+  <si>
+    <t>d BR</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1228,6 +1512,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1249,7 +1548,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -1300,12 +1599,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1369,9 +1692,34 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3684,7 +4032,793 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>297180</xdr:colOff>
+      <xdr:row>416</xdr:row>
+      <xdr:rowOff>100965</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>55425</xdr:colOff>
+      <xdr:row>419</xdr:row>
+      <xdr:rowOff>131499</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="31" name="Picture 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9099960E-C858-6C4A-8CB5-519EA50D3C2C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId35"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12022455" y="72224265"/>
+          <a:ext cx="2067105" cy="611559"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>420</xdr:row>
+      <xdr:rowOff>49530</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>324039</xdr:colOff>
+      <xdr:row>424</xdr:row>
+      <xdr:rowOff>15303</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="32" name="Picture 31">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{76B1F583-1DC5-8597-7B98-E6C1E1DC3C09}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId36"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12144375" y="72934830"/>
+          <a:ext cx="2190939" cy="731583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>666750</xdr:colOff>
+      <xdr:row>407</xdr:row>
+      <xdr:rowOff>24765</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2629070</xdr:colOff>
+      <xdr:row>409</xdr:row>
+      <xdr:rowOff>186738</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="41" name="Picture 40">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FDD63A37-3CC6-6588-2B7A-5ED718B8F990}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId37"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9248775" y="70433565"/>
+          <a:ext cx="1962320" cy="542973"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>426</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>769620</xdr:colOff>
+      <xdr:row>428</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="43" name="Picture 42">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B42F046-A29A-1677-AD2A-9A596B393042}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId38">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="75514200"/>
+          <a:ext cx="769620" cy="510540"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>430</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>243840</xdr:colOff>
+      <xdr:row>431</xdr:row>
+      <xdr:rowOff>72390</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="44" name="Picture 43">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5CB6D2FB-D88F-44B5-892F-D776E87C3CFD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId39">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="74714100"/>
+          <a:ext cx="243840" cy="243840"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>432</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>251460</xdr:colOff>
+      <xdr:row>433</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="45" name="Picture 44">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ACDA624A-C868-CC11-AF41-5E1D369231BC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId40">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="76581000"/>
+          <a:ext cx="251460" cy="251460"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>418</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>167640</xdr:colOff>
+      <xdr:row>419</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="46" name="Picture 45">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A59E46F9-1F37-8F14-679D-0C2931F454FD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId41">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="73990200"/>
+          <a:ext cx="167640" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>421</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>167640</xdr:colOff>
+      <xdr:row>422</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="47" name="Picture 46">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C5799D57-65EB-4396-8D9A-D4EDE0DF22E1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId42">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="74561700"/>
+          <a:ext cx="167640" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>100965</xdr:colOff>
+      <xdr:row>455</xdr:row>
+      <xdr:rowOff>49530</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2720566</xdr:colOff>
+      <xdr:row>457</xdr:row>
+      <xdr:rowOff>131483</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="48" name="Picture 47">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{60BD924D-D7CE-2B72-C40A-BF79190A8BA9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId43"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8682990" y="79097505"/>
+          <a:ext cx="2611981" cy="438188"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>458</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>198120</xdr:colOff>
+      <xdr:row>459</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="49" name="Picture 48">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F3922C97-F4CB-8D7B-2A45-47E9B7013A6F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId44">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="6134100" y="81160620"/>
+          <a:ext cx="198120" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2741295</xdr:colOff>
+      <xdr:row>498</xdr:row>
+      <xdr:rowOff>150495</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>550545</xdr:colOff>
+      <xdr:row>503</xdr:row>
+      <xdr:rowOff>93414</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="42" name="Picture 41">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{23F3A13E-5E16-BAD6-6EFD-232BF0B5351C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId45"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12113895" y="86570820"/>
+          <a:ext cx="4945380" cy="811599"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>503</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>213360</xdr:colOff>
+      <xdr:row>504</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="50" name="Picture 49">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A89468F4-DCFF-550B-9992-E8959269CAB7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId46">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="89047320"/>
+          <a:ext cx="213360" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+  <rel r:id="rId2"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4004,10 +5138,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77F27C94-6297-45CB-8ED2-81D711DA05BE}">
-  <dimension ref="A1:J426"/>
+  <dimension ref="A1:J510"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="80.5" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="90.8984375" style="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32.09765625" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="41.296875" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="30.09765625" style="6" bestFit="1" customWidth="1"/>
@@ -4731,7 +5865,7 @@
       <c r="B90" s="6">
         <v>1.25</v>
       </c>
-      <c r="F90" s="31" t="s">
+      <c r="F90" s="36" t="s">
         <v>118</v>
       </c>
     </row>
@@ -4739,7 +5873,7 @@
       <c r="A91" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="F91" s="31"/>
+      <c r="F91" s="36"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
@@ -4751,13 +5885,13 @@
       <c r="C92" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="F92" s="31"/>
+      <c r="F92" s="36"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="F93" s="31"/>
+      <c r="F93" s="36"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
@@ -4769,13 +5903,13 @@
       <c r="C94" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="F94" s="31"/>
+      <c r="F94" s="36"/>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="F95" s="31"/>
+      <c r="F95" s="36"/>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
@@ -4787,13 +5921,13 @@
       <c r="C96" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="F96" s="31"/>
+      <c r="F96" s="36"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="F97" s="31"/>
+      <c r="F97" s="36"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
@@ -4805,13 +5939,13 @@
       <c r="C98" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="F98" s="31"/>
+      <c r="F98" s="36"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="F99" s="31"/>
+      <c r="F99" s="36"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
@@ -4823,7 +5957,7 @@
       <c r="C100" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="F100" s="31"/>
+      <c r="F100" s="36"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="12" t="s">
@@ -5736,13 +6870,13 @@
       <c r="A227" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="C227" s="31" t="s">
+      <c r="C227" s="36" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228"/>
-      <c r="C228" s="31"/>
+      <c r="C228" s="36"/>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
@@ -5752,7 +6886,7 @@
         <f>2*B225+70</f>
         <v>570</v>
       </c>
-      <c r="C229" s="31"/>
+      <c r="C229" s="36"/>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
@@ -5762,17 +6896,17 @@
         <f>2*B226+70</f>
         <v>510</v>
       </c>
-      <c r="C230" s="31"/>
+      <c r="C230" s="36"/>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" s="11" t="s">
         <v>256</v>
       </c>
-      <c r="C231" s="31"/>
+      <c r="C231" s="36"/>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232"/>
-      <c r="C232" s="31"/>
+      <c r="C232" s="36"/>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
@@ -5782,7 +6916,7 @@
         <f>1.8*B225</f>
         <v>450</v>
       </c>
-      <c r="C233" s="31"/>
+      <c r="C233" s="36"/>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
@@ -5792,16 +6926,16 @@
         <f>1.8*B226</f>
         <v>396</v>
       </c>
-      <c r="C234" s="31"/>
+      <c r="C234" s="36"/>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C235" s="31"/>
+      <c r="C235" s="36"/>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="C236" s="31"/>
+      <c r="C236" s="36"/>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
@@ -5810,7 +6944,7 @@
       <c r="B237" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C237" s="31"/>
+      <c r="C237" s="36"/>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
@@ -5819,7 +6953,7 @@
       <c r="B238" s="6">
         <v>1.75</v>
       </c>
-      <c r="C238" s="31"/>
+      <c r="C238" s="36"/>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" s="12" t="s">
@@ -5850,7 +6984,7 @@
       <c r="B244" s="6">
         <v>6</v>
       </c>
-      <c r="C244" s="31" t="s">
+      <c r="C244" s="36" t="s">
         <v>244</v>
       </c>
     </row>
@@ -5861,7 +6995,7 @@
       <c r="B245" s="6">
         <v>6</v>
       </c>
-      <c r="C245" s="31"/>
+      <c r="C245" s="36"/>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" s="12" t="s">
@@ -6080,8 +7214,8 @@
     <row r="282" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A282"/>
       <c r="B282" s="6">
-        <f>0.53*B281*(B77+1)</f>
-        <v>0.66303000000000001</v>
+        <f>ROUND(0.53*B281*(B31+1),3)</f>
+        <v>1.0509999999999999</v>
       </c>
     </row>
     <row r="283" spans="1:2" x14ac:dyDescent="0.25">
@@ -6097,12 +7231,16 @@
       <c r="A285" s="11" t="s">
         <v>262</v>
       </c>
+      <c r="B285">
+        <f>ROUND(B280*(B31+1)*(C67*B283/(B271^2*B31*B281))^(1/3),2)</f>
+        <v>141.94999999999999</v>
+      </c>
     </row>
     <row r="286" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A286"/>
-      <c r="B286">
-        <f>ROUND(B280*(B31+1)*(C67*B283/(B271^2*B31*B281))^(1/3),2)</f>
-        <v>141.94999999999999</v>
+      <c r="B286" s="6">
+        <f>140</f>
+        <v>140</v>
       </c>
     </row>
     <row r="288" spans="1:2" x14ac:dyDescent="0.25">
@@ -6121,18 +7259,18 @@
       </c>
       <c r="B290" s="6">
         <f>0.01*B286</f>
-        <v>1.4195</v>
-      </c>
-      <c r="C290" s="31">
+        <v>1.4000000000000001</v>
+      </c>
+      <c r="C290" s="36">
         <v>2</v>
       </c>
     </row>
     <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B291" s="6">
         <f>0.02*B286</f>
-        <v>2.839</v>
-      </c>
-      <c r="C291" s="31"/>
+        <v>2.8000000000000003</v>
+      </c>
+      <c r="C291" s="36"/>
       <c r="D291" s="6" t="s">
         <v>267</v>
       </c>
@@ -6156,7 +7294,7 @@
       </c>
       <c r="B295" s="6">
         <f>ROUND(2*B286/(2*(B31+1)),2)</f>
-        <v>21.48</v>
+        <v>21.18</v>
       </c>
       <c r="C295" s="6">
         <v>21</v>
@@ -6695,8 +7833,8 @@
         <v>340</v>
       </c>
       <c r="B377" s="6">
-        <f>C355*B373*B375</f>
-        <v>1.37151</v>
+        <f>ROUND(C355*B373*B375,3)</f>
+        <v>1.3720000000000001</v>
       </c>
     </row>
     <row r="378" spans="1:2" x14ac:dyDescent="0.25">
@@ -6708,7 +7846,7 @@
       <c r="A379"/>
       <c r="B379" s="6">
         <f>ROUND(2*C67*B377*B366*B368*B370/(B340*B316*C290),2)</f>
-        <v>53.37</v>
+        <v>53.39</v>
       </c>
     </row>
     <row r="380" spans="1:2" x14ac:dyDescent="0.25">
@@ -6720,7 +7858,7 @@
       <c r="A381"/>
       <c r="B381" s="6">
         <f>ROUND(B379*B371/B370,2)</f>
-        <v>47.56</v>
+        <v>47.58</v>
       </c>
     </row>
     <row r="383" spans="1:2" x14ac:dyDescent="0.25">
@@ -6763,7 +7901,7 @@
       <c r="A398"/>
       <c r="B398" s="6">
         <f>B379*B392</f>
-        <v>106.74</v>
+        <v>106.78</v>
       </c>
       <c r="C398" s="6" t="s">
         <v>350</v>
@@ -6773,7 +7911,7 @@
       <c r="A399"/>
       <c r="B399" s="6">
         <f>B381*B392</f>
-        <v>95.12</v>
+        <v>95.16</v>
       </c>
       <c r="C399" s="6" t="s">
         <v>351</v>
@@ -6794,54 +7932,85 @@
       <c r="B405" s="29"/>
       <c r="C405" s="29"/>
     </row>
-    <row r="406" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A406" s="27"/>
+    <row r="406" spans="1:3" ht="15.6" x14ac:dyDescent="0.25">
+      <c r="A406" s="31" t="s">
+        <v>354</v>
+      </c>
       <c r="B406" s="29"/>
       <c r="C406" s="29"/>
     </row>
     <row r="407" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A407" s="27"/>
+      <c r="A407" s="32" t="s">
+        <v>355</v>
+      </c>
       <c r="B407" s="29"/>
       <c r="C407" s="29"/>
     </row>
     <row r="408" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A408" s="27"/>
+      <c r="A408" s="33" t="s">
+        <v>356</v>
+      </c>
       <c r="B408" s="29"/>
       <c r="C408" s="29"/>
     </row>
     <row r="409" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A409" s="27"/>
-      <c r="B409" s="29"/>
+      <c r="A409" s="27" t="s">
+        <v>357</v>
+      </c>
+      <c r="B409" s="29">
+        <f>B53</f>
+        <v>29277.85</v>
+      </c>
       <c r="C409" s="29"/>
     </row>
     <row r="410" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A410" s="27"/>
+      <c r="A410" s="33" t="s">
+        <v>358</v>
+      </c>
       <c r="B410" s="29"/>
       <c r="C410" s="29"/>
     </row>
     <row r="411" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A411" s="27"/>
+      <c r="A411" s="27" t="s">
+        <v>359</v>
+      </c>
       <c r="B411" s="29"/>
       <c r="C411" s="29"/>
     </row>
     <row r="412" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A412" s="27"/>
-      <c r="B412" s="29"/>
+      <c r="B412" s="29">
+        <v>32</v>
+      </c>
       <c r="C412" s="29"/>
     </row>
     <row r="413" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A413" s="27"/>
+      <c r="A413" s="32" t="s">
+        <v>360</v>
+      </c>
       <c r="B413" s="29"/>
       <c r="C413" s="29"/>
     </row>
     <row r="414" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A414" s="27"/>
-      <c r="B414" s="29"/>
-      <c r="C414" s="29"/>
+      <c r="A414" s="27" t="s">
+        <v>361</v>
+      </c>
+      <c r="B414" s="29" t="s">
+        <v>363</v>
+      </c>
+      <c r="C414" s="29">
+        <f>2</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="415" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A415" s="27"/>
-      <c r="B415" s="29"/>
+      <c r="A415" s="27" t="s">
+        <v>362</v>
+      </c>
+      <c r="B415" s="29">
+        <f>C414*B409</f>
+        <v>58555.7</v>
+      </c>
       <c r="C415" s="29"/>
     </row>
     <row r="416" spans="1:3" ht="15" x14ac:dyDescent="0.25">
@@ -6850,19 +8019,28 @@
       <c r="C416" s="29"/>
     </row>
     <row r="417" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A417" s="27"/>
+      <c r="A417" s="32" t="s">
+        <v>365</v>
+      </c>
       <c r="B417" s="29"/>
       <c r="C417" s="29"/>
     </row>
     <row r="418" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A418" s="27"/>
+      <c r="A418" s="33" t="s">
+        <v>364</v>
+      </c>
       <c r="B418" s="29"/>
       <c r="C418" s="29"/>
     </row>
     <row r="419" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A419" s="27"/>
-      <c r="B419" s="29"/>
-      <c r="C419" s="29"/>
+      <c r="A419"/>
+      <c r="B419" s="29">
+        <f>ROUND(2*C414*B409/(B435*B436*B441*B437),3)</f>
+        <v>0.83</v>
+      </c>
+      <c r="C419" s="29" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="420" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A420" s="27"/>
@@ -6870,14 +8048,21 @@
       <c r="C420" s="29"/>
     </row>
     <row r="421" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A421" s="27"/>
+      <c r="A421" s="33" t="s">
+        <v>366</v>
+      </c>
       <c r="B421" s="29"/>
       <c r="C421" s="29"/>
     </row>
     <row r="422" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A422" s="27"/>
-      <c r="B422" s="29"/>
-      <c r="C422" s="29"/>
+      <c r="A422"/>
+      <c r="B422" s="29">
+        <f>ROUND(C414*B409*B440/(0.1*B441^3*B436*B435),3)</f>
+        <v>18.376000000000001</v>
+      </c>
+      <c r="C422" s="29" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="423" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A423" s="27"/>
@@ -6890,8 +8075,7 @@
       <c r="C424" s="29"/>
     </row>
     <row r="425" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A425" s="27"/>
-      <c r="B425" s="29"/>
+      <c r="A425"/>
       <c r="C425" s="29"/>
     </row>
     <row r="426" spans="1:3" ht="15" x14ac:dyDescent="0.25">
@@ -6899,15 +8083,592 @@
       <c r="B426" s="29"/>
       <c r="C426" s="29"/>
     </row>
+    <row r="427" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A427"/>
+    </row>
+    <row r="431" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="B431" s="29">
+        <f>125</f>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="433" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A433"/>
+      <c r="B433" s="6">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="435" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A435" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="B435" s="6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="436" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A436" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="B436" s="6">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="437" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A437" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B437">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="438" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A438" t="s">
+        <v>370</v>
+      </c>
+      <c r="B438">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="439" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A439" t="s">
+        <v>371</v>
+      </c>
+      <c r="B439">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="440" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A440" t="s">
+        <v>372</v>
+      </c>
+      <c r="B440" s="6">
+        <f>B438+B439/2</f>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="441" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A441" t="s">
+        <v>373</v>
+      </c>
+      <c r="B441">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="444" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A444" s="4" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="445" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A445" s="4" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="446" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A446" s="37" t="s">
+        <v>377</v>
+      </c>
+      <c r="B446" s="37" t="s">
+        <v>187</v>
+      </c>
+      <c r="C446" s="37" t="s">
+        <v>378</v>
+      </c>
+      <c r="D446" s="37" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E446" s="37" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="447" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A447" s="38"/>
+      <c r="B447" s="38"/>
+      <c r="C447" s="38"/>
+      <c r="D447" s="38"/>
+      <c r="E447" s="38"/>
+    </row>
+    <row r="448" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A448" s="34" t="s">
+        <v>379</v>
+      </c>
+      <c r="B448" s="35" t="s">
+        <v>188</v>
+      </c>
+      <c r="C448" s="35" t="s">
+        <v>380</v>
+      </c>
+      <c r="D448" s="35">
+        <v>750</v>
+      </c>
+      <c r="E448" s="35">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="450" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A450" s="4" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="451" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A451" s="11" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="452" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A452" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="B452" s="6">
+        <f>ROUND(2*B409/B316,3)</f>
+        <v>1394.5150000000001</v>
+      </c>
+    </row>
+    <row r="453" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A453" s="11" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="454" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A454" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="B454" s="6">
+        <f>ROUND(B452*TAN(RADIANS(B332))/COS(B294),3)</f>
+        <v>507.56200000000001</v>
+      </c>
+    </row>
+    <row r="455" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A455" s="11" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="456" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A456" t="s">
+        <v>387</v>
+      </c>
+      <c r="B456" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="458" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A458" s="4" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="459" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A459" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="B459"/>
+      <c r="C459" s="6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="460" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A460" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="B460" s="6">
+        <f>(B409/(0.2*C459))^(1/3)</f>
+        <v>21.370071516649542</v>
+      </c>
+    </row>
+    <row r="461" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A461" t="s">
+        <v>391</v>
+      </c>
+      <c r="B461" s="6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="462" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A462" s="12" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="463" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A463" t="s">
+        <v>392</v>
+      </c>
+      <c r="B463" s="6">
+        <v>17</v>
+      </c>
+      <c r="C463" s="6" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="464" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A464" s="12" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="465" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A465" t="s">
+        <v>406</v>
+      </c>
+      <c r="B465" s="6">
+        <f>1.2*B461</f>
+        <v>30</v>
+      </c>
+      <c r="C465" s="6">
+        <f>1.5*B461</f>
+        <v>37.5</v>
+      </c>
+      <c r="D465" s="6">
+        <v>35</v>
+      </c>
+      <c r="E465" s="6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="466" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A466" s="12" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="467" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A467" t="s">
+        <v>407</v>
+      </c>
+      <c r="B467" s="6">
+        <f>1.4*B461</f>
+        <v>35</v>
+      </c>
+      <c r="C467" s="6">
+        <f>2.5*B461</f>
+        <v>62.5</v>
+      </c>
+      <c r="D467" s="6">
+        <v>50</v>
+      </c>
+      <c r="E467" s="6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="468" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A468" s="12" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="469" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A469" t="s">
+        <v>397</v>
+      </c>
+      <c r="B469" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="470" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A470" s="12" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="471" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A471" t="s">
+        <v>399</v>
+      </c>
+      <c r="B471" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="472" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A472" s="12" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="473" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A473" t="s">
+        <v>401</v>
+      </c>
+      <c r="B473" s="6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="474" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A474" s="12" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="475" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A475" t="s">
+        <v>403</v>
+      </c>
+      <c r="B475" s="6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="476" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A476" s="12" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="477" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A477" t="s">
+        <v>408</v>
+      </c>
+      <c r="B477" s="6">
+        <f>0.5*(B467+B463)+B473+B475</f>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="478" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A478" s="12" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="479" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A479" t="s">
+        <v>415</v>
+      </c>
+      <c r="B479" s="6">
+        <f>2*B481</f>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="480" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A480" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="481" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A481" t="s">
+        <v>410</v>
+      </c>
+      <c r="B481" s="6">
+        <f>0.5*(B465+B463)+B469+B471</f>
+        <v>43.5</v>
+      </c>
+    </row>
+    <row r="482" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A482" s="12" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="483" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A483" t="s">
+        <v>412</v>
+      </c>
+      <c r="B483" s="6">
+        <f>B340</f>
+        <v>41.699999999999996</v>
+      </c>
+    </row>
+    <row r="485" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A485" s="4" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="486" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A486" t="s">
+        <v>416</v>
+      </c>
+      <c r="B486" s="6">
+        <f>ROUND(2*B409/B436,3)</f>
+        <v>650.61900000000003</v>
+      </c>
+    </row>
+    <row r="487" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A487" t="s">
+        <v>417</v>
+      </c>
+      <c r="B487" s="6">
+        <f>0.2*B486</f>
+        <v>130.12380000000002</v>
+      </c>
+    </row>
+    <row r="488" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A488" t="s">
+        <v>418</v>
+      </c>
+      <c r="B488" s="6">
+        <v>483.37619999999998</v>
+      </c>
+    </row>
+    <row r="489" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A489" s="6" t="s">
+        <v>419</v>
+      </c>
+      <c r="B489" s="6">
+        <f>B454-B491</f>
+        <v>253.78200000000001</v>
+      </c>
+    </row>
+    <row r="490" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A490" s="39" t="s">
+        <v>420</v>
+      </c>
+      <c r="B490" s="6">
+        <v>781.01499999999999</v>
+      </c>
+    </row>
+    <row r="491" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A491" s="39" t="s">
+        <v>421</v>
+      </c>
+      <c r="B491" s="6">
+        <f>253.78</f>
+        <v>253.78</v>
+      </c>
+    </row>
+    <row r="492" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A492" s="40" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="493" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A493" s="39" t="s">
+        <v>422</v>
+      </c>
+      <c r="B493" s="6">
+        <f>B490*B481</f>
+        <v>33974.152499999997</v>
+      </c>
+      <c r="C493" s="6">
+        <f>B487*(B477+B481)+B488*B481</f>
+        <v>33974.182800000002</v>
+      </c>
+      <c r="D493" s="36" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="494" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A494" s="39" t="s">
+        <v>424</v>
+      </c>
+      <c r="B494" s="6">
+        <f>B491*B481</f>
+        <v>11039.43</v>
+      </c>
+      <c r="D494" s="36"/>
+    </row>
+    <row r="496" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A496" s="4" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="497" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A497" s="40" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="498" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A498" s="39" t="s">
+        <v>427</v>
+      </c>
+      <c r="B498" s="6">
+        <f>SQRT(0+0+0.75*B409^2)</f>
+        <v>25355.361868190226</v>
+      </c>
+    </row>
+    <row r="499" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A499" s="40" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="500" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A500" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="B500" s="6">
+        <f>SQRT(0+(B487*B477)^2+0.75*B409^2)</f>
+        <v>26381.693749617192</v>
+      </c>
+    </row>
+    <row r="501" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A501" s="11" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="502" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A502" s="39" t="s">
+        <v>431</v>
+      </c>
+      <c r="B502" s="6">
+        <f>SQRT(B493^2+B494^2+0.75*B409^2)</f>
+        <v>43806.465599098847</v>
+      </c>
+    </row>
+    <row r="503" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A503" s="41" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="504" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A504"/>
+      <c r="B504" s="6">
+        <f>63</f>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="505" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A505" s="11" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="506" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A506" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="B506" s="6">
+        <f>(B498/(0.1*B504))^(1/3)</f>
+        <v>15.906565612513687</v>
+      </c>
+      <c r="C506" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="507" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A507" s="42" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="508" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A508" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="B508" s="6">
+        <f t="shared" ref="B507:B510" si="0">(B500/(0.1*B506))^(1/3)</f>
+        <v>25.502069076896909</v>
+      </c>
+      <c r="C508" s="6">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="509" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A509" s="42" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="510" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A510" s="39" t="s">
+        <v>437</v>
+      </c>
+      <c r="B510" s="6">
+        <f t="shared" si="0"/>
+        <v>25.802053159314557</v>
+      </c>
+      <c r="C510" s="6">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="10">
+    <mergeCell ref="D493:D494"/>
     <mergeCell ref="F90:F100"/>
     <mergeCell ref="C227:C238"/>
     <mergeCell ref="C244:C245"/>
     <mergeCell ref="C290:C291"/>
+    <mergeCell ref="A446:A447"/>
+    <mergeCell ref="B446:B447"/>
+    <mergeCell ref="C446:C447"/>
+    <mergeCell ref="D446:D447"/>
+    <mergeCell ref="E446:E447"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
hoàn thành tính toán thiết kế trục I
</commit_message>
<xml_diff>
--- a/tínhtoans.xlsx
+++ b/tínhtoans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Đồ án tkm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0C0F40-5B29-4B5C-8B8D-629F6D72C7CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BAF4F55-B09D-4DC2-BB1F-59487031ED5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{75337E03-C337-4BFE-A279-78895F300CE2}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{75337E03-C337-4BFE-A279-78895F300CE2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="474">
   <si>
     <t>Bánh răng trụ răng thẳng</t>
   </si>
@@ -1408,12 +1408,120 @@
   <si>
     <t>d BR</t>
   </si>
+  <si>
+    <t>4.2.8. Chọn then và kiểm nghiệm then</t>
+  </si>
+  <si>
+    <t>a. Then bằng để lắp khớp nối</t>
+  </si>
+  <si>
+    <t>Chiều rộng then</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>Chiều cao then</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>t1</t>
+  </si>
+  <si>
+    <t>Chiều sâu rãnh then trên lỗ</t>
+  </si>
+  <si>
+    <t>Chiều sâu rãnh then trên trục</t>
+  </si>
+  <si>
+    <t>t2</t>
+  </si>
+  <si>
+    <t>Chiều dài then</t>
+  </si>
+  <si>
+    <t>l_t</t>
+  </si>
+  <si>
+    <t>thỏa mãn &lt; 50 MPa</t>
+  </si>
+  <si>
+    <t>thỏa mãn nhỏ hơn 1/3(60-90) MPa</t>
+  </si>
+  <si>
+    <t>b. Then bằng để lắp bánh răng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đường kính trục </t>
+  </si>
+  <si>
+    <t>4.2.9. Tính kiểm nghiệm trục về độ bền mỏi</t>
+  </si>
+  <si>
+    <t>Hệ số an toàn chỉ xét riêng ứng suất tiếp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giới hạn mỏi uốn </t>
+  </si>
+  <si>
+    <t xml:space="preserve">   </t>
+  </si>
+  <si>
+    <t>Biên độ và trị số trung bình của ứng suất pháp và ứng suất tiếp tại tiết diện j</t>
+  </si>
+  <si>
+    <t>Đối với trục quay, ứng suất uốn thay đôir theo chu kì đối xứng</t>
+  </si>
+  <si>
+    <t>Khi trục quay 1 chiều ứng suất xoắn thay đổi theo chu kỳ mạch động</t>
+  </si>
+  <si>
+    <t>hệ số kể đến ảnh hưởng của trị số ứng suất trung bình dến độ bền mỏi</t>
+  </si>
+  <si>
+    <t>hệ số tập trung ứng suất do trạng thái bề mặt, phụ thuộc vào phương pháp gia công và độ nhẵn bề mặt</t>
+  </si>
+  <si>
+    <t>K_x</t>
+  </si>
+  <si>
+    <t>hệ số tăng bền bề mặt trục, phụ thuộc vào phương pháp tăng bền bề mặt, cơ tính vật liệu</t>
+  </si>
+  <si>
+    <t>K_y</t>
+  </si>
+  <si>
+    <t>hệ số kích thước kể đến ảnh hưởng của kích thước tiết diện trục đến giới hạn mỏi</t>
+  </si>
+  <si>
+    <t>hệ số tập trung ứng suất thực tê khi uốn và khi xoắn, trị số của chúng phụ thuộc vào loại yếu tố gây tập trung ứng suất</t>
+  </si>
+  <si>
+    <t>Hệ số</t>
+  </si>
+  <si>
+    <t>Trục có 1 rãnh then</t>
+  </si>
+  <si>
+    <t>Momen cản uốn</t>
+  </si>
+  <si>
+    <t>Momen cản xoắn</t>
+  </si>
+  <si>
+    <t>thỏa mãn &gt; [s] = 2.5...3</t>
+  </si>
+  <si>
+    <t>4.2.10. Tính kiểm nghiệm trục về độ bền tĩnh</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1527,6 +1635,18 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1628,7 +1748,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1707,19 +1827,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4731,6 +4852,2461 @@
         <a:xfrm>
           <a:off x="0" y="89047320"/>
           <a:ext cx="213360" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>510</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1078746</xdr:colOff>
+      <xdr:row>516</xdr:row>
+      <xdr:rowOff>81999</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="51" name="Picture 50">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{77A71DB6-205F-00E2-C4EF-AAE49D5AC60B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId47"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9934575" y="88620600"/>
+          <a:ext cx="5955546" cy="967824"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>527</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>167640</xdr:colOff>
+      <xdr:row>528</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="52" name="Picture 51">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E69F76AE-299F-B6DB-6BC8-8CFE51CDEC70}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId41">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="93253560"/>
+          <a:ext cx="167640" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>528</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>144780</xdr:colOff>
+      <xdr:row>529</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="53" name="Picture 52">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8648140-B452-94C9-C2D0-747C1C0A3F55}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId48">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="93428820"/>
+          <a:ext cx="144780" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>543</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>167640</xdr:colOff>
+      <xdr:row>544</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="54" name="Picture 53">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D05A7A3D-9296-434D-BFA2-84B887DBBD88}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId41">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="93253560"/>
+          <a:ext cx="167640" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>544</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>144780</xdr:colOff>
+      <xdr:row>545</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="55" name="Picture 54">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{48DC5D5D-FC0E-4C0B-AD1F-D71917AEC2DD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId48">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="93428820"/>
+          <a:ext cx="144780" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>547</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2484335</xdr:colOff>
+      <xdr:row>549</xdr:row>
+      <xdr:rowOff>83858</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="56" name="Picture 55">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EE473826-65B8-AD11-AE94-3B0F4F7F187F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId49"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="96758760"/>
+          <a:ext cx="2484335" cy="434378"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>552</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>213360</xdr:colOff>
+      <xdr:row>552</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="59" name="Picture 58">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{234B9259-11D1-49AC-438D-7BDF30600AAA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId50">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="97459800"/>
+          <a:ext cx="213360" cy="228600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>3764280</xdr:colOff>
+      <xdr:row>543</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>5913306</xdr:colOff>
+      <xdr:row>549</xdr:row>
+      <xdr:rowOff>83913</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="61" name="Picture 60">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6477120A-E325-45A0-03B9-2ED2AD86065E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId51"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3764280" y="96118680"/>
+          <a:ext cx="2149026" cy="1074513"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>551</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>243840</xdr:colOff>
+      <xdr:row>551</xdr:row>
+      <xdr:rowOff>205740</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="63" name="Picture 62">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1F2D4245-FF4F-D450-7326-D776276DAAFE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId52">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="97459800"/>
+          <a:ext cx="243840" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>553</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>553</xdr:row>
+      <xdr:rowOff>205740</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="64" name="Picture 63">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6010FF4B-41B8-5120-1965-E687E577A248}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId53">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="97848420"/>
+          <a:ext cx="228600" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>555</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>220980</xdr:colOff>
+      <xdr:row>556</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="65" name="Picture 64">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0A7D01C9-CB61-C721-0FD0-2050BB9076F3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId54">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="98237040"/>
+          <a:ext cx="220980" cy="228600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>555</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>3063505</xdr:colOff>
+      <xdr:row>557</xdr:row>
+      <xdr:rowOff>45758</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="66" name="Picture 65">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A369387E-C4D6-9992-15AF-B42BD086DAB9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId55"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9372600" y="98412300"/>
+          <a:ext cx="3063505" cy="434378"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>558</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2446232</xdr:colOff>
+      <xdr:row>559</xdr:row>
+      <xdr:rowOff>114325</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="67" name="Picture 66">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{396DC03C-50E8-7560-ADB1-9FBED15683F4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId56"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="98800920"/>
+          <a:ext cx="2446232" cy="289585"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>561</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2453853</xdr:colOff>
+      <xdr:row>562</xdr:row>
+      <xdr:rowOff>167670</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="68" name="Picture 67">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{23A53C7B-34E7-BC81-149A-757EBADC8A6A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId57"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="99326700"/>
+          <a:ext cx="2453853" cy="342930"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>564</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>198120</xdr:colOff>
+      <xdr:row>564</xdr:row>
+      <xdr:rowOff>205740</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="69" name="Picture 68">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FF88A2BD-1767-F021-632E-5E089C2FF8A0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId58">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="99852480"/>
+          <a:ext cx="198120" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>565</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>175260</xdr:colOff>
+      <xdr:row>566</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="70" name="Picture 69">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{239B5431-8F29-2CF1-2D6E-5074BB582A1E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId59">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="100065840"/>
+          <a:ext cx="175260" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>571</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>160020</xdr:colOff>
+      <xdr:row>571</xdr:row>
+      <xdr:rowOff>205740</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="71" name="Picture 70">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6E283639-1515-BB09-92CF-2EDD1B82B52B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId60">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="101117400"/>
+          <a:ext cx="160020" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>572</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>137160</xdr:colOff>
+      <xdr:row>572</xdr:row>
+      <xdr:rowOff>205740</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="72" name="Picture 71">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{747A5485-BA75-9847-1510-8AD88AEEF4FE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId61">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="101330760"/>
+          <a:ext cx="137160" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>574</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>464820</xdr:colOff>
+      <xdr:row>575</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="75" name="Picture 74">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{782108F2-0004-7E94-11AA-D1F81EC65E3D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId62">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="101719380"/>
+          <a:ext cx="464820" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>575</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>388620</xdr:colOff>
+      <xdr:row>576</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="77" name="Picture 76">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1BCA4DE1-893F-91EC-9AC1-A101B644CAD5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId63">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="101894640"/>
+          <a:ext cx="388620" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>577</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>312420</xdr:colOff>
+      <xdr:row>578</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="78" name="Picture 77">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B4F1D6EB-77B9-FB21-FD0E-FC2DEB752E5C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId64">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="102245160"/>
+          <a:ext cx="312420" cy="228600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>578</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>297180</xdr:colOff>
+      <xdr:row>579</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="79" name="Picture 78">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C71F486D-9738-386C-4F4B-716AFE1A9A7A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId65">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="102458520"/>
+          <a:ext cx="297180" cy="228600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>129540</xdr:colOff>
+      <xdr:row>577</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2240463</xdr:colOff>
+      <xdr:row>579</xdr:row>
+      <xdr:rowOff>45758</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="80" name="Picture 79">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CF0074B6-593C-556D-6FB5-8353BB0523BD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId66"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9502140" y="102245160"/>
+          <a:ext cx="2110923" cy="434378"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>15240</xdr:colOff>
+      <xdr:row>580</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>960475</xdr:colOff>
+      <xdr:row>582</xdr:row>
+      <xdr:rowOff>99098</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="84" name="Picture 83">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DCCD5351-17AD-AEB0-1E77-B75636400A45}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId67"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9387840" y="102824280"/>
+          <a:ext cx="4092295" cy="434378"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>581</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>205740</xdr:colOff>
+      <xdr:row>582</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="89" name="Picture 88">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7CDDD56D-F79C-6DFD-5D94-606862F5EFDE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId68">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="102984300"/>
+          <a:ext cx="205740" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>583</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>274320</xdr:colOff>
+      <xdr:row>584</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="90" name="Picture 89">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7F7F87C9-FA11-F144-CD3A-DF14F9A0D750}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId69">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="103334820"/>
+          <a:ext cx="274320" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>585</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>464820</xdr:colOff>
+      <xdr:row>586</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="91" name="Picture 90">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BA17E858-F52D-2936-4A70-99B8B80D203A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId70">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="103685340"/>
+          <a:ext cx="464820" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>586</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>845820</xdr:colOff>
+      <xdr:row>587</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="92" name="Picture 91">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C019149-BC8A-F3EA-8DFA-0C378231F16C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId71">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="103860600"/>
+          <a:ext cx="845820" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>588</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1501140</xdr:colOff>
+      <xdr:row>590</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="93" name="Picture 92">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D659EED9-46DE-DB06-EA77-52C2BCCA9B4E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId72">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="104211120"/>
+          <a:ext cx="1501140" cy="350520"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>591</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>220980</xdr:colOff>
+      <xdr:row>592</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="94" name="Picture 93">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8FF341A9-08A4-0519-2CF6-289FEC31A23F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId73">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="104736900"/>
+          <a:ext cx="220980" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>592</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>205740</xdr:colOff>
+      <xdr:row>593</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="95" name="Picture 94">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9D0EC5F7-3BBC-BDDE-D5B5-2FA3C56D7DE9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId74">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="104912160"/>
+          <a:ext cx="205740" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>594</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>144780</xdr:colOff>
+      <xdr:row>595</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="96" name="Picture 95">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9EE3F511-4EA4-3917-37EA-9007F171C8EA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId75">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="105262680"/>
+          <a:ext cx="144780" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>597</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1600200</xdr:colOff>
+      <xdr:row>598</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="97" name="Picture 96">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{423E0F06-69E2-A3B5-D6E3-6D8C05160F1E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId76">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="105788460"/>
+          <a:ext cx="1600200" cy="259080"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>600</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>99060</xdr:colOff>
+      <xdr:row>601</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="98" name="Picture 97">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{90193A35-8543-7EB5-CA21-D0232BBCBECA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId77">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="106314240"/>
+          <a:ext cx="99060" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>3947160</xdr:colOff>
+      <xdr:row>593</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>5471292</xdr:colOff>
+      <xdr:row>599</xdr:row>
+      <xdr:rowOff>7703</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="99" name="Picture 98">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5625B720-8F0C-CE8D-3F83-AFB3B9EAA820}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId78"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3947160" y="105186480"/>
+          <a:ext cx="1524132" cy="960203"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>601</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>602</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="100" name="Picture 99">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0D581366-CF5B-B411-731F-41F8B734301D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId79">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="106489500"/>
+          <a:ext cx="76200" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>602</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>609600</xdr:colOff>
+      <xdr:row>603</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="101" name="Picture 100">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8F79ABEF-73B0-BA86-A0DF-13CD38588131}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId80">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="106664760"/>
+          <a:ext cx="609600" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>603</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>205740</xdr:colOff>
+      <xdr:row>604</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="102" name="Picture 101">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{28FAB78B-8EF3-63D1-EFAA-DE87301BF90C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId81">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="106840020"/>
+          <a:ext cx="205740" cy="205740"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5138,7 +7714,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77F27C94-6297-45CB-8ED2-81D711DA05BE}">
-  <dimension ref="A1:J510"/>
+  <dimension ref="A1:J604"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="90.8984375" style="6" bestFit="1" customWidth="1"/>
@@ -5865,7 +8441,7 @@
       <c r="B90" s="6">
         <v>1.25</v>
       </c>
-      <c r="F90" s="36" t="s">
+      <c r="F90" s="39" t="s">
         <v>118</v>
       </c>
     </row>
@@ -5873,7 +8449,7 @@
       <c r="A91" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="F91" s="36"/>
+      <c r="F91" s="39"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
@@ -5885,13 +8461,13 @@
       <c r="C92" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="F92" s="36"/>
+      <c r="F92" s="39"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="F93" s="36"/>
+      <c r="F93" s="39"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
@@ -5903,13 +8479,13 @@
       <c r="C94" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="F94" s="36"/>
+      <c r="F94" s="39"/>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="F95" s="36"/>
+      <c r="F95" s="39"/>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
@@ -5921,13 +8497,13 @@
       <c r="C96" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="F96" s="36"/>
+      <c r="F96" s="39"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="F97" s="36"/>
+      <c r="F97" s="39"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
@@ -5939,13 +8515,13 @@
       <c r="C98" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="F98" s="36"/>
+      <c r="F98" s="39"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="F99" s="36"/>
+      <c r="F99" s="39"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
@@ -5957,7 +8533,7 @@
       <c r="C100" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="F100" s="36"/>
+      <c r="F100" s="39"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="12" t="s">
@@ -6870,13 +9446,13 @@
       <c r="A227" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="C227" s="36" t="s">
+      <c r="C227" s="39" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228"/>
-      <c r="C228" s="36"/>
+      <c r="C228" s="39"/>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
@@ -6886,7 +9462,7 @@
         <f>2*B225+70</f>
         <v>570</v>
       </c>
-      <c r="C229" s="36"/>
+      <c r="C229" s="39"/>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
@@ -6896,17 +9472,17 @@
         <f>2*B226+70</f>
         <v>510</v>
       </c>
-      <c r="C230" s="36"/>
+      <c r="C230" s="39"/>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" s="11" t="s">
         <v>256</v>
       </c>
-      <c r="C231" s="36"/>
+      <c r="C231" s="39"/>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232"/>
-      <c r="C232" s="36"/>
+      <c r="C232" s="39"/>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
@@ -6916,7 +9492,7 @@
         <f>1.8*B225</f>
         <v>450</v>
       </c>
-      <c r="C233" s="36"/>
+      <c r="C233" s="39"/>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
@@ -6926,16 +9502,16 @@
         <f>1.8*B226</f>
         <v>396</v>
       </c>
-      <c r="C234" s="36"/>
+      <c r="C234" s="39"/>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C235" s="36"/>
+      <c r="C235" s="39"/>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="C236" s="36"/>
+      <c r="C236" s="39"/>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
@@ -6944,7 +9520,7 @@
       <c r="B237" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C237" s="36"/>
+      <c r="C237" s="39"/>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
@@ -6953,7 +9529,7 @@
       <c r="B238" s="6">
         <v>1.75</v>
       </c>
-      <c r="C238" s="36"/>
+      <c r="C238" s="39"/>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" s="12" t="s">
@@ -6984,7 +9560,7 @@
       <c r="B244" s="6">
         <v>6</v>
       </c>
-      <c r="C244" s="36" t="s">
+      <c r="C244" s="39" t="s">
         <v>244</v>
       </c>
     </row>
@@ -6995,7 +9571,7 @@
       <c r="B245" s="6">
         <v>6</v>
       </c>
-      <c r="C245" s="36"/>
+      <c r="C245" s="39"/>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" s="12" t="s">
@@ -7261,7 +9837,7 @@
         <f>0.01*B286</f>
         <v>1.4000000000000001</v>
       </c>
-      <c r="C290" s="36">
+      <c r="C290" s="39">
         <v>2</v>
       </c>
     </row>
@@ -7270,7 +9846,7 @@
         <f>0.02*B286</f>
         <v>2.8000000000000003</v>
       </c>
-      <c r="C291" s="36"/>
+      <c r="C291" s="39"/>
       <c r="D291" s="6" t="s">
         <v>267</v>
       </c>
@@ -8221,8 +10797,8 @@
         <v>383</v>
       </c>
       <c r="B452" s="6">
-        <f>ROUND(2*B409/B316,3)</f>
-        <v>1394.5150000000001</v>
+        <f>ROUND(2*B55/B316,3)</f>
+        <v>1366.184</v>
       </c>
     </row>
     <row r="453" spans="1:3" x14ac:dyDescent="0.25">
@@ -8236,7 +10812,7 @@
       </c>
       <c r="B454" s="6">
         <f>ROUND(B452*TAN(RADIANS(B332))/COS(B294),3)</f>
-        <v>507.56200000000001</v>
+        <v>497.25</v>
       </c>
     </row>
     <row r="455" spans="1:3" x14ac:dyDescent="0.25">
@@ -8271,8 +10847,8 @@
         <v>390</v>
       </c>
       <c r="B460" s="6">
-        <f>(B409/(0.2*C459))^(1/3)</f>
-        <v>21.370071516649542</v>
+        <f>(B55/(0.2*C459))^(1/3)</f>
+        <v>21.224361851997458</v>
       </c>
     </row>
     <row r="461" spans="1:3" x14ac:dyDescent="0.25">
@@ -8465,8 +11041,8 @@
         <v>416</v>
       </c>
       <c r="B486" s="6">
-        <f>ROUND(2*B409/B436,3)</f>
-        <v>650.61900000000003</v>
+        <f>ROUND(2*B55/B436,3)</f>
+        <v>637.40099999999995</v>
       </c>
     </row>
     <row r="487" spans="1:4" x14ac:dyDescent="0.25">
@@ -8475,7 +11051,7 @@
       </c>
       <c r="B487" s="6">
         <f>0.2*B486</f>
-        <v>130.12380000000002</v>
+        <v>127.4802</v>
       </c>
     </row>
     <row r="488" spans="1:4" x14ac:dyDescent="0.25">
@@ -8492,11 +11068,11 @@
       </c>
       <c r="B489" s="6">
         <f>B454-B491</f>
-        <v>253.78200000000001</v>
+        <v>243.47</v>
       </c>
     </row>
     <row r="490" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A490" s="39" t="s">
+      <c r="A490" t="s">
         <v>420</v>
       </c>
       <c r="B490" s="6">
@@ -8504,7 +11080,7 @@
       </c>
     </row>
     <row r="491" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A491" s="39" t="s">
+      <c r="A491" t="s">
         <v>421</v>
       </c>
       <c r="B491" s="6">
@@ -8513,12 +11089,12 @@
       </c>
     </row>
     <row r="492" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A492" s="40" t="s">
+      <c r="A492" s="12" t="s">
         <v>423</v>
       </c>
     </row>
     <row r="493" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A493" s="39" t="s">
+      <c r="A493" t="s">
         <v>422</v>
       </c>
       <c r="B493" s="6">
@@ -8527,21 +11103,21 @@
       </c>
       <c r="C493" s="6">
         <f>B487*(B477+B481)+B488*B481</f>
-        <v>33974.182800000002</v>
-      </c>
-      <c r="D493" s="36" t="s">
+        <v>33711.1446</v>
+      </c>
+      <c r="D493" s="39" t="s">
         <v>432</v>
       </c>
     </row>
     <row r="494" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A494" s="39" t="s">
+      <c r="A494" t="s">
         <v>424</v>
       </c>
       <c r="B494" s="6">
         <f>B491*B481</f>
         <v>11039.43</v>
       </c>
-      <c r="D494" s="36"/>
+      <c r="D494" s="39"/>
     </row>
     <row r="496" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A496" s="4" t="s">
@@ -8549,21 +11125,21 @@
       </c>
     </row>
     <row r="497" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A497" s="40" t="s">
+      <c r="A497" s="12" t="s">
         <v>426</v>
       </c>
     </row>
     <row r="498" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A498" s="39" t="s">
+      <c r="A498" t="s">
         <v>427</v>
       </c>
       <c r="B498" s="6">
-        <f>SQRT(0+0+0.75*B409^2)</f>
-        <v>25355.361868190226</v>
+        <f>SQRT(0+0+0.75*B55^2)</f>
+        <v>24840.241297765206</v>
       </c>
     </row>
     <row r="499" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A499" s="40" t="s">
+      <c r="A499" s="12" t="s">
         <v>428</v>
       </c>
     </row>
@@ -8572,8 +11148,8 @@
         <v>429</v>
       </c>
       <c r="B500" s="6">
-        <f>SQRT(0+(B487*B477)^2+0.75*B409^2)</f>
-        <v>26381.693749617192</v>
+        <f>SQRT(0+(B487*B477)^2+0.75*B55^2)</f>
+        <v>25845.722185627495</v>
       </c>
     </row>
     <row r="501" spans="1:3" x14ac:dyDescent="0.25">
@@ -8582,16 +11158,16 @@
       </c>
     </row>
     <row r="502" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A502" s="39" t="s">
+      <c r="A502" t="s">
         <v>431</v>
       </c>
       <c r="B502" s="6">
-        <f>SQRT(B493^2+B494^2+0.75*B409^2)</f>
-        <v>43806.465599098847</v>
+        <f>SQRT(B493^2+B494^2+0.75*B55^2)</f>
+        <v>43510.339467181315</v>
       </c>
     </row>
     <row r="503" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A503" s="41" t="s">
+      <c r="A503" s="36" t="s">
         <v>433</v>
       </c>
     </row>
@@ -8613,14 +11189,14 @@
       </c>
       <c r="B506" s="6">
         <f>(B498/(0.1*B504))^(1/3)</f>
-        <v>15.906565612513687</v>
+        <v>15.798108308598721</v>
       </c>
       <c r="C506" s="6">
         <v>20</v>
       </c>
     </row>
     <row r="507" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A507" s="42" t="s">
+      <c r="A507" s="12" t="s">
         <v>435</v>
       </c>
     </row>
@@ -8629,28 +11205,536 @@
         <v>287</v>
       </c>
       <c r="B508" s="6">
-        <f t="shared" ref="B507:B510" si="0">(B500/(0.1*B506))^(1/3)</f>
-        <v>25.502069076896909</v>
+        <f t="shared" ref="B508:B510" si="0">(B500/(0.1*B506))^(1/3)</f>
+        <v>25.386014763892227</v>
       </c>
       <c r="C508" s="6">
         <v>30</v>
       </c>
     </row>
     <row r="509" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A509" s="42" t="s">
+      <c r="A509" s="12" t="s">
         <v>436</v>
       </c>
     </row>
     <row r="510" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A510" s="39" t="s">
+      <c r="A510" t="s">
         <v>437</v>
       </c>
       <c r="B510" s="6">
         <f t="shared" si="0"/>
-        <v>25.802053159314557</v>
+        <v>25.782952457296389</v>
       </c>
       <c r="C510" s="6">
         <v>35</v>
+      </c>
+    </row>
+    <row r="512" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A512" s="4" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="514" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A514" s="4" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="515" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A515" s="42" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="516" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A516" s="41" t="s">
+        <v>390</v>
+      </c>
+      <c r="B516" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="517" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A517" s="11" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="518" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A518" s="6" t="s">
+        <v>441</v>
+      </c>
+      <c r="B518" s="6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="519" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A519" s="11" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="520" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A520" s="40" t="s">
+        <v>443</v>
+      </c>
+      <c r="B520" s="6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="521" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A521" s="11" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="522" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A522" s="40" t="s">
+        <v>444</v>
+      </c>
+      <c r="B522" s="6">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="523" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A523" s="42" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="524" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A524" s="40" t="s">
+        <v>447</v>
+      </c>
+      <c r="B524" s="6">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="525" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A525" s="42" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="526" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A526" s="40" t="s">
+        <v>449</v>
+      </c>
+      <c r="B526" s="6">
+        <f>0.8*B467</f>
+        <v>28</v>
+      </c>
+      <c r="C526" s="6">
+        <f>0.9*B467</f>
+        <v>31.5</v>
+      </c>
+      <c r="D526" s="6">
+        <v>30</v>
+      </c>
+      <c r="E526" s="6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="528" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A528"/>
+      <c r="B528" s="6">
+        <f>2*B55/(B516*D526*(B520-B522))</f>
+        <v>38.244053333333333</v>
+      </c>
+      <c r="C528" s="6" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="529" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A529"/>
+      <c r="B529" s="6">
+        <f>2*B55/(B516*B518*D526)</f>
+        <v>15.935022222222223</v>
+      </c>
+      <c r="C529" s="6" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="530" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A530" s="4" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="531" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A531" s="11" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="532" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A532" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="B532" s="6">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="533" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A533" s="42" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="534" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A534" s="6" t="s">
+        <v>441</v>
+      </c>
+      <c r="B534" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="535" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A535" s="11" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="536" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A536" s="40" t="s">
+        <v>443</v>
+      </c>
+      <c r="B536" s="6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="537" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A537" s="42" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="538" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A538" s="40" t="s">
+        <v>444</v>
+      </c>
+      <c r="B538" s="6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="539" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A539" s="42" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="540" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A540" s="40" t="s">
+        <v>447</v>
+      </c>
+      <c r="B540" s="6">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="541" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A541" s="42" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="542" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A542" s="40" t="s">
+        <v>449</v>
+      </c>
+      <c r="B542" s="6">
+        <f>0.8*B465</f>
+        <v>24</v>
+      </c>
+      <c r="C542" s="6">
+        <f>0.9*B465</f>
+        <v>27</v>
+      </c>
+      <c r="D542" s="6">
+        <v>25</v>
+      </c>
+      <c r="E542" s="6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="544" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A544"/>
+      <c r="B544" s="6">
+        <f>2*B55/(B532*D542*(B536-B538))</f>
+        <v>21.853744761904764</v>
+      </c>
+      <c r="C544" s="6" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="545" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A545"/>
+      <c r="B545" s="6">
+        <f>2*B55/(B532*B534*D542)</f>
+        <v>6.5561234285714285</v>
+      </c>
+      <c r="C545" s="6" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="547" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A547" s="4" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="551" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A551" s="11" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="552" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A552" s="43" t="s">
+        <v>457</v>
+      </c>
+      <c r="B552" s="6">
+        <f>0.436*D448</f>
+        <v>327</v>
+      </c>
+    </row>
+    <row r="553" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A553" s="11" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="554" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A554" s="43" t="s">
+        <v>117</v>
+      </c>
+      <c r="B554" s="6">
+        <f>0.58*B552</f>
+        <v>189.66</v>
+      </c>
+    </row>
+    <row r="555" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A555" s="11" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="556" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A556" s="43" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="558" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A558" s="11" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="559" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A559" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="561" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A561" s="11" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="564" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A564" s="42" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="565" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A565" s="43" t="s">
+        <v>117</v>
+      </c>
+      <c r="B565" s="6">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="566" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A566"/>
+      <c r="B566" s="6">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="567" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A567" s="42" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="568" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A568" s="40" t="s">
+        <v>463</v>
+      </c>
+      <c r="B568" s="6">
+        <f>1.1</f>
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="569" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A569" s="42" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="570" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A570" s="40" t="s">
+        <v>465</v>
+      </c>
+      <c r="B570" s="6">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="571" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A571" s="42" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="572" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A572" s="43" t="s">
+        <v>117</v>
+      </c>
+      <c r="B572" s="6">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="573" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A573" s="43" t="s">
+        <v>117</v>
+      </c>
+      <c r="B573" s="6">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="574" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A574" s="42" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="575" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A575"/>
+      <c r="B575" s="40">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="576" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A576"/>
+      <c r="B576" s="40">
+        <v>2.35</v>
+      </c>
+    </row>
+    <row r="577" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A577" s="11" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="578" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A578" s="43" t="s">
+        <v>117</v>
+      </c>
+      <c r="B578" s="6">
+        <f>ROUND((B575+B568-1)/B570,3)</f>
+        <v>1.3959999999999999</v>
+      </c>
+    </row>
+    <row r="579" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A579"/>
+      <c r="B579" s="6">
+        <f>ROUND((B576+B568-1)/B570,3)</f>
+        <v>1.0209999999999999</v>
+      </c>
+    </row>
+    <row r="580" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A580" s="11" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="581" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A581" s="11" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="582" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A582"/>
+      <c r="B582" s="6">
+        <f>ROUND(PI()*C510^3/32 - B534*B538*(C510-B538)^2/(2*C510),3)</f>
+        <v>3566.386</v>
+      </c>
+    </row>
+    <row r="583" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A583" s="12" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="584" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A584"/>
+      <c r="B584" s="6">
+        <f>ROUND(PI()*C510^3/16 - B534*B538*(C510-B538)^2/(2*C510),3)</f>
+        <v>7775.6289999999999</v>
+      </c>
+    </row>
+    <row r="586" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A586"/>
+      <c r="B586" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="587" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A587"/>
+      <c r="B587" s="6">
+        <f>ROUND(SQRT(B493^2+B494^2)/B582,3)</f>
+        <v>10.016999999999999</v>
+      </c>
+    </row>
+    <row r="589" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A589"/>
+      <c r="B589" s="6">
+        <f>ROUND(B55/(2*B584),3)</f>
+        <v>1.8440000000000001</v>
+      </c>
+    </row>
+    <row r="592" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A592"/>
+      <c r="B592" s="6">
+        <f>ROUND(B552/(B578*B587+B565*B586),3)</f>
+        <v>23.384</v>
+      </c>
+    </row>
+    <row r="593" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A593"/>
+      <c r="B593" s="6">
+        <f>ROUND(B554/(B579*B589+B566*B589),3)</f>
+        <v>96.034000000000006</v>
+      </c>
+    </row>
+    <row r="595" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A595"/>
+      <c r="B595" s="6">
+        <f>B592*B593/SQRT(B592^2+B593^2)</f>
+        <v>22.720150033294086</v>
+      </c>
+      <c r="C595" s="6" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="597" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A597" s="4" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="598" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A598"/>
+    </row>
+    <row r="601" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A601"/>
+      <c r="B601" s="6">
+        <f>ROUND(SQRT(B493^2+B494^2)/(0.1*C510^3),3)</f>
+        <v>8.3320000000000007</v>
+      </c>
+    </row>
+    <row r="602" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A602"/>
+      <c r="B602" s="6">
+        <f>ROUND(B55/(0.2*C510^3),3)</f>
+        <v>3.3450000000000002</v>
+      </c>
+    </row>
+    <row r="603" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A603"/>
+      <c r="B603" s="6">
+        <f>0.8*E448</f>
+        <v>360</v>
+      </c>
+    </row>
+    <row r="604" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A604"/>
+      <c r="B604" s="6">
+        <f>ROUND(SQRT(B601^2+3*B602^2),3)</f>
+        <v>10.148</v>
+      </c>
+      <c r="C604" s="6" t="s">
+        <v>374</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
done excel tính toán thiết kế và chọn ổ lăn cho trục I
</commit_message>
<xml_diff>
--- a/tínhtoans.xlsx
+++ b/tínhtoans.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Đồ án tkm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BAF4F55-B09D-4DC2-BB1F-59487031ED5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB439C15-D711-4261-A53D-FC2958B3D904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{75337E03-C337-4BFE-A279-78895F300CE2}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{75337E03-C337-4BFE-A279-78895F300CE2}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_Toc233408285" localSheetId="0">Sheet1!$A$28</definedName>
+    <definedName name="_Toc233408285" localSheetId="1">Sheet1!$A$28</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -71,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="474">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="542">
   <si>
     <t>Bánh răng trụ răng thẳng</t>
   </si>
@@ -1346,9 +1347,6 @@
     <t>F_t</t>
   </si>
   <si>
-    <t>f_kn</t>
-  </si>
-  <si>
     <t>FxB</t>
   </si>
   <si>
@@ -1496,9 +1494,6 @@
     <t>hệ số kích thước kể đến ảnh hưởng của kích thước tiết diện trục đến giới hạn mỏi</t>
   </si>
   <si>
-    <t>hệ số tập trung ứng suất thực tê khi uốn và khi xoắn, trị số của chúng phụ thuộc vào loại yếu tố gây tập trung ứng suất</t>
-  </si>
-  <si>
     <t>Hệ số</t>
   </si>
   <si>
@@ -1515,13 +1510,223 @@
   </si>
   <si>
     <t>4.2.10. Tính kiểm nghiệm trục về độ bền tĩnh</t>
+  </si>
+  <si>
+    <t>4.3. Chọn và kiểm nghiệm ổ lăn cho trục I</t>
+  </si>
+  <si>
+    <t>4.3.1. Chọn ô lăn</t>
+  </si>
+  <si>
+    <t>Lực hướng tâm tác dụng lên ổ lăn</t>
+  </si>
+  <si>
+    <t>F_r0</t>
+  </si>
+  <si>
+    <t>F_r1</t>
+  </si>
+  <si>
+    <t>Chọn ổ bi đỡ 1 dãy</t>
+  </si>
+  <si>
+    <t>d10 = d11</t>
+  </si>
+  <si>
+    <t>Kí hiệu ổ</t>
+  </si>
+  <si>
+    <t>Đường kính bi</t>
+  </si>
+  <si>
+    <t>d (mm)</t>
+  </si>
+  <si>
+    <t>D (mm)</t>
+  </si>
+  <si>
+    <t>r (mm)</t>
+  </si>
+  <si>
+    <t>C (kN)</t>
+  </si>
+  <si>
+    <t>C_o (kN)</t>
+  </si>
+  <si>
+    <t>4.3.2. Kiểm nghiệm khả năng chịu tải động</t>
+  </si>
+  <si>
+    <t>a) Kiểm nghiệm tại tiết diện lắp bánh răng</t>
+  </si>
+  <si>
+    <t>b) Kiểm nghiệm tại tiết diện lắp khớp nối</t>
+  </si>
+  <si>
+    <t>W1</t>
+  </si>
+  <si>
+    <t>W_o1</t>
+  </si>
+  <si>
+    <t>Không cần tăng bền</t>
+  </si>
+  <si>
+    <t>Bảng 10.10 tr 198</t>
+  </si>
+  <si>
+    <t>Bảng 10.12 tr 199</t>
+  </si>
+  <si>
+    <t>Bảng 10.11 tr 198</t>
+  </si>
+  <si>
+    <t>hệ số tập trung ứng suất thực tê khi uốn và khi xoắn, đối với trục có rãnh then</t>
+  </si>
+  <si>
+    <t>nội suy</t>
+  </si>
+  <si>
+    <t>F_kn</t>
+  </si>
+  <si>
+    <t>Mj</t>
+  </si>
+  <si>
+    <t>infinity</t>
+  </si>
+  <si>
+    <t>c) Kiểm nghiệm tại tiết diện lắp ổ lăn</t>
+  </si>
+  <si>
+    <t>W2</t>
+  </si>
+  <si>
+    <t>W_o2</t>
+  </si>
+  <si>
+    <t>Sự tập trung ứng suất tại ổ lăn là lắp ghép có độ dôi</t>
+  </si>
+  <si>
+    <t>hệ số tập trung ứng suất thực tê khi uốn và khi xoắn, đối với bề mặt trục lắp có độ dôi</t>
+  </si>
+  <si>
+    <t>Tải trọng động quy ước</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Hệ số tải trọng hướng tâm</t>
+  </si>
+  <si>
+    <t>Hệ số tải trọng dọc trục</t>
+  </si>
+  <si>
+    <t>Hệ số kể đến vòng nào quay, hệ vòng trong quay thì</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>Hệ số kể đến ảnh hưởng của nhiệt độ</t>
+  </si>
+  <si>
+    <t>k_t</t>
+  </si>
+  <si>
+    <t>Hệ số kể đến đặc tính tải trọng, va đập vừa và rung động, quá tải ngắn hạn</t>
+  </si>
+  <si>
+    <t>k_đ</t>
+  </si>
+  <si>
+    <t>Fa</t>
+  </si>
+  <si>
+    <t>Q0</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>Tiến hành kiểm nghiệm với Q lớn hơn</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>Tuổi thọ của ô tính bằng số vòng quay</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>triệu vòng</t>
+  </si>
+  <si>
+    <t>Kiểm tra</t>
+  </si>
+  <si>
+    <t>Cd</t>
+  </si>
+  <si>
+    <t>đối với ổ bi</t>
+  </si>
+  <si>
+    <t>&lt; 17.6 kN</t>
+  </si>
+  <si>
+    <t>thỏa mãn khả năng tải động</t>
+  </si>
+  <si>
+    <t>4.3.3. Kiểm nghiệm khả năng chịu tải tĩnh</t>
+  </si>
+  <si>
+    <t>Khả năng tải tĩnh nhằm đề phòng biến dạng dư, theo điều kiện</t>
+  </si>
+  <si>
+    <t>Qt: Tải trọng tĩnh quy ước</t>
+  </si>
+  <si>
+    <t>Co: Khả năng tải tĩnh</t>
+  </si>
+  <si>
+    <t>Đối với ổ bi đỡ</t>
+  </si>
+  <si>
+    <t>Qt = Fr</t>
+  </si>
+  <si>
+    <t>Qt0</t>
+  </si>
+  <si>
+    <t>Qt1</t>
+  </si>
+  <si>
+    <t>Tiến hành kiểm nghiệm với Qt lớn hơn</t>
+  </si>
+  <si>
+    <t>Qt</t>
+  </si>
+  <si>
+    <t>&lt; C0 = 11600 N</t>
+  </si>
+  <si>
+    <t>4.4. Thiết kế trục II</t>
+  </si>
+  <si>
+    <t>4.4.1. Chọn vật liệu thiết kế truc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1647,6 +1852,13 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="4" tint="0.39997558519241921"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1668,7 +1880,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -1743,12 +1955,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1828,19 +2053,40 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4879,9 +5125,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1078746</xdr:colOff>
+      <xdr:colOff>1086366</xdr:colOff>
       <xdr:row>516</xdr:row>
-      <xdr:rowOff>81999</xdr:rowOff>
+      <xdr:rowOff>91524</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5207,9 +5453,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>2484335</xdr:colOff>
+      <xdr:colOff>2495765</xdr:colOff>
       <xdr:row>549</xdr:row>
-      <xdr:rowOff>83858</xdr:rowOff>
+      <xdr:rowOff>95288</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5322,9 +5568,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>5913306</xdr:colOff>
+      <xdr:colOff>5924736</xdr:colOff>
       <xdr:row>549</xdr:row>
-      <xdr:rowOff>83913</xdr:rowOff>
+      <xdr:rowOff>95343</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5581,7 +5827,7 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>3063505</xdr:colOff>
       <xdr:row>557</xdr:row>
-      <xdr:rowOff>45758</xdr:rowOff>
+      <xdr:rowOff>57188</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5623,7 +5869,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>2446232</xdr:colOff>
+      <xdr:colOff>2457662</xdr:colOff>
       <xdr:row>559</xdr:row>
       <xdr:rowOff>114325</xdr:rowOff>
     </xdr:to>
@@ -5668,8 +5914,8 @@
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>2453853</xdr:colOff>
-      <xdr:row>562</xdr:row>
-      <xdr:rowOff>167670</xdr:rowOff>
+      <xdr:row>563</xdr:row>
+      <xdr:rowOff>30</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5848,13 +6094,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>571</xdr:row>
+      <xdr:row>572</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>160020</xdr:colOff>
-      <xdr:row>571</xdr:row>
+      <xdr:row>572</xdr:row>
       <xdr:rowOff>205740</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -5919,14 +6165,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>572</xdr:row>
+      <xdr:row>573</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>137160</xdr:colOff>
-      <xdr:row>572</xdr:row>
-      <xdr:rowOff>205740</xdr:rowOff>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>574</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5966,8 +6212,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="0" y="101330760"/>
-          <a:ext cx="137160" cy="205740"/>
+          <a:off x="0" y="99469575"/>
+          <a:ext cx="133350" cy="209550"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5990,13 +6236,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>574</xdr:row>
+      <xdr:row>575</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>464820</xdr:colOff>
-      <xdr:row>575</xdr:row>
+      <xdr:row>576</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6061,13 +6307,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>575</xdr:row>
+      <xdr:row>576</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>388620</xdr:colOff>
-      <xdr:row>576</xdr:row>
+      <xdr:row>577</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6132,13 +6378,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>577</xdr:row>
+      <xdr:row>578</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>312420</xdr:colOff>
-      <xdr:row>578</xdr:row>
+      <xdr:row>579</xdr:row>
       <xdr:rowOff>15240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6203,13 +6449,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>578</xdr:row>
+      <xdr:row>579</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>297180</xdr:colOff>
-      <xdr:row>579</xdr:row>
+      <xdr:row>580</xdr:row>
       <xdr:rowOff>53340</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6274,14 +6520,14 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>129540</xdr:colOff>
-      <xdr:row>577</xdr:row>
+      <xdr:row>578</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2240463</xdr:colOff>
-      <xdr:row>579</xdr:row>
-      <xdr:rowOff>45758</xdr:rowOff>
+      <xdr:colOff>2230938</xdr:colOff>
+      <xdr:row>580</xdr:row>
+      <xdr:rowOff>57188</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6318,14 +6564,14 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>15240</xdr:colOff>
-      <xdr:row>580</xdr:row>
+      <xdr:row>581</xdr:row>
       <xdr:rowOff>15240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>960475</xdr:colOff>
-      <xdr:row>582</xdr:row>
-      <xdr:rowOff>99098</xdr:rowOff>
+      <xdr:colOff>971905</xdr:colOff>
+      <xdr:row>583</xdr:row>
+      <xdr:rowOff>91478</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6362,13 +6608,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>581</xdr:row>
+      <xdr:row>582</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>205740</xdr:colOff>
-      <xdr:row>582</xdr:row>
+      <xdr:row>583</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6433,13 +6679,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>583</xdr:row>
+      <xdr:row>584</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>274320</xdr:colOff>
-      <xdr:row>584</xdr:row>
+      <xdr:row>585</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6504,13 +6750,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>585</xdr:row>
+      <xdr:row>586</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>464820</xdr:colOff>
-      <xdr:row>586</xdr:row>
+      <xdr:row>587</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6575,13 +6821,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>586</xdr:row>
+      <xdr:row>587</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>845820</xdr:colOff>
-      <xdr:row>587</xdr:row>
+      <xdr:row>588</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6646,13 +6892,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>588</xdr:row>
+      <xdr:row>589</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>1501140</xdr:colOff>
-      <xdr:row>590</xdr:row>
+      <xdr:row>591</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6717,13 +6963,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>591</xdr:row>
+      <xdr:row>592</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>220980</xdr:colOff>
-      <xdr:row>592</xdr:row>
+      <xdr:row>593</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6788,13 +7034,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>592</xdr:row>
+      <xdr:row>593</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>205740</xdr:colOff>
-      <xdr:row>593</xdr:row>
+      <xdr:row>594</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6859,13 +7105,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>594</xdr:row>
+      <xdr:row>595</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>144780</xdr:colOff>
-      <xdr:row>595</xdr:row>
+      <xdr:row>596</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6930,13 +7176,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>597</xdr:row>
+      <xdr:row>656</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>1600200</xdr:colOff>
-      <xdr:row>598</xdr:row>
+      <xdr:row>657</xdr:row>
       <xdr:rowOff>83820</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -7001,13 +7247,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>600</xdr:row>
+      <xdr:row>659</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>99060</xdr:colOff>
-      <xdr:row>601</xdr:row>
+      <xdr:row>660</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -7071,15 +7317,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>3947160</xdr:colOff>
-      <xdr:row>593</xdr:row>
-      <xdr:rowOff>99060</xdr:rowOff>
+      <xdr:colOff>4446270</xdr:colOff>
+      <xdr:row>657</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>5471292</xdr:colOff>
-      <xdr:row>599</xdr:row>
-      <xdr:rowOff>7703</xdr:rowOff>
+      <xdr:colOff>5960877</xdr:colOff>
+      <xdr:row>662</xdr:row>
+      <xdr:rowOff>133433</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7102,8 +7348,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3947160" y="105186480"/>
-          <a:ext cx="1524132" cy="960203"/>
+          <a:off x="4446270" y="104205405"/>
+          <a:ext cx="1518417" cy="960203"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7116,13 +7362,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>601</xdr:row>
+      <xdr:row>660</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>76200</xdr:colOff>
-      <xdr:row>602</xdr:row>
+      <xdr:row>661</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -7187,13 +7433,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>602</xdr:row>
+      <xdr:row>661</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>609600</xdr:colOff>
-      <xdr:row>603</xdr:row>
+      <xdr:row>662</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -7258,13 +7504,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>603</xdr:row>
+      <xdr:row>662</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>205740</xdr:colOff>
-      <xdr:row>604</xdr:row>
+      <xdr:row>663</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -7307,6 +7553,1967 @@
         <a:xfrm>
           <a:off x="0" y="106840020"/>
           <a:ext cx="205740" cy="205740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>599</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>601</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="58" name="Picture 57">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C39A552-44DB-20F3-2358-CCEED2DD4893}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId82">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="103889175"/>
+          <a:ext cx="257175" cy="314325"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>600</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
+      <xdr:row>602</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="60" name="Picture 59">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C3A7316C-7AA0-E5A7-E715-6E6E8326BF07}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId83">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="28575" y="104041575"/>
+          <a:ext cx="219075" cy="314325"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>600</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2000250</xdr:colOff>
+      <xdr:row>603</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="62" name="Picture 61">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CBDC0C3A-8491-F5DD-7F89-10D7469FF3E3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId84">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="38100" y="104127300"/>
+          <a:ext cx="1962150" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>607</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>160020</xdr:colOff>
+      <xdr:row>607</xdr:row>
+      <xdr:rowOff>205740</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="57" name="Picture 56">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{630834A6-59F9-409B-8D3F-251E260074D9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId60">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="99260025"/>
+          <a:ext cx="161925" cy="209550"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>608</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>137160</xdr:colOff>
+      <xdr:row>608</xdr:row>
+      <xdr:rowOff>205740</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="73" name="Picture 72">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DED28150-A408-40E5-9DA0-1A3B97B9623C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId61">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="99469575"/>
+          <a:ext cx="133350" cy="209550"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>609</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>611</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="81" name="Picture 80">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E4EE418E-402E-3AA7-5071-54CE1B587B07}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId85">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="66675" y="105717975"/>
+          <a:ext cx="190500" cy="295275"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>610</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
+      <xdr:row>612</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="82" name="Picture 81">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BF802D52-8E44-8D79-E8E6-F72224B14217}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId86">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="76200" y="105908475"/>
+          <a:ext cx="171450" cy="295275"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>614</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>312420</xdr:colOff>
+      <xdr:row>615</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="85" name="Picture 84">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{210E1D78-CE7F-468E-AB5F-8A19EEA24791}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId64">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="100364925"/>
+          <a:ext cx="314325" cy="228600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>615</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>297180</xdr:colOff>
+      <xdr:row>616</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="86" name="Picture 85">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87C117E8-9BCD-49CD-BF60-561EAB9FFD15}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId65">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="100574475"/>
+          <a:ext cx="295275" cy="228600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>620</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>622</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="103" name="Picture 102">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5149F28C-7DC0-8250-78BF-98B775A8C66F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId87">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="107794425"/>
+          <a:ext cx="133350" cy="314325"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>618</xdr:row>
+      <xdr:rowOff>1905</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>278130</xdr:colOff>
+      <xdr:row>619</xdr:row>
+      <xdr:rowOff>140970</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="105" name="Picture 104">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1AB339FD-0760-E812-432F-BD6D1DEE69ED}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId88">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="68580" y="107377230"/>
+          <a:ext cx="209550" cy="310515"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>616</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
+      <xdr:row>618</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="106" name="Picture 105">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{17045DA6-1C21-E985-5BF8-40ADBB44114C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId89">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="57150" y="107156250"/>
+          <a:ext cx="219075" cy="314325"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>627</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>629</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="119" name="Picture 118">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D2FE9CE5-469A-4951-8227-34B970DB9588}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId82">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="104056815"/>
+          <a:ext cx="255270" cy="316230"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>628</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
+      <xdr:row>630</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="120" name="Picture 119">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B5FE9045-AF53-474F-9C08-C6C84CB27CB2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId83">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="26670" y="104213025"/>
+          <a:ext cx="217170" cy="316230"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>628</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2000250</xdr:colOff>
+      <xdr:row>631</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="121" name="Picture 120">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5812A5D4-8D7C-4BC3-88D5-CF480D5ACB30}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId84">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="38100" y="104300655"/>
+          <a:ext cx="1958340" cy="518160"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>642</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>312420</xdr:colOff>
+      <xdr:row>643</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="126" name="Picture 125">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{212470DF-AA9B-41E3-A9E6-A15F8C349F90}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId64">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="106651425"/>
+          <a:ext cx="314325" cy="228600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>643</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>297180</xdr:colOff>
+      <xdr:row>644</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="127" name="Picture 126">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{28D7E457-E7B6-4842-BDF3-DE7BD01FA4FB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId65">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="106860975"/>
+          <a:ext cx="295275" cy="228600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>648</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>650</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="128" name="Picture 127">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CC95C717-9BF0-48DE-8850-D300739F509F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId87">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="107794425"/>
+          <a:ext cx="129540" cy="316230"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>645</xdr:row>
+      <xdr:rowOff>87630</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>224790</xdr:colOff>
+      <xdr:row>647</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="129" name="Picture 128">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8DB4E8EC-2D2E-45A3-BAE8-67DD9C9925B8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId88">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="9525" y="112206405"/>
+          <a:ext cx="215265" cy="308610"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>24765</xdr:colOff>
+      <xdr:row>644</xdr:row>
+      <xdr:rowOff>87630</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>249555</xdr:colOff>
+      <xdr:row>646</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="130" name="Picture 129">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12EA79B6-7C8D-43E2-9712-F7E70F3AA3FE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId89">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="24765" y="112034955"/>
+          <a:ext cx="224790" cy="308610"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>635</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>160020</xdr:colOff>
+      <xdr:row>635</xdr:row>
+      <xdr:rowOff>205740</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="131" name="Picture 130">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{868841ED-B672-4422-9E3D-7F79FF8B2609}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId60">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="99260025"/>
+          <a:ext cx="161925" cy="209550"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>636</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>637</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="132" name="Picture 131">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{372F4B75-2224-45A0-81E5-30BD5F3026EC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId61">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="99469575"/>
+          <a:ext cx="129540" cy="209550"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>638</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>464820</xdr:colOff>
+      <xdr:row>639</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="133" name="Picture 132">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{931B66F4-D7F4-4A1A-A0C4-EA4443B828E8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId62">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="99850575"/>
+          <a:ext cx="466725" cy="200025"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>639</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>388620</xdr:colOff>
+      <xdr:row>640</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="134" name="Picture 133">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D84D2FAD-50DB-4AA1-A115-BC2B966AF265}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId63">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="100022025"/>
+          <a:ext cx="390525" cy="200025"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2314575</xdr:colOff>
+      <xdr:row>587</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>472751</xdr:colOff>
+      <xdr:row>596</xdr:row>
+      <xdr:rowOff>131</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="135" name="Picture 134">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BFBD0EE0-84B9-05DD-AF0E-13363EE7F7F9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId90"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12277725" y="101984175"/>
+          <a:ext cx="3587426" cy="1505081"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>678</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1028700</xdr:colOff>
+      <xdr:row>679</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="136" name="Picture 135">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0DEA4A44-2BBB-1870-E539-07249D0B4160}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId91">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="266700" y="117814725"/>
+          <a:ext cx="762000" cy="228600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>680</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1581150</xdr:colOff>
+      <xdr:row>682</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="137" name="Picture 136">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CEFFD8C0-F4F8-8F5B-DC1F-1B82AB1182F1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId92">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="118310025"/>
+          <a:ext cx="1581150" cy="200025"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>704</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>548640</xdr:colOff>
+      <xdr:row>705</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="138" name="Picture 137">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C1D17460-97DC-203F-5DDB-DDD09C7D3BC4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId93">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="124792740"/>
+          <a:ext cx="548640" cy="205740"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7713,11 +9920,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAB77A47-A7BE-4D4A-B9B2-7BD4BBB02747}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77F27C94-6297-45CB-8ED2-81D711DA05BE}">
-  <dimension ref="A1:J604"/>
+  <dimension ref="A1:J724"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="90.8984375" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="98.59765625" style="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32.09765625" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="41.296875" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="30.09765625" style="6" bestFit="1" customWidth="1"/>
@@ -8441,7 +10657,7 @@
       <c r="B90" s="6">
         <v>1.25</v>
       </c>
-      <c r="F90" s="39" t="s">
+      <c r="F90" s="43" t="s">
         <v>118</v>
       </c>
     </row>
@@ -8449,7 +10665,7 @@
       <c r="A91" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="F91" s="39"/>
+      <c r="F91" s="43"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
@@ -8461,13 +10677,13 @@
       <c r="C92" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="F92" s="39"/>
+      <c r="F92" s="43"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="F93" s="39"/>
+      <c r="F93" s="43"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
@@ -8479,13 +10695,13 @@
       <c r="C94" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="F94" s="39"/>
+      <c r="F94" s="43"/>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="F95" s="39"/>
+      <c r="F95" s="43"/>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
@@ -8497,13 +10713,13 @@
       <c r="C96" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="F96" s="39"/>
+      <c r="F96" s="43"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="F97" s="39"/>
+      <c r="F97" s="43"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
@@ -8515,13 +10731,13 @@
       <c r="C98" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="F98" s="39"/>
+      <c r="F98" s="43"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="F99" s="39"/>
+      <c r="F99" s="43"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
@@ -8533,7 +10749,7 @@
       <c r="C100" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="F100" s="39"/>
+      <c r="F100" s="43"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="12" t="s">
@@ -9446,13 +11662,13 @@
       <c r="A227" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="C227" s="39" t="s">
+      <c r="C227" s="43" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228"/>
-      <c r="C228" s="39"/>
+      <c r="C228" s="43"/>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
@@ -9462,7 +11678,7 @@
         <f>2*B225+70</f>
         <v>570</v>
       </c>
-      <c r="C229" s="39"/>
+      <c r="C229" s="43"/>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
@@ -9472,17 +11688,17 @@
         <f>2*B226+70</f>
         <v>510</v>
       </c>
-      <c r="C230" s="39"/>
+      <c r="C230" s="43"/>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" s="11" t="s">
         <v>256</v>
       </c>
-      <c r="C231" s="39"/>
+      <c r="C231" s="43"/>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232"/>
-      <c r="C232" s="39"/>
+      <c r="C232" s="43"/>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
@@ -9492,7 +11708,7 @@
         <f>1.8*B225</f>
         <v>450</v>
       </c>
-      <c r="C233" s="39"/>
+      <c r="C233" s="43"/>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
@@ -9502,16 +11718,16 @@
         <f>1.8*B226</f>
         <v>396</v>
       </c>
-      <c r="C234" s="39"/>
+      <c r="C234" s="43"/>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C235" s="39"/>
+      <c r="C235" s="43"/>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="C236" s="39"/>
+      <c r="C236" s="43"/>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
@@ -9520,7 +11736,7 @@
       <c r="B237" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C237" s="39"/>
+      <c r="C237" s="43"/>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
@@ -9529,7 +11745,7 @@
       <c r="B238" s="6">
         <v>1.75</v>
       </c>
-      <c r="C238" s="39"/>
+      <c r="C238" s="43"/>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" s="12" t="s">
@@ -9560,7 +11776,7 @@
       <c r="B244" s="6">
         <v>6</v>
       </c>
-      <c r="C244" s="39" t="s">
+      <c r="C244" s="43" t="s">
         <v>244</v>
       </c>
     </row>
@@ -9571,7 +11787,7 @@
       <c r="B245" s="6">
         <v>6</v>
       </c>
-      <c r="C245" s="39"/>
+      <c r="C245" s="43"/>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" s="12" t="s">
@@ -9837,7 +12053,7 @@
         <f>0.01*B286</f>
         <v>1.4000000000000001</v>
       </c>
-      <c r="C290" s="39">
+      <c r="C290" s="43">
         <v>2</v>
       </c>
     </row>
@@ -9846,7 +12062,7 @@
         <f>0.02*B286</f>
         <v>2.8000000000000003</v>
       </c>
-      <c r="C291" s="39"/>
+      <c r="C291" s="43"/>
       <c r="D291" s="6" t="s">
         <v>267</v>
       </c>
@@ -10742,28 +12958,28 @@
       </c>
     </row>
     <row r="446" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A446" s="37" t="s">
+      <c r="A446" s="44" t="s">
         <v>377</v>
       </c>
-      <c r="B446" s="37" t="s">
+      <c r="B446" s="44" t="s">
         <v>187</v>
       </c>
-      <c r="C446" s="37" t="s">
+      <c r="C446" s="44" t="s">
         <v>378</v>
       </c>
-      <c r="D446" s="37" t="e" vm="1">
+      <c r="D446" s="44" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="E446" s="37" t="e" vm="2">
+      <c r="E446" s="44" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="447" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A447" s="38"/>
-      <c r="B447" s="38"/>
-      <c r="C447" s="38"/>
-      <c r="D447" s="38"/>
-      <c r="E447" s="38"/>
+      <c r="A447" s="45"/>
+      <c r="B447" s="45"/>
+      <c r="C447" s="45"/>
+      <c r="D447" s="45"/>
+      <c r="E447" s="45"/>
     </row>
     <row r="448" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A448" s="34" t="s">
@@ -11041,22 +13257,22 @@
         <v>416</v>
       </c>
       <c r="B486" s="6">
-        <f>ROUND(2*B55/B436,3)</f>
-        <v>637.40099999999995</v>
+        <f>ROUND(2*B53/B436,3)</f>
+        <v>650.61900000000003</v>
       </c>
     </row>
     <row r="487" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A487" t="s">
-        <v>417</v>
+        <v>497</v>
       </c>
       <c r="B487" s="6">
         <f>0.2*B486</f>
-        <v>127.4802</v>
+        <v>130.12380000000002</v>
       </c>
     </row>
     <row r="488" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A488" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B488" s="6">
         <v>483.37619999999998</v>
@@ -11064,7 +13280,7 @@
     </row>
     <row r="489" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A489" s="6" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B489" s="6">
         <f>B454-B491</f>
@@ -11073,7 +13289,7 @@
     </row>
     <row r="490" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A490" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B490" s="6">
         <v>781.01499999999999</v>
@@ -11081,7 +13297,7 @@
     </row>
     <row r="491" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A491" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B491" s="6">
         <f>253.78</f>
@@ -11090,12 +13306,12 @@
     </row>
     <row r="492" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A492" s="12" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="493" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A493" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B493" s="6">
         <f>B490*B481</f>
@@ -11103,35 +13319,35 @@
       </c>
       <c r="C493" s="6">
         <f>B487*(B477+B481)+B488*B481</f>
-        <v>33711.1446</v>
-      </c>
-      <c r="D493" s="39" t="s">
-        <v>432</v>
+        <v>33974.182800000002</v>
+      </c>
+      <c r="D493" s="43" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="494" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A494" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B494" s="6">
         <f>B491*B481</f>
         <v>11039.43</v>
       </c>
-      <c r="D494" s="39"/>
+      <c r="D494" s="43"/>
     </row>
     <row r="496" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A496" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="497" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A497" s="12" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="498" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A498" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B498" s="6">
         <f>SQRT(0+0+0.75*B55^2)</f>
@@ -11140,26 +13356,26 @@
     </row>
     <row r="499" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A499" s="12" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="500" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A500" s="6" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B500" s="6">
         <f>SQRT(0+(B487*B477)^2+0.75*B55^2)</f>
-        <v>25845.722185627495</v>
+        <v>25887.004024469807</v>
       </c>
     </row>
     <row r="501" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A501" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="502" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A502" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B502" s="6">
         <f>SQRT(B493^2+B494^2+0.75*B55^2)</f>
@@ -11168,7 +13384,7 @@
     </row>
     <row r="503" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A503" s="36" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="504" spans="1:3" x14ac:dyDescent="0.25">
@@ -11180,7 +13396,7 @@
     </row>
     <row r="505" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A505" s="11" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="506" spans="1:3" x14ac:dyDescent="0.25">
@@ -11197,7 +13413,7 @@
     </row>
     <row r="507" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A507" s="12" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="508" spans="1:3" x14ac:dyDescent="0.25">
@@ -11206,7 +13422,7 @@
       </c>
       <c r="B508" s="6">
         <f t="shared" ref="B508:B510" si="0">(B500/(0.1*B506))^(1/3)</f>
-        <v>25.386014763892227</v>
+        <v>25.39952343272725</v>
       </c>
       <c r="C508" s="6">
         <v>30</v>
@@ -11214,16 +13430,16 @@
     </row>
     <row r="509" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A509" s="12" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="510" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A510" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B510" s="6">
         <f t="shared" si="0"/>
-        <v>25.782952457296389</v>
+        <v>25.778380781876219</v>
       </c>
       <c r="C510" s="6">
         <v>35</v>
@@ -11231,21 +13447,21 @@
     </row>
     <row r="512" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A512" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="514" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A514" s="4" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="515" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A515" s="42" t="s">
+      <c r="A515" s="12" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="516" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A516" s="41" t="s">
+      <c r="A516" s="37" t="s">
         <v>390</v>
       </c>
       <c r="B516" s="6">
@@ -11254,12 +13470,12 @@
     </row>
     <row r="517" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A517" s="11" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="518" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A518" s="6" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B518" s="6">
         <v>6</v>
@@ -11267,12 +13483,12 @@
     </row>
     <row r="519" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A519" s="11" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="520" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A520" t="s">
         <v>442</v>
-      </c>
-    </row>
-    <row r="520" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A520" s="40" t="s">
-        <v>443</v>
       </c>
       <c r="B520" s="6">
         <v>6</v>
@@ -11280,38 +13496,38 @@
     </row>
     <row r="521" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A521" s="11" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="522" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A522" s="40" t="s">
-        <v>444</v>
+      <c r="A522" t="s">
+        <v>443</v>
       </c>
       <c r="B522" s="6">
         <v>3.5</v>
       </c>
     </row>
     <row r="523" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A523" s="42" t="s">
-        <v>445</v>
+      <c r="A523" s="12" t="s">
+        <v>444</v>
       </c>
     </row>
     <row r="524" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A524" s="40" t="s">
-        <v>447</v>
+      <c r="A524" t="s">
+        <v>446</v>
       </c>
       <c r="B524" s="6">
         <v>2.8</v>
       </c>
     </row>
     <row r="525" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A525" s="42" t="s">
+      <c r="A525" s="12" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="526" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A526" t="s">
         <v>448</v>
-      </c>
-    </row>
-    <row r="526" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A526" s="40" t="s">
-        <v>449</v>
       </c>
       <c r="B526" s="6">
         <f>0.8*B467</f>
@@ -11335,7 +13551,7 @@
         <v>38.244053333333333</v>
       </c>
       <c r="C528" s="6" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="529" spans="1:5" x14ac:dyDescent="0.25">
@@ -11345,17 +13561,17 @@
         <v>15.935022222222223</v>
       </c>
       <c r="C529" s="6" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="530" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A530" s="4" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="531" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A531" s="11" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="532" spans="1:5" x14ac:dyDescent="0.25">
@@ -11367,13 +13583,13 @@
       </c>
     </row>
     <row r="533" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A533" s="42" t="s">
-        <v>440</v>
+      <c r="A533" s="12" t="s">
+        <v>439</v>
       </c>
     </row>
     <row r="534" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A534" s="6" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B534" s="6">
         <v>10</v>
@@ -11381,51 +13597,51 @@
     </row>
     <row r="535" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A535" s="11" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="536" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A536" t="s">
         <v>442</v>
-      </c>
-    </row>
-    <row r="536" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A536" s="40" t="s">
-        <v>443</v>
       </c>
       <c r="B536" s="6">
         <v>8</v>
       </c>
     </row>
     <row r="537" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A537" s="42" t="s">
-        <v>446</v>
+      <c r="A537" s="12" t="s">
+        <v>445</v>
       </c>
     </row>
     <row r="538" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A538" s="40" t="s">
-        <v>444</v>
+      <c r="A538" t="s">
+        <v>443</v>
       </c>
       <c r="B538" s="6">
         <v>5</v>
       </c>
     </row>
     <row r="539" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A539" s="42" t="s">
-        <v>445</v>
+      <c r="A539" s="12" t="s">
+        <v>444</v>
       </c>
     </row>
     <row r="540" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A540" s="40" t="s">
-        <v>447</v>
+      <c r="A540" t="s">
+        <v>446</v>
       </c>
       <c r="B540" s="6">
         <v>3.3</v>
       </c>
     </row>
     <row r="541" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A541" s="42" t="s">
+      <c r="A541" s="12" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="542" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A542" t="s">
         <v>448</v>
-      </c>
-    </row>
-    <row r="542" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A542" s="40" t="s">
-        <v>449</v>
       </c>
       <c r="B542" s="6">
         <f>0.8*B465</f>
@@ -11464,17 +13680,17 @@
     </row>
     <row r="547" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A547" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="551" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A551" s="11" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="552" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A552" s="38" t="s">
         <v>456</v>
-      </c>
-    </row>
-    <row r="552" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A552" s="43" t="s">
-        <v>457</v>
       </c>
       <c r="B552" s="6">
         <f>0.436*D448</f>
@@ -11483,11 +13699,11 @@
     </row>
     <row r="553" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A553" s="11" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="554" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A554" s="43" t="s">
+      <c r="A554" s="38" t="s">
         <v>117</v>
       </c>
       <c r="B554" s="6">
@@ -11497,17 +13713,17 @@
     </row>
     <row r="555" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A555" s="11" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="556" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A556" s="43" t="s">
+      <c r="A556" s="38" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="558" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A558" s="11" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="559" spans="1:3" x14ac:dyDescent="0.25">
@@ -11515,240 +13731,1000 @@
         <v>1</v>
       </c>
     </row>
-    <row r="561" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="561" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A561" s="11" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="564" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A564" s="12" t="s">
         <v>460</v>
       </c>
     </row>
-    <row r="564" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A564" s="42" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="565" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A565" s="43" t="s">
+    <row r="565" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A565" s="38" t="s">
         <v>117</v>
       </c>
       <c r="B565" s="6">
         <v>0.1</v>
       </c>
     </row>
-    <row r="566" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="566" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A566"/>
       <c r="B566" s="6">
         <v>0.05</v>
       </c>
     </row>
-    <row r="567" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A567" s="42" t="s">
+    <row r="567" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A567" s="12" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="568" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A568" t="s">
         <v>462</v>
-      </c>
-    </row>
-    <row r="568" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A568" s="40" t="s">
-        <v>463</v>
       </c>
       <c r="B568" s="6">
         <f>1.1</f>
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="569" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A569" s="42" t="s">
+    <row r="569" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A569" s="12" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="570" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A570" t="s">
         <v>464</v>
       </c>
-    </row>
-    <row r="570" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A570" s="40" t="s">
+      <c r="B570" s="6">
+        <v>1</v>
+      </c>
+      <c r="C570" s="6" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="571" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A571" s="42" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="572" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A572" s="12" t="s">
         <v>465</v>
       </c>
-      <c r="B570" s="6">
-        <v>2.4</v>
-      </c>
-    </row>
-    <row r="571" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A571" s="42" t="s">
+      <c r="B572" s="6" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="573" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A573" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="B573" s="6">
+        <v>0.86499999999999999</v>
+      </c>
+      <c r="C573" s="43" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="574" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A574" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="B574" s="6">
+        <v>0.79500000000000004</v>
+      </c>
+      <c r="C574" s="43"/>
+    </row>
+    <row r="575" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A575" s="12" t="s">
+        <v>504</v>
+      </c>
+      <c r="B575" s="6" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="576" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A576"/>
+      <c r="B576">
+        <v>3.125</v>
+      </c>
+      <c r="C576" s="43" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="577" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A577"/>
+      <c r="B577">
+        <v>2.2749999999999999</v>
+      </c>
+      <c r="C577" s="43"/>
+    </row>
+    <row r="578" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A578" s="11" t="s">
         <v>466</v>
       </c>
     </row>
-    <row r="572" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A572" s="43" t="s">
+    <row r="579" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A579" s="38" t="s">
         <v>117</v>
       </c>
-      <c r="B572" s="6">
-        <v>0.85</v>
-      </c>
-    </row>
-    <row r="573" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A573" s="43" t="s">
-        <v>117</v>
-      </c>
-      <c r="B573" s="6">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="574" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A574" s="42" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="575" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A575"/>
-      <c r="B575" s="40">
-        <v>3.25</v>
-      </c>
-    </row>
-    <row r="576" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A576"/>
-      <c r="B576" s="40">
-        <v>2.35</v>
-      </c>
-    </row>
-    <row r="577" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A577" s="11" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="578" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A578" s="43" t="s">
-        <v>117</v>
-      </c>
-      <c r="B578" s="6">
-        <f>ROUND((B575+B568-1)/B570,3)</f>
-        <v>1.3959999999999999</v>
-      </c>
-    </row>
-    <row r="579" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A579"/>
       <c r="B579" s="6">
         <f>ROUND((B576+B568-1)/B570,3)</f>
-        <v>1.0209999999999999</v>
-      </c>
-    </row>
-    <row r="580" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A580" s="11" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="581" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3.2250000000000001</v>
+      </c>
+    </row>
+    <row r="580" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A580"/>
+      <c r="B580" s="6">
+        <f>ROUND((B577+B568-1)/B570,3)</f>
+        <v>2.375</v>
+      </c>
+    </row>
+    <row r="581" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A581" s="11" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="582" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A582"/>
-      <c r="B582" s="6">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="582" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A582" s="11" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="583" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A583"/>
+      <c r="B583" s="6">
         <f>ROUND(PI()*C510^3/32 - B534*B538*(C510-B538)^2/(2*C510),3)</f>
         <v>3566.386</v>
       </c>
     </row>
-    <row r="583" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A583" s="12" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="584" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A584"/>
-      <c r="B584" s="6">
+    <row r="584" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A584" s="12" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="585" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A585"/>
+      <c r="B585" s="6">
         <f>ROUND(PI()*C510^3/16 - B534*B538*(C510-B538)^2/(2*C510),3)</f>
         <v>7775.6289999999999</v>
       </c>
     </row>
-    <row r="586" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A586"/>
-      <c r="B586" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="587" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="587" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A587"/>
       <c r="B587" s="6">
-        <f>ROUND(SQRT(B493^2+B494^2)/B582,3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="588" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A588"/>
+      <c r="B588" s="6">
+        <f>ROUND(SQRT(B493^2+B494^2)/B583,3)</f>
         <v>10.016999999999999</v>
       </c>
     </row>
-    <row r="589" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A589"/>
-      <c r="B589" s="6">
-        <f>ROUND(B55/(2*B584),3)</f>
+    <row r="590" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A590"/>
+      <c r="B590" s="6">
+        <f>ROUND(B55/(2*B585),3)</f>
         <v>1.8440000000000001</v>
-      </c>
-    </row>
-    <row r="592" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A592"/>
-      <c r="B592" s="6">
-        <f>ROUND(B552/(B578*B587+B565*B586),3)</f>
-        <v>23.384</v>
       </c>
     </row>
     <row r="593" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A593"/>
       <c r="B593" s="6">
-        <f>ROUND(B554/(B579*B589+B566*B589),3)</f>
-        <v>96.034000000000006</v>
-      </c>
-    </row>
-    <row r="595" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A595"/>
-      <c r="B595" s="6">
-        <f>B592*B593/SQRT(B592^2+B593^2)</f>
-        <v>22.720150033294086</v>
-      </c>
-      <c r="C595" s="6" t="s">
-        <v>472</v>
+        <f>ROUND(B552/(B579*B588+B565*B587),3)</f>
+        <v>10.122</v>
+      </c>
+    </row>
+    <row r="594" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A594"/>
+      <c r="B594" s="6">
+        <f>ROUND(B554/(B580*B590+B566*B590),3)</f>
+        <v>42.412999999999997</v>
+      </c>
+    </row>
+    <row r="596" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A596"/>
+      <c r="B596" s="6">
+        <f>B593*B594/SQRT(B593^2+B594^2)</f>
+        <v>9.8455052497783537</v>
+      </c>
+      <c r="C596" s="6" t="s">
+        <v>470</v>
       </c>
     </row>
     <row r="597" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A597" s="4" t="s">
-        <v>473</v>
+        <v>488</v>
       </c>
     </row>
     <row r="598" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A598"/>
+      <c r="A598" s="37" t="s">
+        <v>498</v>
+      </c>
+      <c r="B598" s="6">
+        <f>0</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="599" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A599" s="37" t="s">
+        <v>489</v>
+      </c>
+      <c r="B599" s="6">
+        <f>ROUND(PI()*C506^3/32-B518*B522*(C506-B522)^2/(2*B516),3)</f>
+        <v>642.46699999999998</v>
+      </c>
+    </row>
+    <row r="600" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A600" s="37" t="s">
+        <v>490</v>
+      </c>
+      <c r="B600" s="6">
+        <f>ROUND(PI()*C506^3/16-B518*B522*(C506-B522)^2/(2*B516),3)</f>
+        <v>1427.865</v>
+      </c>
     </row>
     <row r="601" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A601"/>
       <c r="B601" s="6">
-        <f>ROUND(SQRT(B493^2+B494^2)/(0.1*C510^3),3)</f>
-        <v>8.3320000000000007</v>
+        <f>0</f>
+        <v>0</v>
       </c>
     </row>
     <row r="602" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A602"/>
       <c r="B602" s="6">
-        <f>ROUND(B55/(0.2*C510^3),3)</f>
-        <v>3.3450000000000002</v>
+        <f>ROUND(B598/B599,3)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="603" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A603"/>
       <c r="B603" s="6">
+        <f>ROUND(B55/(2*B600),3)</f>
+        <v>10.044</v>
+      </c>
+    </row>
+    <row r="604" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A604" s="4"/>
+    </row>
+    <row r="605" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A605" s="4"/>
+    </row>
+    <row r="606" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A606" s="4"/>
+    </row>
+    <row r="607" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A607" s="12" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="608" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A608" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="B608" s="6">
+        <v>0.92</v>
+      </c>
+    </row>
+    <row r="609" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A609" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="B609" s="6">
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="610" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A610" s="12" t="s">
+        <v>495</v>
+      </c>
+      <c r="B610" s="6" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="611" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A611"/>
+      <c r="B611" s="6">
+        <v>1.9475</v>
+      </c>
+      <c r="C611" s="43" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="612" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A612"/>
+      <c r="B612" s="46">
+        <v>1.7949999999999999</v>
+      </c>
+      <c r="C612" s="43"/>
+    </row>
+    <row r="613" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A613" s="4"/>
+    </row>
+    <row r="614" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A614" s="11" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="615" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A615" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="B615" s="6">
+        <f>ROUND((B611/B608+B568-1)/B570,3)</f>
+        <v>2.2170000000000001</v>
+      </c>
+    </row>
+    <row r="616" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A616"/>
+      <c r="B616" s="6">
+        <f>ROUND((B612/B609+B568-1)/B570,3)</f>
+        <v>2.117</v>
+      </c>
+    </row>
+    <row r="617" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A617" s="4"/>
+    </row>
+    <row r="618" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A618" s="4"/>
+    </row>
+    <row r="619" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A619"/>
+      <c r="B619" s="6" t="e">
+        <f>ROUND(B552/(B615*B602+B565*B601),3)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C619" s="6" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="620" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A620"/>
+      <c r="B620" s="6">
+        <f>ROUND(B554/(B616*B603+B566*B603),3)</f>
+        <v>8.7140000000000004</v>
+      </c>
+    </row>
+    <row r="621" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A621" s="4"/>
+    </row>
+    <row r="622" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A622"/>
+      <c r="B622" s="6">
+        <f>B620</f>
+        <v>8.7140000000000004</v>
+      </c>
+      <c r="C622" s="6" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="623" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A623" s="4"/>
+    </row>
+    <row r="624" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A624" s="4" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="625" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A625" s="4"/>
+    </row>
+    <row r="626" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A626" s="37" t="s">
+        <v>498</v>
+      </c>
+      <c r="B626" s="6">
+        <f>SQRT(7286.9328^2+0^2)</f>
+        <v>7286.9327999999996</v>
+      </c>
+    </row>
+    <row r="627" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A627" s="37" t="s">
+        <v>501</v>
+      </c>
+      <c r="B627" s="6">
+        <f>ROUND(PI()*C508^3/32,3)</f>
+        <v>2650.7190000000001</v>
+      </c>
+    </row>
+    <row r="628" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A628" s="37" t="s">
+        <v>502</v>
+      </c>
+      <c r="B628" s="6">
+        <f>ROUND(PI()*C508^3/16,3)</f>
+        <v>5301.4380000000001</v>
+      </c>
+    </row>
+    <row r="629" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A629"/>
+      <c r="B629" s="6">
+        <f>0</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="630" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A630"/>
+      <c r="B630" s="6">
+        <f>ROUND(B626/B627,3)</f>
+        <v>2.7490000000000001</v>
+      </c>
+    </row>
+    <row r="631" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A631"/>
+      <c r="B631" s="6">
+        <f>ROUND(B55/(2*B628),3)</f>
+        <v>2.7050000000000001</v>
+      </c>
+    </row>
+    <row r="632" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A632" s="4"/>
+    </row>
+    <row r="633" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A633" s="37" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="634" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A634" s="4"/>
+    </row>
+    <row r="635" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A635" s="12" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="636" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A636" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="B636" s="6">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="637" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A637" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="B637" s="6">
+        <v>0.81</v>
+      </c>
+    </row>
+    <row r="638" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A638" s="12" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="639" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A639"/>
+      <c r="B639">
+        <v>3.125</v>
+      </c>
+    </row>
+    <row r="640" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A640"/>
+      <c r="B640">
+        <v>2.2749999999999999</v>
+      </c>
+    </row>
+    <row r="641" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A641" s="4"/>
+    </row>
+    <row r="642" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A642" s="11" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="643" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A643" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="B643" s="6">
+        <f>(B639+B568-1)/B570</f>
+        <v>3.2249999999999996</v>
+      </c>
+    </row>
+    <row r="644" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A644"/>
+      <c r="B644" s="6">
+        <f>(B640+B568-1)/B570</f>
+        <v>2.375</v>
+      </c>
+    </row>
+    <row r="645" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A645" s="4"/>
+    </row>
+    <row r="646" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A646" s="4"/>
+      <c r="B646" s="6">
+        <f>ROUND(B552/(B643*B630+B565*B629),3)</f>
+        <v>36.884</v>
+      </c>
+    </row>
+    <row r="647" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A647"/>
+      <c r="B647" s="6">
+        <f>ROUND(B554/(B566*B631+B644*B631),3)</f>
+        <v>28.913</v>
+      </c>
+    </row>
+    <row r="648" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A648"/>
+    </row>
+    <row r="649" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A649" s="4"/>
+    </row>
+    <row r="650" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A650"/>
+      <c r="B650" s="47">
+        <f>B646*B647/SQRT(B646^2+B647^2)</f>
+        <v>22.754973776977636</v>
+      </c>
+      <c r="C650" s="6" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="651" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A651" s="4"/>
+    </row>
+    <row r="652" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A652" s="4"/>
+    </row>
+    <row r="653" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A653" s="4"/>
+    </row>
+    <row r="654" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A654" s="4"/>
+    </row>
+    <row r="656" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A656" s="4" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="657" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A657"/>
+    </row>
+    <row r="660" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A660"/>
+      <c r="B660" s="6">
+        <f>ROUND(SQRT(B493^2+B494^2)/(0.1*C510^3),3)</f>
+        <v>8.3320000000000007</v>
+      </c>
+    </row>
+    <row r="661" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A661"/>
+      <c r="B661" s="6">
+        <f>ROUND(B55/(0.2*C510^3),3)</f>
+        <v>3.3450000000000002</v>
+      </c>
+    </row>
+    <row r="662" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A662"/>
+      <c r="B662" s="6">
         <f>0.8*E448</f>
         <v>360</v>
       </c>
     </row>
-    <row r="604" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A604"/>
-      <c r="B604" s="6">
-        <f>ROUND(SQRT(B601^2+3*B602^2),3)</f>
+    <row r="663" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A663"/>
+      <c r="B663" s="6">
+        <f>ROUND(SQRT(B660^2+3*B661^2),3)</f>
         <v>10.148</v>
       </c>
-      <c r="C604" s="6" t="s">
+      <c r="C663" s="6" t="s">
         <v>374</v>
       </c>
     </row>
+    <row r="665" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A665" s="4" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="666" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A666" s="4" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="667" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A667" s="11" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="668" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A668" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="B668" s="6">
+        <f>ROUND(SQRT(B488^2+B489^2),3)</f>
+        <v>541.23</v>
+      </c>
+    </row>
+    <row r="669" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A669" s="6" t="s">
+        <v>476</v>
+      </c>
+      <c r="B669" s="6">
+        <f>ROUND(SQRT(B490^2+B491^2),3)</f>
+        <v>821.21199999999999</v>
+      </c>
+    </row>
+    <row r="670" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A670" s="6" t="s">
+        <v>516</v>
+      </c>
+      <c r="B670" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="671" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A671" s="39" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="672" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A672" t="s">
+        <v>478</v>
+      </c>
+      <c r="B672" s="6">
+        <f>C508</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="673" spans="1:8" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="674" spans="1:8" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A674" s="40" t="s">
+        <v>479</v>
+      </c>
+      <c r="B674" s="41" t="s">
+        <v>481</v>
+      </c>
+      <c r="C674" s="41" t="s">
+        <v>482</v>
+      </c>
+      <c r="D674" s="41" t="s">
+        <v>124</v>
+      </c>
+      <c r="E674" s="41" t="s">
+        <v>483</v>
+      </c>
+      <c r="F674" s="41" t="s">
+        <v>480</v>
+      </c>
+      <c r="G674" s="41" t="s">
+        <v>484</v>
+      </c>
+      <c r="H674" s="41" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="675" spans="1:8" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A675" s="34">
+        <v>307</v>
+      </c>
+      <c r="B675" s="35">
+        <v>25</v>
+      </c>
+      <c r="C675" s="35">
+        <v>80</v>
+      </c>
+      <c r="D675" s="35">
+        <v>21</v>
+      </c>
+      <c r="E675" s="35">
+        <v>2.5</v>
+      </c>
+      <c r="F675" s="35">
+        <v>14.29</v>
+      </c>
+      <c r="G675" s="35">
+        <v>26.2</v>
+      </c>
+      <c r="H675" s="35">
+        <v>17.899999999999999</v>
+      </c>
+    </row>
+    <row r="678" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A678" s="4" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="680" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A680" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="B680" s="6">
+        <v>3</v>
+      </c>
+      <c r="C680" s="6" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="681" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A681" s="12" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="683" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A683" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="B683" s="6">
+        <f>(B686*B690*B668+B688*B670)*B692*B694</f>
+        <v>757.72199999999998</v>
+      </c>
+    </row>
+    <row r="684" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A684" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="B684" s="6">
+        <f>(B686*B690*B669+B670*B688)*B692*B694</f>
+        <v>1149.6967999999999</v>
+      </c>
+    </row>
+    <row r="685" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A685" s="11" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="686" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A686" t="s">
+        <v>506</v>
+      </c>
+      <c r="B686" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="687" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A687" s="12" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="688" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A688" s="6" t="s">
+        <v>507</v>
+      </c>
+      <c r="B688" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="689" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A689" s="48" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="690" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A690" s="46" t="s">
+        <v>511</v>
+      </c>
+      <c r="B690" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="691" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A691" s="48" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="692" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A692" s="46" t="s">
+        <v>513</v>
+      </c>
+      <c r="B692" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="693" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A693" s="48" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="694" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A694" s="46" t="s">
+        <v>515</v>
+      </c>
+      <c r="B694" s="6">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="696" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A696" s="46" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="697" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A697" s="46" t="s">
+        <v>520</v>
+      </c>
+      <c r="B697" s="6">
+        <f>MAX(B683,B684)</f>
+        <v>1149.6967999999999</v>
+      </c>
+    </row>
+    <row r="698" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A698" s="48" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="699" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A699" s="46" t="s">
+        <v>522</v>
+      </c>
+      <c r="B699" s="6">
+        <f>60*F2*C66/10^6</f>
+        <v>1127.0999999999999</v>
+      </c>
+      <c r="C699" s="6" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="700" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A700" s="48" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="701" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A701" s="46" t="s">
+        <v>525</v>
+      </c>
+      <c r="B701" s="6">
+        <f>B697*B699^(1/3)</f>
+        <v>11964.764066420434</v>
+      </c>
+      <c r="C701" s="6" t="s">
+        <v>527</v>
+      </c>
+      <c r="D701" s="6" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="703" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A703" s="4" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="704" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A704" s="46" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="705" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A705"/>
+    </row>
+    <row r="707" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A707" s="6" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="708" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A708" s="46" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="710" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A710" s="11" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="711" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A711" s="46" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="712" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A712" s="46" t="s">
+        <v>535</v>
+      </c>
+      <c r="B712" s="6">
+        <f>B668</f>
+        <v>541.23</v>
+      </c>
+    </row>
+    <row r="713" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A713" s="46" t="s">
+        <v>536</v>
+      </c>
+      <c r="B713" s="6">
+        <f>B669</f>
+        <v>821.21199999999999</v>
+      </c>
+    </row>
+    <row r="715" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A715" s="46" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="716" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A716" s="46" t="s">
+        <v>538</v>
+      </c>
+      <c r="B716" s="6">
+        <f>MAX(B712:B713)</f>
+        <v>821.21199999999999</v>
+      </c>
+      <c r="C716" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="D716" s="6" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="719" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A719" s="13" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="720" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A720" s="4" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="721" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="722" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A722" s="51" t="s">
+        <v>377</v>
+      </c>
+      <c r="B722" s="51" t="s">
+        <v>187</v>
+      </c>
+      <c r="C722" s="51" t="s">
+        <v>223</v>
+      </c>
+      <c r="D722" s="51" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E722" s="51" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="723" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A723" s="52"/>
+      <c r="B723" s="52"/>
+      <c r="C723" s="52"/>
+      <c r="D723" s="52"/>
+      <c r="E723" s="52"/>
+    </row>
+    <row r="724" spans="1:5" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A724" s="49" t="s">
+        <v>379</v>
+      </c>
+      <c r="B724" s="50" t="s">
+        <v>188</v>
+      </c>
+      <c r="C724" s="50" t="s">
+        <v>380</v>
+      </c>
+      <c r="D724" s="50">
+        <v>750</v>
+      </c>
+      <c r="E724" s="50">
+        <v>450</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="18">
+    <mergeCell ref="D722:D723"/>
+    <mergeCell ref="E722:E723"/>
+    <mergeCell ref="C573:C574"/>
+    <mergeCell ref="C576:C577"/>
+    <mergeCell ref="C611:C612"/>
+    <mergeCell ref="A722:A723"/>
+    <mergeCell ref="B722:B723"/>
+    <mergeCell ref="C722:C723"/>
+    <mergeCell ref="A446:A447"/>
+    <mergeCell ref="B446:B447"/>
+    <mergeCell ref="C446:C447"/>
+    <mergeCell ref="D446:D447"/>
+    <mergeCell ref="E446:E447"/>
     <mergeCell ref="D493:D494"/>
     <mergeCell ref="F90:F100"/>
     <mergeCell ref="C227:C238"/>
     <mergeCell ref="C244:C245"/>
     <mergeCell ref="C290:C291"/>
-    <mergeCell ref="A446:A447"/>
-    <mergeCell ref="B446:B447"/>
-    <mergeCell ref="C446:C447"/>
-    <mergeCell ref="D446:D447"/>
-    <mergeCell ref="E446:E447"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>